<commit_message>
Redesign Dashboard: Key Metrics, Goal Tracker, Balance by Bank, multi-line growth
- Key Metrics: Total Balance, Total Deposited, Total Interest Credited, Total Withdrawn
- Personal Goal Tracker: editable target, Maya goal balance, progress %
- Balance by Bank table (doubles as pie source)
- Savings Growth: one cumulative line per bank over 24 months (Jan 2026-Dec 2027)
- Monthly Interest Earned: 24-month column chart
- Live 24-month projection matrix driving the charts
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -225,6 +225,24 @@
     <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -254,7 +272,7 @@
                   <a:srgbClr val="1F3864"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>📈 Savings Growth (12-Month Projection)</a:t>
+              <a:t>Savings Growth by Bank (Cumulative Balance)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -272,11 +290,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!$E$54</c:f>
+              <c:f>Dashboard!$B$79</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Total Savings</c:v>
+                  <c:v>Maya</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -284,106 +302,1292 @@
           <c:spPr>
             <a:ln w="28575">
               <a:solidFill>
-                <a:srgbClr val="2E5496"/>
+                <a:srgbClr val="4472C4"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
           <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
+            <c:symbol val="none"/>
           </c:marker>
           <c:cat>
-            <c:numRef>
-              <c:f>Dashboard!$D$55:$D$67</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+            <c:strRef>
+              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>Jan 2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>Feb 2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2</c:v>
+                  <c:v>Mar 2026</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3</c:v>
+                  <c:v>Apr 2026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4</c:v>
+                  <c:v>May 2026</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5</c:v>
+                  <c:v>Jun 2026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6</c:v>
+                  <c:v>Jul 2026</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7</c:v>
+                  <c:v>Aug 2026</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8</c:v>
+                  <c:v>Sep 2026</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9</c:v>
+                  <c:v>Oct 2026</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>10</c:v>
+                  <c:v>Nov 2026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>11</c:v>
+                  <c:v>Dec 2026</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>12</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$E$55:$E$67</c:f>
+              <c:f>Dashboard!$B$80:$B$103</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>493062.5</c:v>
+                  <c:v>273000.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>495554.2355</c:v>
+                  <c:v>274518.2827</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>498059.5779</c:v>
+                  <c:v>276045.4702</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>500578.6069</c:v>
+                  <c:v>277581.6181</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>503111.4031</c:v>
+                  <c:v>279126.7825</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>505658.0474</c:v>
+                  <c:v>280681.0197</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>508218.6212</c:v>
+                  <c:v>282244.3866</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>510793.2064</c:v>
+                  <c:v>283816.9403</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>513381.8857</c:v>
+                  <c:v>285398.7383</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>515984.7418</c:v>
+                  <c:v>286989.8385</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>518601.8585</c:v>
+                  <c:v>288590.2994</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>521233.3197</c:v>
+                  <c:v>290200.1795</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>523879.2099</c:v>
+                  <c:v>291819.5381</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>293448.4346</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>295086.9288</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>296735.0811</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>298392.9523</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>300060.6034</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>301738.0959</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>303425.4918</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>305122.8534</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>306830.2436</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>308547.7254</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>310275.3626</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$C$79</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>UNO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:solidFill>
+                <a:srgbClr val="ED7D31"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$C$80:$C$103</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>125000.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>125573.0196</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>126148.7525</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>126727.2117</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>127308.4106</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>127892.3623</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>128479.0801</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>129068.5775</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>129660.8679</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>130255.9648</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>130853.8817</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>131454.6324</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>132058.2305</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>132664.6898</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>133274.0242</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>133886.2475</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>134501.3739</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>135119.4172</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>135740.3917</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>136364.3115</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>136991.1909</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>137621.0443</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>138253.8859</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>138889.7304</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$D$79</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Tonik</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:solidFill>
+                <a:srgbClr val="70AD47"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$D$80:$D$103</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>50000.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50266.6667</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>50534.8889</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>50804.6763</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>51076.0386</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>51348.9855</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>51623.5269</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>51899.6725</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>52177.4325</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>52456.8167</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>52737.8353</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>53020.4983</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>53304.8161</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>53590.7987</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>53878.4567</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>54167.8003</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>54458.8401</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>54751.5865</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>55046.0502</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>55342.2418</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>55640.1721</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>55939.8519</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>56241.292</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>56544.5034</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$E$79</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Banko</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$E$80:$E$103</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>15062.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15125.387</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15188.5366</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15251.9499</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15315.6279</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>15379.5717</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>15443.7826</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>15508.2615</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>15573.0096</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>15638.028</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>15703.3179</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>15768.8804</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>15834.7167</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15900.8278</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15967.2149</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16033.8792</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>16100.8218</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>16168.0439</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>16235.5466</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>16303.3312</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>16371.3988</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>16439.7506</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>16508.3877</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>16577.3115</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$F$79</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CIMB</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:solidFill>
+                <a:srgbClr val="7030A0"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$F$80:$F$103</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>10000.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10019.1844</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10038.4057</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10057.6638</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10076.9589</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10096.291</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10115.6601</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>10135.0665</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10154.51</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10173.9909</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10193.5091</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10213.0648</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>10232.658</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>10252.2888</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>10271.9572</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>10291.6634</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>10311.4074</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>10331.1892</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>10351.009</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>10370.8669</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10390.7628</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>10410.6969</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>10430.6692</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>10450.6799</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$G$79</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>GoTyme</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:solidFill>
+                <a:srgbClr val="843C0C"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$G$80:$G$103</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>12000.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12030.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>12060.075</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12090.2252</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>12120.4508</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>12150.7519</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>12181.1288</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12211.5816</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>12242.1105</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>12272.7158</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12303.3976</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12334.1561</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12364.9915</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>12395.904</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>12426.8937</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>12457.961</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>12489.1059</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>12520.3286</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>12551.6294</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>12583.0085</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>12614.466</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>12646.0022</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>12677.6172</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>12709.3113</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$H$79</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Maribank</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$H$80:$H$103</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>8000.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8021.6951</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8043.449</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8065.2619</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8087.1339</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8109.0653</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8131.0561</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8153.1066</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8175.2169</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8197.3871</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8219.6175</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>8241.9081</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8264.2592</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8286.6709</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8309.1434</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8331.6768</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8354.2713</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8376.9271</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>8399.6444</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>8422.4233</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>8445.2639</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>8468.1665</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>8491.1311</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>8514.1581</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -423,12 +1627,25 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:p>
+                <a:r>
+                  <a:t>Cumulative Balance (PHP)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:numFmt formatCode="#,##0" sourceLinked="0"/>
         <c:crossAx val="111"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="b"/>
+      <c:legendPos val="r"/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -476,18 +1693,18 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!$B$54</c:f>
+              <c:f>Dashboard!$B$16</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Total Savings</c:v>
+                  <c:v>Balance</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$55:$A$61</c:f>
+              <c:f>Dashboard!$A$17:$A$23</c:f>
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
@@ -516,7 +1733,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$55:$B$61</c:f>
+              <c:f>Dashboard!$B$17:$B$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -588,7 +1805,7 @@
                   <a:srgbClr val="1F3864"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>📊 Monthly Interest Earned</a:t>
+              <a:t>Monthly Interest Earned</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -607,7 +1824,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!$F$54</c:f>
+              <c:f>Dashboard!$I$79</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -622,91 +1839,162 @@
             </a:solidFill>
           </c:spPr>
           <c:cat>
-            <c:numRef>
-              <c:f>Dashboard!$D$56:$D$67</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+            <c:strRef>
+              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>Jan 2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>Feb 2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3</c:v>
+                  <c:v>Mar 2026</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4</c:v>
+                  <c:v>Apr 2026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5</c:v>
+                  <c:v>May 2026</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6</c:v>
+                  <c:v>Jun 2026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>7</c:v>
+                  <c:v>Jul 2026</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>8</c:v>
+                  <c:v>Aug 2026</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>9</c:v>
+                  <c:v>Sep 2026</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>10</c:v>
+                  <c:v>Oct 2026</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11</c:v>
+                  <c:v>Nov 2026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>12</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$F$56:$F$67</c:f>
+              <c:f>Dashboard!$I$80:$I$103</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2491.7355</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>2505.3423</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2519.029</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2532.7962</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2546.6443</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>2560.5738</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>2574.5853</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>2588.6792</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>2602.8562</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>2617.1167</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>2631.4612</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>2645.8903</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2660.4045</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2675.0044</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2689.6904</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2704.4633</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2719.3234</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2734.2713</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2749.3077</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2764.433</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2779.6479</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2794.9528</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2810.3485</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -744,6 +2032,19 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:p>
+                <a:r>
+                  <a:t>Interest (PHP)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
         <c:numFmt formatCode="#,##0" sourceLinked="0"/>
         <c:crossAx val="333"/>
       </c:valAx>
@@ -764,13 +2065,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:row>50</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -792,15 +2093,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -824,13 +2125,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>49</xdr:row>
+      <xdr:row>74</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -886,15 +2187,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="4" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
@@ -958,7 +2259,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Overview of your savings across all digital banks. Figures update automatically from the Deposit, Transactions and Interest tabs.</t>
+          <t xml:space="preserve">A live overview of everything in this workbook. Add deposits on the Deposit tab and this page updates automatically.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -975,486 +2276,1323 @@
       <c r="M3" s="5"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">📊 Overview</t>
-        </is>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
+      <c r="A4" t="inlineStr" s="24">
+        <is>
+          <t xml:space="preserve">🔑 Key Metrics</t>
+        </is>
+      </c>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" t="inlineStr" s="12">
-        <is>
-          <t xml:space="preserve">Total Savings</t>
-        </is>
-      </c>
-      <c r="B5" s="12"/>
-      <c r="C5" t="inlineStr" s="12">
-        <is>
-          <t xml:space="preserve">Total Deposits</t>
-        </is>
-      </c>
-      <c r="D5" s="12"/>
-      <c r="E5" t="inlineStr" s="12">
-        <is>
-          <t xml:space="preserve">Proj. Interest (1 Yr)</t>
-        </is>
-      </c>
-      <c r="F5" s="12"/>
-      <c r="G5" t="inlineStr" s="12">
-        <is>
-          <t xml:space="preserve">Proj. Balance (1 Yr)</t>
-        </is>
-      </c>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="L5" s="12"/>
-      <c r="M5" s="12"/>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="13">
+      <c r="A5" t="inlineStr" s="25">
+        <is>
+          <t xml:space="preserve">Total Balance (All Accounts)</t>
+        </is>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="26">
         <f>SUM(Balance!$F$6:$F$19)</f>
         <v>493062.5</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13">
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" t="inlineStr" s="25">
+        <is>
+          <t xml:space="preserve">Total Deposited (All-Time)</t>
+        </is>
+      </c>
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="26">
         <f>SUM(Balance!$D$6:$D$19)</f>
         <v>490000.0</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13">
-        <f>SUM(Balance!$G$6:$G$19)</f>
-        <v>30816.71</v>
-      </c>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13">
-        <f>SUM(Balance!$H$6:$H$19)</f>
-        <v>523879.21</v>
-      </c>
-      <c r="H6" s="13"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-    </row>
-    <row r="7" ht="8" customHeight="1"/>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" t="inlineStr" s="4">
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" t="inlineStr" s="25">
+        <is>
+          <t xml:space="preserve">Total Interest Credited</t>
+        </is>
+      </c>
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="26">
+        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$B$6:$B$205,"Interest")</f>
+        <v>62.5</v>
+      </c>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" t="inlineStr" s="25">
+        <is>
+          <t xml:space="preserve">Total Withdrawn</t>
+        </is>
+      </c>
+      <c r="B8" s="25"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="26">
+        <f>-SUMIFS(Transactions!$E$6:$E$205,Transactions!$B$6:$B$205,"Withdrawal")</f>
+        <v>2000</v>
+      </c>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+    </row>
+    <row r="9" ht="6" customHeight="1"/>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" t="inlineStr" s="24">
+        <is>
+          <t xml:space="preserve">🎯 Personal Goal Tracker</t>
+        </is>
+      </c>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="24"/>
+      <c r="M10" s="24"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" t="inlineStr" s="25">
+        <is>
+          <t xml:space="preserve">Your Savings Goal Target</t>
+        </is>
+      </c>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="28">
+        <v>100000</v>
+      </c>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" t="inlineStr" s="25">
+        <is>
+          <t xml:space="preserve">Maya Personal Goal — Current Balance</t>
+        </is>
+      </c>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="26">
+        <f>IFERROR(VLOOKUP("Maya - Personal Goal",Balance!$C$6:$F$19,4,FALSE),0)</f>
+        <v>25000.0</v>
+      </c>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" t="inlineStr" s="25">
+        <is>
+          <t xml:space="preserve">Progress Toward Goal</t>
+        </is>
+      </c>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="27">
+        <f>IFERROR(E12/E11,0)</f>
+        <v>0.25</v>
+      </c>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+    </row>
+    <row r="14" ht="6" customHeight="1"/>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" t="inlineStr" s="24">
+        <is>
+          <t xml:space="preserve">🏦 Balance by Bank</t>
+        </is>
+      </c>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="24"/>
+      <c r="L15" s="24"/>
+      <c r="M15" s="24"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Bank</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="B17" s="29">
+        <f>SUMIF(Balance!$B$6:$B$19,A17,Balance!$F$6:$F$19)</f>
+        <v>273000.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="B18" s="29">
+        <f>SUMIF(Balance!$B$6:$B$19,A18,Balance!$F$6:$F$19)</f>
+        <v>125000.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="B19" s="29">
+        <f>SUMIF(Balance!$B$6:$B$19,A19,Balance!$F$6:$F$19)</f>
+        <v>50000.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Banko</t>
+        </is>
+      </c>
+      <c r="B20" s="29">
+        <f>SUMIF(Balance!$B$6:$B$19,A20,Balance!$F$6:$F$19)</f>
+        <v>15062.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">CIMB</t>
+        </is>
+      </c>
+      <c r="B21" s="29">
+        <f>SUMIF(Balance!$B$6:$B$19,A21,Balance!$F$6:$F$19)</f>
+        <v>10000.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">GoTyme</t>
+        </is>
+      </c>
+      <c r="B22" s="29">
+        <f>SUMIF(Balance!$B$6:$B$19,A22,Balance!$F$6:$F$19)</f>
+        <v>12000.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maribank</t>
+        </is>
+      </c>
+      <c r="B23" s="29">
+        <f>SUMIF(Balance!$B$6:$B$19,A23,Balance!$F$6:$F$19)</f>
+        <v>8000.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
+      </c>
+      <c r="B24" s="16">
+        <f>SUM(B17:B23)</f>
+        <v>493062.5</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" t="inlineStr" s="24">
+        <is>
+          <t xml:space="preserve">📈 Savings Growth by Bank (Cumulative Balance)</t>
+        </is>
+      </c>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" t="inlineStr" s="24">
+        <is>
+          <t xml:space="preserve">📊 Monthly Interest Earned</t>
+        </is>
+      </c>
+      <c r="B51" s="24"/>
+      <c r="C51" s="24"/>
+      <c r="D51" s="24"/>
+      <c r="E51" s="24"/>
+      <c r="F51" s="24"/>
+      <c r="G51" s="24"/>
+      <c r="H51" s="24"/>
+      <c r="I51" s="24"/>
+      <c r="J51" s="24"/>
+      <c r="K51" s="24"/>
+      <c r="L51" s="24"/>
+      <c r="M51" s="24"/>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">🗂 Chart Data (auto-calculated — do not edit)</t>
         </is>
       </c>
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-      <c r="I52" s="4"/>
-      <c r="J52" s="4"/>
-      <c r="K52" s="4"/>
-      <c r="L52" s="4"/>
-      <c r="M52" s="4"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr" s="22">
-        <is>
-          <t xml:space="preserve">Bank</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr" s="22">
-        <is>
-          <t xml:space="preserve">Total Savings</t>
-        </is>
-      </c>
-      <c r="C54" s="22"/>
-      <c r="D54" t="inlineStr" s="22">
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4"/>
+      <c r="G77" s="4"/>
+      <c r="H77" s="4"/>
+      <c r="I77" s="4"/>
+      <c r="J77" s="4"/>
+      <c r="K77" s="4"/>
+      <c r="L77" s="4"/>
+      <c r="M77" s="4"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr" s="22">
         <is>
           <t xml:space="preserve">Month</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr" s="22">
-        <is>
-          <t xml:space="preserve">Total Savings</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr" s="22">
-        <is>
-          <t xml:space="preserve">Interest Earned</t>
-        </is>
-      </c>
-      <c r="G54" s="22"/>
-      <c r="H54" s="22"/>
-      <c r="I54" s="22"/>
-      <c r="J54" s="22"/>
-      <c r="K54" s="22"/>
-      <c r="L54" s="22"/>
-      <c r="M54" s="22"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr" s="7">
+      <c r="B79" t="inlineStr" s="22">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="B55" s="8">
-        <f>SUMIF(Balance!$B$6:$B$19,A55,Balance!$F$6:$F$19)</f>
+      <c r="C79" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Banko</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">CIMB</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">GoTyme</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Maribank</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Total Interest</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jan 2026</t>
+        </is>
+      </c>
+      <c r="B80" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>273000.0</v>
       </c>
-      <c r="C55" s="7"/>
-      <c r="D55" s="10">
+      <c r="C80" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
+        <v>125000.0</v>
+      </c>
+      <c r="D80" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
+        <v>50000.0</v>
+      </c>
+      <c r="E80" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
+        <v>15062.5</v>
+      </c>
+      <c r="F80" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
+        <v>10000.0</v>
+      </c>
+      <c r="G80" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
+        <v>12000.0</v>
+      </c>
+      <c r="H80" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
+        <v>8000.0</v>
+      </c>
+      <c r="I80" s="8">
         <v>0</v>
       </c>
-      <c r="E55" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D55)</f>
-        <v>493062.5</v>
-      </c>
-      <c r="F55" s="8">
-        <v>0</v>
-      </c>
-      <c r="G55" s="21"/>
-      <c r="H55" s="21"/>
-      <c r="I55" s="21"/>
-      <c r="J55" s="21"/>
-      <c r="K55" s="21"/>
-      <c r="L55" s="21"/>
-      <c r="M55" s="21"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO</t>
-        </is>
-      </c>
-      <c r="B56" s="8">
-        <f>SUMIF(Balance!$B$6:$B$19,A56,Balance!$F$6:$F$19)</f>
-        <v>125000.0</v>
-      </c>
-      <c r="C56" s="7"/>
-      <c r="D56" s="10">
-        <v>1</v>
-      </c>
-      <c r="E56" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D56)</f>
-        <v>495554.24</v>
-      </c>
-      <c r="F56" s="8">
-        <f>E56-E55</f>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Feb 2026</t>
+        </is>
+      </c>
+      <c r="B81" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
+        <v>274518.28</v>
+      </c>
+      <c r="C81" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
+        <v>125573.02</v>
+      </c>
+      <c r="D81" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
+        <v>50266.67</v>
+      </c>
+      <c r="E81" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
+        <v>15125.39</v>
+      </c>
+      <c r="F81" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
+        <v>10019.18</v>
+      </c>
+      <c r="G81" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
+        <v>12030.0</v>
+      </c>
+      <c r="H81" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
+        <v>8021.7</v>
+      </c>
+      <c r="I81" s="8">
+        <f>SUM(B81:H81)-SUM(B80:H80)</f>
         <v>2491.74</v>
       </c>
-      <c r="G56" s="21"/>
-      <c r="H56" s="21"/>
-      <c r="I56" s="21"/>
-      <c r="J56" s="21"/>
-      <c r="K56" s="21"/>
-      <c r="L56" s="21"/>
-      <c r="M56" s="21"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik</t>
-        </is>
-      </c>
-      <c r="B57" s="8">
-        <f>SUMIF(Balance!$B$6:$B$19,A57,Balance!$F$6:$F$19)</f>
-        <v>50000.0</v>
-      </c>
-      <c r="C57" s="7"/>
-      <c r="D57" s="10">
-        <v>2</v>
-      </c>
-      <c r="E57" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D57)</f>
-        <v>498059.58</v>
-      </c>
-      <c r="F57" s="8">
-        <f>E57-E56</f>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Mar 2026</t>
+        </is>
+      </c>
+      <c r="B82" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
+        <v>276045.47</v>
+      </c>
+      <c r="C82" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
+        <v>126148.75</v>
+      </c>
+      <c r="D82" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
+        <v>50534.89</v>
+      </c>
+      <c r="E82" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
+        <v>15188.54</v>
+      </c>
+      <c r="F82" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
+        <v>10038.41</v>
+      </c>
+      <c r="G82" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
+        <v>12060.07</v>
+      </c>
+      <c r="H82" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
+        <v>8043.45</v>
+      </c>
+      <c r="I82" s="8">
+        <f>SUM(B82:H82)-SUM(B81:H81)</f>
         <v>2505.34</v>
       </c>
-      <c r="G57" s="21"/>
-      <c r="H57" s="21"/>
-      <c r="I57" s="21"/>
-      <c r="J57" s="21"/>
-      <c r="K57" s="21"/>
-      <c r="L57" s="21"/>
-      <c r="M57" s="21"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Banko</t>
-        </is>
-      </c>
-      <c r="B58" s="8">
-        <f>SUMIF(Balance!$B$6:$B$19,A58,Balance!$F$6:$F$19)</f>
-        <v>15062.5</v>
-      </c>
-      <c r="C58" s="7"/>
-      <c r="D58" s="10">
-        <v>3</v>
-      </c>
-      <c r="E58" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D58)</f>
-        <v>500578.61</v>
-      </c>
-      <c r="F58" s="8">
-        <f>E58-E57</f>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Apr 2026</t>
+        </is>
+      </c>
+      <c r="B83" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
+        <v>277581.62</v>
+      </c>
+      <c r="C83" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
+        <v>126727.21</v>
+      </c>
+      <c r="D83" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
+        <v>50804.68</v>
+      </c>
+      <c r="E83" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
+        <v>15251.95</v>
+      </c>
+      <c r="F83" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
+        <v>10057.66</v>
+      </c>
+      <c r="G83" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
+        <v>12090.23</v>
+      </c>
+      <c r="H83" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
+        <v>8065.26</v>
+      </c>
+      <c r="I83" s="8">
+        <f>SUM(B83:H83)-SUM(B82:H82)</f>
         <v>2519.03</v>
       </c>
-      <c r="G58" s="21"/>
-      <c r="H58" s="21"/>
-      <c r="I58" s="21"/>
-      <c r="J58" s="21"/>
-      <c r="K58" s="21"/>
-      <c r="L58" s="21"/>
-      <c r="M58" s="21"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CIMB</t>
-        </is>
-      </c>
-      <c r="B59" s="8">
-        <f>SUMIF(Balance!$B$6:$B$19,A59,Balance!$F$6:$F$19)</f>
-        <v>10000.0</v>
-      </c>
-      <c r="C59" s="7"/>
-      <c r="D59" s="10">
-        <v>4</v>
-      </c>
-      <c r="E59" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D59)</f>
-        <v>503111.4</v>
-      </c>
-      <c r="F59" s="8">
-        <f>E59-E58</f>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">May 2026</t>
+        </is>
+      </c>
+      <c r="B84" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
+        <v>279126.78</v>
+      </c>
+      <c r="C84" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
+        <v>127308.41</v>
+      </c>
+      <c r="D84" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
+        <v>51076.04</v>
+      </c>
+      <c r="E84" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
+        <v>15315.63</v>
+      </c>
+      <c r="F84" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
+        <v>10076.96</v>
+      </c>
+      <c r="G84" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
+        <v>12120.45</v>
+      </c>
+      <c r="H84" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
+        <v>8087.13</v>
+      </c>
+      <c r="I84" s="8">
+        <f>SUM(B84:H84)-SUM(B83:H83)</f>
         <v>2532.8</v>
       </c>
-      <c r="G59" s="21"/>
-      <c r="H59" s="21"/>
-      <c r="I59" s="21"/>
-      <c r="J59" s="21"/>
-      <c r="K59" s="21"/>
-      <c r="L59" s="21"/>
-      <c r="M59" s="21"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">GoTyme</t>
-        </is>
-      </c>
-      <c r="B60" s="8">
-        <f>SUMIF(Balance!$B$6:$B$19,A60,Balance!$F$6:$F$19)</f>
-        <v>12000.0</v>
-      </c>
-      <c r="C60" s="7"/>
-      <c r="D60" s="10">
-        <v>5</v>
-      </c>
-      <c r="E60" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D60)</f>
-        <v>505658.05</v>
-      </c>
-      <c r="F60" s="8">
-        <f>E60-E59</f>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jun 2026</t>
+        </is>
+      </c>
+      <c r="B85" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
+        <v>280681.02</v>
+      </c>
+      <c r="C85" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
+        <v>127892.36</v>
+      </c>
+      <c r="D85" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
+        <v>51348.99</v>
+      </c>
+      <c r="E85" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
+        <v>15379.57</v>
+      </c>
+      <c r="F85" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
+        <v>10096.29</v>
+      </c>
+      <c r="G85" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
+        <v>12150.75</v>
+      </c>
+      <c r="H85" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
+        <v>8109.07</v>
+      </c>
+      <c r="I85" s="8">
+        <f>SUM(B85:H85)-SUM(B84:H84)</f>
         <v>2546.64</v>
       </c>
-      <c r="G60" s="21"/>
-      <c r="H60" s="21"/>
-      <c r="I60" s="21"/>
-      <c r="J60" s="21"/>
-      <c r="K60" s="21"/>
-      <c r="L60" s="21"/>
-      <c r="M60" s="21"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maribank</t>
-        </is>
-      </c>
-      <c r="B61" s="8">
-        <f>SUMIF(Balance!$B$6:$B$19,A61,Balance!$F$6:$F$19)</f>
-        <v>8000.0</v>
-      </c>
-      <c r="C61" s="7"/>
-      <c r="D61" s="10">
-        <v>6</v>
-      </c>
-      <c r="E61" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D61)</f>
-        <v>508218.62</v>
-      </c>
-      <c r="F61" s="8">
-        <f>E61-E60</f>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jul 2026</t>
+        </is>
+      </c>
+      <c r="B86" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
+        <v>282244.39</v>
+      </c>
+      <c r="C86" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
+        <v>128479.08</v>
+      </c>
+      <c r="D86" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
+        <v>51623.53</v>
+      </c>
+      <c r="E86" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
+        <v>15443.78</v>
+      </c>
+      <c r="F86" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
+        <v>10115.66</v>
+      </c>
+      <c r="G86" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
+        <v>12181.13</v>
+      </c>
+      <c r="H86" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
+        <v>8131.06</v>
+      </c>
+      <c r="I86" s="8">
+        <f>SUM(B86:H86)-SUM(B85:H85)</f>
         <v>2560.57</v>
       </c>
-      <c r="G61" s="21"/>
-      <c r="H61" s="21"/>
-      <c r="I61" s="21"/>
-      <c r="J61" s="21"/>
-      <c r="K61" s="21"/>
-      <c r="L61" s="21"/>
-      <c r="M61" s="21"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="7"/>
-      <c r="B62" s="8"/>
-      <c r="C62" s="7"/>
-      <c r="D62" s="10">
-        <v>7</v>
-      </c>
-      <c r="E62" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D62)</f>
-        <v>510793.21</v>
-      </c>
-      <c r="F62" s="8">
-        <f>E62-E61</f>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Aug 2026</t>
+        </is>
+      </c>
+      <c r="B87" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
+        <v>283816.94</v>
+      </c>
+      <c r="C87" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
+        <v>129068.58</v>
+      </c>
+      <c r="D87" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
+        <v>51899.67</v>
+      </c>
+      <c r="E87" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
+        <v>15508.26</v>
+      </c>
+      <c r="F87" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
+        <v>10135.07</v>
+      </c>
+      <c r="G87" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
+        <v>12211.58</v>
+      </c>
+      <c r="H87" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
+        <v>8153.11</v>
+      </c>
+      <c r="I87" s="8">
+        <f>SUM(B87:H87)-SUM(B86:H86)</f>
         <v>2574.59</v>
       </c>
-      <c r="G62" s="21"/>
-      <c r="H62" s="21"/>
-      <c r="I62" s="21"/>
-      <c r="J62" s="21"/>
-      <c r="K62" s="21"/>
-      <c r="L62" s="21"/>
-      <c r="M62" s="21"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="7"/>
-      <c r="B63" s="8"/>
-      <c r="C63" s="7"/>
-      <c r="D63" s="10">
-        <v>8</v>
-      </c>
-      <c r="E63" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D63)</f>
-        <v>513381.89</v>
-      </c>
-      <c r="F63" s="8">
-        <f>E63-E62</f>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Sep 2026</t>
+        </is>
+      </c>
+      <c r="B88" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
+        <v>285398.74</v>
+      </c>
+      <c r="C88" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
+        <v>129660.87</v>
+      </c>
+      <c r="D88" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
+        <v>52177.43</v>
+      </c>
+      <c r="E88" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
+        <v>15573.01</v>
+      </c>
+      <c r="F88" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
+        <v>10154.51</v>
+      </c>
+      <c r="G88" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
+        <v>12242.11</v>
+      </c>
+      <c r="H88" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
+        <v>8175.22</v>
+      </c>
+      <c r="I88" s="8">
+        <f>SUM(B88:H88)-SUM(B87:H87)</f>
         <v>2588.68</v>
       </c>
-      <c r="G63" s="21"/>
-      <c r="H63" s="21"/>
-      <c r="I63" s="21"/>
-      <c r="J63" s="21"/>
-      <c r="K63" s="21"/>
-      <c r="L63" s="21"/>
-      <c r="M63" s="21"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="7"/>
-      <c r="B64" s="8"/>
-      <c r="C64" s="7"/>
-      <c r="D64" s="10">
-        <v>9</v>
-      </c>
-      <c r="E64" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D64)</f>
-        <v>515984.74</v>
-      </c>
-      <c r="F64" s="8">
-        <f>E64-E63</f>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Oct 2026</t>
+        </is>
+      </c>
+      <c r="B89" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
+        <v>286989.84</v>
+      </c>
+      <c r="C89" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
+        <v>130255.96</v>
+      </c>
+      <c r="D89" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
+        <v>52456.82</v>
+      </c>
+      <c r="E89" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
+        <v>15638.03</v>
+      </c>
+      <c r="F89" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
+        <v>10173.99</v>
+      </c>
+      <c r="G89" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
+        <v>12272.72</v>
+      </c>
+      <c r="H89" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
+        <v>8197.39</v>
+      </c>
+      <c r="I89" s="8">
+        <f>SUM(B89:H89)-SUM(B88:H88)</f>
         <v>2602.86</v>
       </c>
-      <c r="G64" s="21"/>
-      <c r="H64" s="21"/>
-      <c r="I64" s="21"/>
-      <c r="J64" s="21"/>
-      <c r="K64" s="21"/>
-      <c r="L64" s="21"/>
-      <c r="M64" s="21"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="7"/>
-      <c r="B65" s="8"/>
-      <c r="C65" s="7"/>
-      <c r="D65" s="10">
-        <v>10</v>
-      </c>
-      <c r="E65" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D65)</f>
-        <v>518601.86</v>
-      </c>
-      <c r="F65" s="8">
-        <f>E65-E64</f>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Nov 2026</t>
+        </is>
+      </c>
+      <c r="B90" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
+        <v>288590.3</v>
+      </c>
+      <c r="C90" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
+        <v>130853.88</v>
+      </c>
+      <c r="D90" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
+        <v>52737.84</v>
+      </c>
+      <c r="E90" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
+        <v>15703.32</v>
+      </c>
+      <c r="F90" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
+        <v>10193.51</v>
+      </c>
+      <c r="G90" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
+        <v>12303.4</v>
+      </c>
+      <c r="H90" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
+        <v>8219.62</v>
+      </c>
+      <c r="I90" s="8">
+        <f>SUM(B90:H90)-SUM(B89:H89)</f>
         <v>2617.12</v>
       </c>
-      <c r="G65" s="21"/>
-      <c r="H65" s="21"/>
-      <c r="I65" s="21"/>
-      <c r="J65" s="21"/>
-      <c r="K65" s="21"/>
-      <c r="L65" s="21"/>
-      <c r="M65" s="21"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="7"/>
-      <c r="B66" s="8"/>
-      <c r="C66" s="7"/>
-      <c r="D66" s="10">
-        <v>11</v>
-      </c>
-      <c r="E66" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D66)</f>
-        <v>521233.32</v>
-      </c>
-      <c r="F66" s="8">
-        <f>E66-E65</f>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Dec 2026</t>
+        </is>
+      </c>
+      <c r="B91" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
+        <v>290200.18</v>
+      </c>
+      <c r="C91" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
+        <v>131454.63</v>
+      </c>
+      <c r="D91" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
+        <v>53020.5</v>
+      </c>
+      <c r="E91" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
+        <v>15768.88</v>
+      </c>
+      <c r="F91" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
+        <v>10213.06</v>
+      </c>
+      <c r="G91" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
+        <v>12334.16</v>
+      </c>
+      <c r="H91" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
+        <v>8241.91</v>
+      </c>
+      <c r="I91" s="8">
+        <f>SUM(B91:H91)-SUM(B90:H90)</f>
         <v>2631.46</v>
       </c>
-      <c r="G66" s="21"/>
-      <c r="H66" s="21"/>
-      <c r="I66" s="21"/>
-      <c r="J66" s="21"/>
-      <c r="K66" s="21"/>
-      <c r="L66" s="21"/>
-      <c r="M66" s="21"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="7"/>
-      <c r="B67" s="8"/>
-      <c r="C67" s="7"/>
-      <c r="D67" s="10">
-        <v>12</v>
-      </c>
-      <c r="E67" s="8">
-        <f>SUMPRODUCT(Interest!$G$6:$G$19,Interest!$M$6:$M$19^D67)</f>
-        <v>523879.21</v>
-      </c>
-      <c r="F67" s="8">
-        <f>E67-E66</f>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jan 2027</t>
+        </is>
+      </c>
+      <c r="B92" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
+        <v>291819.54</v>
+      </c>
+      <c r="C92" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
+        <v>132058.23</v>
+      </c>
+      <c r="D92" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
+        <v>53304.82</v>
+      </c>
+      <c r="E92" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
+        <v>15834.72</v>
+      </c>
+      <c r="F92" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
+        <v>10232.66</v>
+      </c>
+      <c r="G92" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
+        <v>12364.99</v>
+      </c>
+      <c r="H92" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
+        <v>8264.26</v>
+      </c>
+      <c r="I92" s="8">
+        <f>SUM(B92:H92)-SUM(B91:H91)</f>
         <v>2645.89</v>
       </c>
-      <c r="G67" s="21"/>
-      <c r="H67" s="21"/>
-      <c r="I67" s="21"/>
-      <c r="J67" s="21"/>
-      <c r="K67" s="21"/>
-      <c r="L67" s="21"/>
-      <c r="M67" s="21"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Feb 2027</t>
+        </is>
+      </c>
+      <c r="B93" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
+        <v>293448.43</v>
+      </c>
+      <c r="C93" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
+        <v>132664.69</v>
+      </c>
+      <c r="D93" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
+        <v>53590.8</v>
+      </c>
+      <c r="E93" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
+        <v>15900.83</v>
+      </c>
+      <c r="F93" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
+        <v>10252.29</v>
+      </c>
+      <c r="G93" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
+        <v>12395.9</v>
+      </c>
+      <c r="H93" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
+        <v>8286.67</v>
+      </c>
+      <c r="I93" s="8">
+        <f>SUM(B93:H93)-SUM(B92:H92)</f>
+        <v>2660.4</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Mar 2027</t>
+        </is>
+      </c>
+      <c r="B94" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
+        <v>295086.93</v>
+      </c>
+      <c r="C94" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
+        <v>133274.02</v>
+      </c>
+      <c r="D94" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
+        <v>53878.46</v>
+      </c>
+      <c r="E94" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
+        <v>15967.21</v>
+      </c>
+      <c r="F94" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
+        <v>10271.96</v>
+      </c>
+      <c r="G94" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
+        <v>12426.89</v>
+      </c>
+      <c r="H94" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
+        <v>8309.14</v>
+      </c>
+      <c r="I94" s="8">
+        <f>SUM(B94:H94)-SUM(B93:H93)</f>
+        <v>2675.0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Apr 2027</t>
+        </is>
+      </c>
+      <c r="B95" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
+        <v>296735.08</v>
+      </c>
+      <c r="C95" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
+        <v>133886.25</v>
+      </c>
+      <c r="D95" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
+        <v>54167.8</v>
+      </c>
+      <c r="E95" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
+        <v>16033.88</v>
+      </c>
+      <c r="F95" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
+        <v>10291.66</v>
+      </c>
+      <c r="G95" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
+        <v>12457.96</v>
+      </c>
+      <c r="H95" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
+        <v>8331.68</v>
+      </c>
+      <c r="I95" s="8">
+        <f>SUM(B95:H95)-SUM(B94:H94)</f>
+        <v>2689.69</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">May 2027</t>
+        </is>
+      </c>
+      <c r="B96" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
+        <v>298392.95</v>
+      </c>
+      <c r="C96" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
+        <v>134501.37</v>
+      </c>
+      <c r="D96" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
+        <v>54458.84</v>
+      </c>
+      <c r="E96" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
+        <v>16100.82</v>
+      </c>
+      <c r="F96" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
+        <v>10311.41</v>
+      </c>
+      <c r="G96" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
+        <v>12489.11</v>
+      </c>
+      <c r="H96" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
+        <v>8354.27</v>
+      </c>
+      <c r="I96" s="8">
+        <f>SUM(B96:H96)-SUM(B95:H95)</f>
+        <v>2704.46</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jun 2027</t>
+        </is>
+      </c>
+      <c r="B97" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
+        <v>300060.6</v>
+      </c>
+      <c r="C97" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
+        <v>135119.42</v>
+      </c>
+      <c r="D97" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
+        <v>54751.59</v>
+      </c>
+      <c r="E97" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
+        <v>16168.04</v>
+      </c>
+      <c r="F97" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
+        <v>10331.19</v>
+      </c>
+      <c r="G97" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
+        <v>12520.33</v>
+      </c>
+      <c r="H97" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
+        <v>8376.93</v>
+      </c>
+      <c r="I97" s="8">
+        <f>SUM(B97:H97)-SUM(B96:H96)</f>
+        <v>2719.32</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jul 2027</t>
+        </is>
+      </c>
+      <c r="B98" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
+        <v>301738.1</v>
+      </c>
+      <c r="C98" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
+        <v>135740.39</v>
+      </c>
+      <c r="D98" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
+        <v>55046.05</v>
+      </c>
+      <c r="E98" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
+        <v>16235.55</v>
+      </c>
+      <c r="F98" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
+        <v>10351.01</v>
+      </c>
+      <c r="G98" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
+        <v>12551.63</v>
+      </c>
+      <c r="H98" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
+        <v>8399.64</v>
+      </c>
+      <c r="I98" s="8">
+        <f>SUM(B98:H98)-SUM(B97:H97)</f>
+        <v>2734.27</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Aug 2027</t>
+        </is>
+      </c>
+      <c r="B99" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
+        <v>303425.49</v>
+      </c>
+      <c r="C99" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
+        <v>136364.31</v>
+      </c>
+      <c r="D99" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
+        <v>55342.24</v>
+      </c>
+      <c r="E99" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
+        <v>16303.33</v>
+      </c>
+      <c r="F99" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
+        <v>10370.87</v>
+      </c>
+      <c r="G99" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
+        <v>12583.01</v>
+      </c>
+      <c r="H99" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
+        <v>8422.42</v>
+      </c>
+      <c r="I99" s="8">
+        <f>SUM(B99:H99)-SUM(B98:H98)</f>
+        <v>2749.31</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Sep 2027</t>
+        </is>
+      </c>
+      <c r="B100" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
+        <v>305122.85</v>
+      </c>
+      <c r="C100" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
+        <v>136991.19</v>
+      </c>
+      <c r="D100" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
+        <v>55640.17</v>
+      </c>
+      <c r="E100" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
+        <v>16371.4</v>
+      </c>
+      <c r="F100" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
+        <v>10390.76</v>
+      </c>
+      <c r="G100" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
+        <v>12614.47</v>
+      </c>
+      <c r="H100" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
+        <v>8445.26</v>
+      </c>
+      <c r="I100" s="8">
+        <f>SUM(B100:H100)-SUM(B99:H99)</f>
+        <v>2764.43</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Oct 2027</t>
+        </is>
+      </c>
+      <c r="B101" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
+        <v>306830.24</v>
+      </c>
+      <c r="C101" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
+        <v>137621.04</v>
+      </c>
+      <c r="D101" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
+        <v>55939.85</v>
+      </c>
+      <c r="E101" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
+        <v>16439.75</v>
+      </c>
+      <c r="F101" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
+        <v>10410.7</v>
+      </c>
+      <c r="G101" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
+        <v>12646.0</v>
+      </c>
+      <c r="H101" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
+        <v>8468.17</v>
+      </c>
+      <c r="I101" s="8">
+        <f>SUM(B101:H101)-SUM(B100:H100)</f>
+        <v>2779.65</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Nov 2027</t>
+        </is>
+      </c>
+      <c r="B102" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
+        <v>308547.73</v>
+      </c>
+      <c r="C102" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
+        <v>138253.89</v>
+      </c>
+      <c r="D102" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
+        <v>56241.29</v>
+      </c>
+      <c r="E102" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
+        <v>16508.39</v>
+      </c>
+      <c r="F102" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
+        <v>10430.67</v>
+      </c>
+      <c r="G102" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
+        <v>12677.62</v>
+      </c>
+      <c r="H102" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
+        <v>8491.13</v>
+      </c>
+      <c r="I102" s="8">
+        <f>SUM(B102:H102)-SUM(B101:H101)</f>
+        <v>2794.95</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Dec 2027</t>
+        </is>
+      </c>
+      <c r="B103" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
+        <v>310275.36</v>
+      </c>
+      <c r="C103" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
+        <v>138889.73</v>
+      </c>
+      <c r="D103" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
+        <v>56544.5</v>
+      </c>
+      <c r="E103" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
+        <v>16577.31</v>
+      </c>
+      <c r="F103" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
+        <v>10450.68</v>
+      </c>
+      <c r="G103" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
+        <v>12709.31</v>
+      </c>
+      <c r="H103" s="8">
+        <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
+        <v>8514.16</v>
+      </c>
+      <c r="I103" s="8">
+        <f>SUM(B103:H103)-SUM(B102:H102)</f>
+        <v>2810.35</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="27">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
@@ -1463,15 +3601,25 @@
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="A52:M52"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="A27:M27"/>
+    <mergeCell ref="A51:M51"/>
+    <mergeCell ref="A77:M77"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2:B2" location="Dashboard!A1" display="🏠 Dashboard"/>

</xml_diff>

<commit_message>
Fix ##### in Dashboard chart-data: compact number format + wider columns
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -241,6 +241,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2187,15 +2190,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
@@ -2662,35 +2665,35 @@
           <t xml:space="preserve">Jan 2026</t>
         </is>
       </c>
-      <c r="B80" s="8">
+      <c r="B80" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>273000.0</v>
       </c>
-      <c r="C80" s="8">
+      <c r="C80" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>125000.0</v>
       </c>
-      <c r="D80" s="8">
+      <c r="D80" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>50000.0</v>
       </c>
-      <c r="E80" s="8">
+      <c r="E80" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>15062.5</v>
       </c>
-      <c r="F80" s="8">
+      <c r="F80" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>10000.0</v>
       </c>
-      <c r="G80" s="8">
+      <c r="G80" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>12000.0</v>
       </c>
-      <c r="H80" s="8">
+      <c r="H80" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>8000.0</v>
       </c>
-      <c r="I80" s="8">
+      <c r="I80" s="30">
         <v>0</v>
       </c>
     </row>
@@ -2700,35 +2703,35 @@
           <t xml:space="preserve">Feb 2026</t>
         </is>
       </c>
-      <c r="B81" s="8">
+      <c r="B81" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>274518.28</v>
       </c>
-      <c r="C81" s="8">
+      <c r="C81" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>125573.02</v>
       </c>
-      <c r="D81" s="8">
+      <c r="D81" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>50266.67</v>
       </c>
-      <c r="E81" s="8">
+      <c r="E81" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>15125.39</v>
       </c>
-      <c r="F81" s="8">
+      <c r="F81" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>10019.18</v>
       </c>
-      <c r="G81" s="8">
+      <c r="G81" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>12030.0</v>
       </c>
-      <c r="H81" s="8">
+      <c r="H81" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>8021.7</v>
       </c>
-      <c r="I81" s="8">
+      <c r="I81" s="30">
         <f>SUM(B81:H81)-SUM(B80:H80)</f>
         <v>2491.74</v>
       </c>
@@ -2739,35 +2742,35 @@
           <t xml:space="preserve">Mar 2026</t>
         </is>
       </c>
-      <c r="B82" s="8">
+      <c r="B82" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>276045.47</v>
       </c>
-      <c r="C82" s="8">
+      <c r="C82" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>126148.75</v>
       </c>
-      <c r="D82" s="8">
+      <c r="D82" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>50534.89</v>
       </c>
-      <c r="E82" s="8">
+      <c r="E82" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>15188.54</v>
       </c>
-      <c r="F82" s="8">
+      <c r="F82" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>10038.41</v>
       </c>
-      <c r="G82" s="8">
+      <c r="G82" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>12060.07</v>
       </c>
-      <c r="H82" s="8">
+      <c r="H82" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>8043.45</v>
       </c>
-      <c r="I82" s="8">
+      <c r="I82" s="30">
         <f>SUM(B82:H82)-SUM(B81:H81)</f>
         <v>2505.34</v>
       </c>
@@ -2778,35 +2781,35 @@
           <t xml:space="preserve">Apr 2026</t>
         </is>
       </c>
-      <c r="B83" s="8">
+      <c r="B83" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>277581.62</v>
       </c>
-      <c r="C83" s="8">
+      <c r="C83" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>126727.21</v>
       </c>
-      <c r="D83" s="8">
+      <c r="D83" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>50804.68</v>
       </c>
-      <c r="E83" s="8">
+      <c r="E83" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>15251.95</v>
       </c>
-      <c r="F83" s="8">
+      <c r="F83" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>10057.66</v>
       </c>
-      <c r="G83" s="8">
+      <c r="G83" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>12090.23</v>
       </c>
-      <c r="H83" s="8">
+      <c r="H83" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>8065.26</v>
       </c>
-      <c r="I83" s="8">
+      <c r="I83" s="30">
         <f>SUM(B83:H83)-SUM(B82:H82)</f>
         <v>2519.03</v>
       </c>
@@ -2817,35 +2820,35 @@
           <t xml:space="preserve">May 2026</t>
         </is>
       </c>
-      <c r="B84" s="8">
+      <c r="B84" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>279126.78</v>
       </c>
-      <c r="C84" s="8">
+      <c r="C84" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>127308.41</v>
       </c>
-      <c r="D84" s="8">
+      <c r="D84" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>51076.04</v>
       </c>
-      <c r="E84" s="8">
+      <c r="E84" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>15315.63</v>
       </c>
-      <c r="F84" s="8">
+      <c r="F84" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>10076.96</v>
       </c>
-      <c r="G84" s="8">
+      <c r="G84" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>12120.45</v>
       </c>
-      <c r="H84" s="8">
+      <c r="H84" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>8087.13</v>
       </c>
-      <c r="I84" s="8">
+      <c r="I84" s="30">
         <f>SUM(B84:H84)-SUM(B83:H83)</f>
         <v>2532.8</v>
       </c>
@@ -2856,35 +2859,35 @@
           <t xml:space="preserve">Jun 2026</t>
         </is>
       </c>
-      <c r="B85" s="8">
+      <c r="B85" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>280681.02</v>
       </c>
-      <c r="C85" s="8">
+      <c r="C85" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>127892.36</v>
       </c>
-      <c r="D85" s="8">
+      <c r="D85" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>51348.99</v>
       </c>
-      <c r="E85" s="8">
+      <c r="E85" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>15379.57</v>
       </c>
-      <c r="F85" s="8">
+      <c r="F85" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>10096.29</v>
       </c>
-      <c r="G85" s="8">
+      <c r="G85" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>12150.75</v>
       </c>
-      <c r="H85" s="8">
+      <c r="H85" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>8109.07</v>
       </c>
-      <c r="I85" s="8">
+      <c r="I85" s="30">
         <f>SUM(B85:H85)-SUM(B84:H84)</f>
         <v>2546.64</v>
       </c>
@@ -2895,35 +2898,35 @@
           <t xml:space="preserve">Jul 2026</t>
         </is>
       </c>
-      <c r="B86" s="8">
+      <c r="B86" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>282244.39</v>
       </c>
-      <c r="C86" s="8">
+      <c r="C86" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>128479.08</v>
       </c>
-      <c r="D86" s="8">
+      <c r="D86" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>51623.53</v>
       </c>
-      <c r="E86" s="8">
+      <c r="E86" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>15443.78</v>
       </c>
-      <c r="F86" s="8">
+      <c r="F86" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>10115.66</v>
       </c>
-      <c r="G86" s="8">
+      <c r="G86" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>12181.13</v>
       </c>
-      <c r="H86" s="8">
+      <c r="H86" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>8131.06</v>
       </c>
-      <c r="I86" s="8">
+      <c r="I86" s="30">
         <f>SUM(B86:H86)-SUM(B85:H85)</f>
         <v>2560.57</v>
       </c>
@@ -2934,35 +2937,35 @@
           <t xml:space="preserve">Aug 2026</t>
         </is>
       </c>
-      <c r="B87" s="8">
+      <c r="B87" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>283816.94</v>
       </c>
-      <c r="C87" s="8">
+      <c r="C87" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>129068.58</v>
       </c>
-      <c r="D87" s="8">
+      <c r="D87" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>51899.67</v>
       </c>
-      <c r="E87" s="8">
+      <c r="E87" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>15508.26</v>
       </c>
-      <c r="F87" s="8">
+      <c r="F87" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>10135.07</v>
       </c>
-      <c r="G87" s="8">
+      <c r="G87" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>12211.58</v>
       </c>
-      <c r="H87" s="8">
+      <c r="H87" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>8153.11</v>
       </c>
-      <c r="I87" s="8">
+      <c r="I87" s="30">
         <f>SUM(B87:H87)-SUM(B86:H86)</f>
         <v>2574.59</v>
       </c>
@@ -2973,35 +2976,35 @@
           <t xml:space="preserve">Sep 2026</t>
         </is>
       </c>
-      <c r="B88" s="8">
+      <c r="B88" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>285398.74</v>
       </c>
-      <c r="C88" s="8">
+      <c r="C88" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>129660.87</v>
       </c>
-      <c r="D88" s="8">
+      <c r="D88" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>52177.43</v>
       </c>
-      <c r="E88" s="8">
+      <c r="E88" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>15573.01</v>
       </c>
-      <c r="F88" s="8">
+      <c r="F88" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>10154.51</v>
       </c>
-      <c r="G88" s="8">
+      <c r="G88" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>12242.11</v>
       </c>
-      <c r="H88" s="8">
+      <c r="H88" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>8175.22</v>
       </c>
-      <c r="I88" s="8">
+      <c r="I88" s="30">
         <f>SUM(B88:H88)-SUM(B87:H87)</f>
         <v>2588.68</v>
       </c>
@@ -3012,35 +3015,35 @@
           <t xml:space="preserve">Oct 2026</t>
         </is>
       </c>
-      <c r="B89" s="8">
+      <c r="B89" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>286989.84</v>
       </c>
-      <c r="C89" s="8">
+      <c r="C89" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>130255.96</v>
       </c>
-      <c r="D89" s="8">
+      <c r="D89" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>52456.82</v>
       </c>
-      <c r="E89" s="8">
+      <c r="E89" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>15638.03</v>
       </c>
-      <c r="F89" s="8">
+      <c r="F89" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>10173.99</v>
       </c>
-      <c r="G89" s="8">
+      <c r="G89" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>12272.72</v>
       </c>
-      <c r="H89" s="8">
+      <c r="H89" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>8197.39</v>
       </c>
-      <c r="I89" s="8">
+      <c r="I89" s="30">
         <f>SUM(B89:H89)-SUM(B88:H88)</f>
         <v>2602.86</v>
       </c>
@@ -3051,35 +3054,35 @@
           <t xml:space="preserve">Nov 2026</t>
         </is>
       </c>
-      <c r="B90" s="8">
+      <c r="B90" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>288590.3</v>
       </c>
-      <c r="C90" s="8">
+      <c r="C90" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>130853.88</v>
       </c>
-      <c r="D90" s="8">
+      <c r="D90" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>52737.84</v>
       </c>
-      <c r="E90" s="8">
+      <c r="E90" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>15703.32</v>
       </c>
-      <c r="F90" s="8">
+      <c r="F90" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>10193.51</v>
       </c>
-      <c r="G90" s="8">
+      <c r="G90" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>12303.4</v>
       </c>
-      <c r="H90" s="8">
+      <c r="H90" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>8219.62</v>
       </c>
-      <c r="I90" s="8">
+      <c r="I90" s="30">
         <f>SUM(B90:H90)-SUM(B89:H89)</f>
         <v>2617.12</v>
       </c>
@@ -3090,35 +3093,35 @@
           <t xml:space="preserve">Dec 2026</t>
         </is>
       </c>
-      <c r="B91" s="8">
+      <c r="B91" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>290200.18</v>
       </c>
-      <c r="C91" s="8">
+      <c r="C91" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>131454.63</v>
       </c>
-      <c r="D91" s="8">
+      <c r="D91" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>53020.5</v>
       </c>
-      <c r="E91" s="8">
+      <c r="E91" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>15768.88</v>
       </c>
-      <c r="F91" s="8">
+      <c r="F91" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>10213.06</v>
       </c>
-      <c r="G91" s="8">
+      <c r="G91" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>12334.16</v>
       </c>
-      <c r="H91" s="8">
+      <c r="H91" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>8241.91</v>
       </c>
-      <c r="I91" s="8">
+      <c r="I91" s="30">
         <f>SUM(B91:H91)-SUM(B90:H90)</f>
         <v>2631.46</v>
       </c>
@@ -3129,35 +3132,35 @@
           <t xml:space="preserve">Jan 2027</t>
         </is>
       </c>
-      <c r="B92" s="8">
+      <c r="B92" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>291819.54</v>
       </c>
-      <c r="C92" s="8">
+      <c r="C92" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>132058.23</v>
       </c>
-      <c r="D92" s="8">
+      <c r="D92" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>53304.82</v>
       </c>
-      <c r="E92" s="8">
+      <c r="E92" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>15834.72</v>
       </c>
-      <c r="F92" s="8">
+      <c r="F92" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>10232.66</v>
       </c>
-      <c r="G92" s="8">
+      <c r="G92" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>12364.99</v>
       </c>
-      <c r="H92" s="8">
+      <c r="H92" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>8264.26</v>
       </c>
-      <c r="I92" s="8">
+      <c r="I92" s="30">
         <f>SUM(B92:H92)-SUM(B91:H91)</f>
         <v>2645.89</v>
       </c>
@@ -3168,35 +3171,35 @@
           <t xml:space="preserve">Feb 2027</t>
         </is>
       </c>
-      <c r="B93" s="8">
+      <c r="B93" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>293448.43</v>
       </c>
-      <c r="C93" s="8">
+      <c r="C93" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>132664.69</v>
       </c>
-      <c r="D93" s="8">
+      <c r="D93" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>53590.8</v>
       </c>
-      <c r="E93" s="8">
+      <c r="E93" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>15900.83</v>
       </c>
-      <c r="F93" s="8">
+      <c r="F93" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>10252.29</v>
       </c>
-      <c r="G93" s="8">
+      <c r="G93" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>12395.9</v>
       </c>
-      <c r="H93" s="8">
+      <c r="H93" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>8286.67</v>
       </c>
-      <c r="I93" s="8">
+      <c r="I93" s="30">
         <f>SUM(B93:H93)-SUM(B92:H92)</f>
         <v>2660.4</v>
       </c>
@@ -3207,35 +3210,35 @@
           <t xml:space="preserve">Mar 2027</t>
         </is>
       </c>
-      <c r="B94" s="8">
+      <c r="B94" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>295086.93</v>
       </c>
-      <c r="C94" s="8">
+      <c r="C94" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>133274.02</v>
       </c>
-      <c r="D94" s="8">
+      <c r="D94" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>53878.46</v>
       </c>
-      <c r="E94" s="8">
+      <c r="E94" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>15967.21</v>
       </c>
-      <c r="F94" s="8">
+      <c r="F94" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>10271.96</v>
       </c>
-      <c r="G94" s="8">
+      <c r="G94" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>12426.89</v>
       </c>
-      <c r="H94" s="8">
+      <c r="H94" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>8309.14</v>
       </c>
-      <c r="I94" s="8">
+      <c r="I94" s="30">
         <f>SUM(B94:H94)-SUM(B93:H93)</f>
         <v>2675.0</v>
       </c>
@@ -3246,35 +3249,35 @@
           <t xml:space="preserve">Apr 2027</t>
         </is>
       </c>
-      <c r="B95" s="8">
+      <c r="B95" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>296735.08</v>
       </c>
-      <c r="C95" s="8">
+      <c r="C95" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>133886.25</v>
       </c>
-      <c r="D95" s="8">
+      <c r="D95" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>54167.8</v>
       </c>
-      <c r="E95" s="8">
+      <c r="E95" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>16033.88</v>
       </c>
-      <c r="F95" s="8">
+      <c r="F95" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>10291.66</v>
       </c>
-      <c r="G95" s="8">
+      <c r="G95" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>12457.96</v>
       </c>
-      <c r="H95" s="8">
+      <c r="H95" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>8331.68</v>
       </c>
-      <c r="I95" s="8">
+      <c r="I95" s="30">
         <f>SUM(B95:H95)-SUM(B94:H94)</f>
         <v>2689.69</v>
       </c>
@@ -3285,35 +3288,35 @@
           <t xml:space="preserve">May 2027</t>
         </is>
       </c>
-      <c r="B96" s="8">
+      <c r="B96" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>298392.95</v>
       </c>
-      <c r="C96" s="8">
+      <c r="C96" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>134501.37</v>
       </c>
-      <c r="D96" s="8">
+      <c r="D96" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>54458.84</v>
       </c>
-      <c r="E96" s="8">
+      <c r="E96" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>16100.82</v>
       </c>
-      <c r="F96" s="8">
+      <c r="F96" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>10311.41</v>
       </c>
-      <c r="G96" s="8">
+      <c r="G96" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>12489.11</v>
       </c>
-      <c r="H96" s="8">
+      <c r="H96" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>8354.27</v>
       </c>
-      <c r="I96" s="8">
+      <c r="I96" s="30">
         <f>SUM(B96:H96)-SUM(B95:H95)</f>
         <v>2704.46</v>
       </c>
@@ -3324,35 +3327,35 @@
           <t xml:space="preserve">Jun 2027</t>
         </is>
       </c>
-      <c r="B97" s="8">
+      <c r="B97" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>300060.6</v>
       </c>
-      <c r="C97" s="8">
+      <c r="C97" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>135119.42</v>
       </c>
-      <c r="D97" s="8">
+      <c r="D97" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>54751.59</v>
       </c>
-      <c r="E97" s="8">
+      <c r="E97" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>16168.04</v>
       </c>
-      <c r="F97" s="8">
+      <c r="F97" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>10331.19</v>
       </c>
-      <c r="G97" s="8">
+      <c r="G97" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>12520.33</v>
       </c>
-      <c r="H97" s="8">
+      <c r="H97" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>8376.93</v>
       </c>
-      <c r="I97" s="8">
+      <c r="I97" s="30">
         <f>SUM(B97:H97)-SUM(B96:H96)</f>
         <v>2719.32</v>
       </c>
@@ -3363,35 +3366,35 @@
           <t xml:space="preserve">Jul 2027</t>
         </is>
       </c>
-      <c r="B98" s="8">
+      <c r="B98" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>301738.1</v>
       </c>
-      <c r="C98" s="8">
+      <c r="C98" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>135740.39</v>
       </c>
-      <c r="D98" s="8">
+      <c r="D98" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>55046.05</v>
       </c>
-      <c r="E98" s="8">
+      <c r="E98" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>16235.55</v>
       </c>
-      <c r="F98" s="8">
+      <c r="F98" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>10351.01</v>
       </c>
-      <c r="G98" s="8">
+      <c r="G98" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>12551.63</v>
       </c>
-      <c r="H98" s="8">
+      <c r="H98" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>8399.64</v>
       </c>
-      <c r="I98" s="8">
+      <c r="I98" s="30">
         <f>SUM(B98:H98)-SUM(B97:H97)</f>
         <v>2734.27</v>
       </c>
@@ -3402,35 +3405,35 @@
           <t xml:space="preserve">Aug 2027</t>
         </is>
       </c>
-      <c r="B99" s="8">
+      <c r="B99" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>303425.49</v>
       </c>
-      <c r="C99" s="8">
+      <c r="C99" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>136364.31</v>
       </c>
-      <c r="D99" s="8">
+      <c r="D99" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>55342.24</v>
       </c>
-      <c r="E99" s="8">
+      <c r="E99" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>16303.33</v>
       </c>
-      <c r="F99" s="8">
+      <c r="F99" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>10370.87</v>
       </c>
-      <c r="G99" s="8">
+      <c r="G99" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>12583.01</v>
       </c>
-      <c r="H99" s="8">
+      <c r="H99" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>8422.42</v>
       </c>
-      <c r="I99" s="8">
+      <c r="I99" s="30">
         <f>SUM(B99:H99)-SUM(B98:H98)</f>
         <v>2749.31</v>
       </c>
@@ -3441,35 +3444,35 @@
           <t xml:space="preserve">Sep 2027</t>
         </is>
       </c>
-      <c r="B100" s="8">
+      <c r="B100" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>305122.85</v>
       </c>
-      <c r="C100" s="8">
+      <c r="C100" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>136991.19</v>
       </c>
-      <c r="D100" s="8">
+      <c r="D100" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>55640.17</v>
       </c>
-      <c r="E100" s="8">
+      <c r="E100" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>16371.4</v>
       </c>
-      <c r="F100" s="8">
+      <c r="F100" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>10390.76</v>
       </c>
-      <c r="G100" s="8">
+      <c r="G100" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>12614.47</v>
       </c>
-      <c r="H100" s="8">
+      <c r="H100" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>8445.26</v>
       </c>
-      <c r="I100" s="8">
+      <c r="I100" s="30">
         <f>SUM(B100:H100)-SUM(B99:H99)</f>
         <v>2764.43</v>
       </c>
@@ -3480,35 +3483,35 @@
           <t xml:space="preserve">Oct 2027</t>
         </is>
       </c>
-      <c r="B101" s="8">
+      <c r="B101" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>306830.24</v>
       </c>
-      <c r="C101" s="8">
+      <c r="C101" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>137621.04</v>
       </c>
-      <c r="D101" s="8">
+      <c r="D101" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>55939.85</v>
       </c>
-      <c r="E101" s="8">
+      <c r="E101" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>16439.75</v>
       </c>
-      <c r="F101" s="8">
+      <c r="F101" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>10410.7</v>
       </c>
-      <c r="G101" s="8">
+      <c r="G101" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>12646.0</v>
       </c>
-      <c r="H101" s="8">
+      <c r="H101" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>8468.17</v>
       </c>
-      <c r="I101" s="8">
+      <c r="I101" s="30">
         <f>SUM(B101:H101)-SUM(B100:H100)</f>
         <v>2779.65</v>
       </c>
@@ -3519,35 +3522,35 @@
           <t xml:space="preserve">Nov 2027</t>
         </is>
       </c>
-      <c r="B102" s="8">
+      <c r="B102" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>308547.73</v>
       </c>
-      <c r="C102" s="8">
+      <c r="C102" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>138253.89</v>
       </c>
-      <c r="D102" s="8">
+      <c r="D102" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>56241.29</v>
       </c>
-      <c r="E102" s="8">
+      <c r="E102" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>16508.39</v>
       </c>
-      <c r="F102" s="8">
+      <c r="F102" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>10430.67</v>
       </c>
-      <c r="G102" s="8">
+      <c r="G102" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>12677.62</v>
       </c>
-      <c r="H102" s="8">
+      <c r="H102" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>8491.13</v>
       </c>
-      <c r="I102" s="8">
+      <c r="I102" s="30">
         <f>SUM(B102:H102)-SUM(B101:H101)</f>
         <v>2794.95</v>
       </c>
@@ -3558,35 +3561,35 @@
           <t xml:space="preserve">Dec 2027</t>
         </is>
       </c>
-      <c r="B103" s="8">
+      <c r="B103" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>310275.36</v>
       </c>
-      <c r="C103" s="8">
+      <c r="C103" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>138889.73</v>
       </c>
-      <c r="D103" s="8">
+      <c r="D103" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>56544.5</v>
       </c>
-      <c r="E103" s="8">
+      <c r="E103" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>16577.31</v>
       </c>
-      <c r="F103" s="8">
+      <c r="F103" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>10450.68</v>
       </c>
-      <c r="G103" s="8">
+      <c r="G103" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>12709.31</v>
       </c>
-      <c r="H103" s="8">
+      <c r="H103" s="30">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>8514.16</v>
       </c>
-      <c r="I103" s="8">
+      <c r="I103" s="30">
         <f>SUM(B103:H103)-SUM(B102:H102)</f>
         <v>2810.35</v>
       </c>

</xml_diff>

<commit_message>
Use PHP currency format for all amount cells (chart-data matrix) + widen columns
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -2192,13 +2192,13 @@
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
@@ -2665,35 +2665,35 @@
           <t xml:space="preserve">Jan 2026</t>
         </is>
       </c>
-      <c r="B80" s="30">
+      <c r="B80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>273000.0</v>
       </c>
-      <c r="C80" s="30">
+      <c r="C80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>125000.0</v>
       </c>
-      <c r="D80" s="30">
+      <c r="D80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>50000.0</v>
       </c>
-      <c r="E80" s="30">
+      <c r="E80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>15062.5</v>
       </c>
-      <c r="F80" s="30">
+      <c r="F80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>10000.0</v>
       </c>
-      <c r="G80" s="30">
+      <c r="G80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>12000.0</v>
       </c>
-      <c r="H80" s="30">
+      <c r="H80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
         <v>8000.0</v>
       </c>
-      <c r="I80" s="30">
+      <c r="I80" s="8">
         <v>0</v>
       </c>
     </row>
@@ -2703,35 +2703,35 @@
           <t xml:space="preserve">Feb 2026</t>
         </is>
       </c>
-      <c r="B81" s="30">
+      <c r="B81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>274518.28</v>
       </c>
-      <c r="C81" s="30">
+      <c r="C81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>125573.02</v>
       </c>
-      <c r="D81" s="30">
+      <c r="D81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>50266.67</v>
       </c>
-      <c r="E81" s="30">
+      <c r="E81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>15125.39</v>
       </c>
-      <c r="F81" s="30">
+      <c r="F81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>10019.18</v>
       </c>
-      <c r="G81" s="30">
+      <c r="G81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>12030.0</v>
       </c>
-      <c r="H81" s="30">
+      <c r="H81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
         <v>8021.7</v>
       </c>
-      <c r="I81" s="30">
+      <c r="I81" s="8">
         <f>SUM(B81:H81)-SUM(B80:H80)</f>
         <v>2491.74</v>
       </c>
@@ -2742,35 +2742,35 @@
           <t xml:space="preserve">Mar 2026</t>
         </is>
       </c>
-      <c r="B82" s="30">
+      <c r="B82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>276045.47</v>
       </c>
-      <c r="C82" s="30">
+      <c r="C82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>126148.75</v>
       </c>
-      <c r="D82" s="30">
+      <c r="D82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>50534.89</v>
       </c>
-      <c r="E82" s="30">
+      <c r="E82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>15188.54</v>
       </c>
-      <c r="F82" s="30">
+      <c r="F82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>10038.41</v>
       </c>
-      <c r="G82" s="30">
+      <c r="G82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>12060.07</v>
       </c>
-      <c r="H82" s="30">
+      <c r="H82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
         <v>8043.45</v>
       </c>
-      <c r="I82" s="30">
+      <c r="I82" s="8">
         <f>SUM(B82:H82)-SUM(B81:H81)</f>
         <v>2505.34</v>
       </c>
@@ -2781,35 +2781,35 @@
           <t xml:space="preserve">Apr 2026</t>
         </is>
       </c>
-      <c r="B83" s="30">
+      <c r="B83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>277581.62</v>
       </c>
-      <c r="C83" s="30">
+      <c r="C83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>126727.21</v>
       </c>
-      <c r="D83" s="30">
+      <c r="D83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>50804.68</v>
       </c>
-      <c r="E83" s="30">
+      <c r="E83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>15251.95</v>
       </c>
-      <c r="F83" s="30">
+      <c r="F83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>10057.66</v>
       </c>
-      <c r="G83" s="30">
+      <c r="G83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>12090.23</v>
       </c>
-      <c r="H83" s="30">
+      <c r="H83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
         <v>8065.26</v>
       </c>
-      <c r="I83" s="30">
+      <c r="I83" s="8">
         <f>SUM(B83:H83)-SUM(B82:H82)</f>
         <v>2519.03</v>
       </c>
@@ -2820,35 +2820,35 @@
           <t xml:space="preserve">May 2026</t>
         </is>
       </c>
-      <c r="B84" s="30">
+      <c r="B84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>279126.78</v>
       </c>
-      <c r="C84" s="30">
+      <c r="C84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>127308.41</v>
       </c>
-      <c r="D84" s="30">
+      <c r="D84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>51076.04</v>
       </c>
-      <c r="E84" s="30">
+      <c r="E84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>15315.63</v>
       </c>
-      <c r="F84" s="30">
+      <c r="F84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>10076.96</v>
       </c>
-      <c r="G84" s="30">
+      <c r="G84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>12120.45</v>
       </c>
-      <c r="H84" s="30">
+      <c r="H84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
         <v>8087.13</v>
       </c>
-      <c r="I84" s="30">
+      <c r="I84" s="8">
         <f>SUM(B84:H84)-SUM(B83:H83)</f>
         <v>2532.8</v>
       </c>
@@ -2859,35 +2859,35 @@
           <t xml:space="preserve">Jun 2026</t>
         </is>
       </c>
-      <c r="B85" s="30">
+      <c r="B85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>280681.02</v>
       </c>
-      <c r="C85" s="30">
+      <c r="C85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>127892.36</v>
       </c>
-      <c r="D85" s="30">
+      <c r="D85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>51348.99</v>
       </c>
-      <c r="E85" s="30">
+      <c r="E85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>15379.57</v>
       </c>
-      <c r="F85" s="30">
+      <c r="F85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>10096.29</v>
       </c>
-      <c r="G85" s="30">
+      <c r="G85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>12150.75</v>
       </c>
-      <c r="H85" s="30">
+      <c r="H85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
         <v>8109.07</v>
       </c>
-      <c r="I85" s="30">
+      <c r="I85" s="8">
         <f>SUM(B85:H85)-SUM(B84:H84)</f>
         <v>2546.64</v>
       </c>
@@ -2898,35 +2898,35 @@
           <t xml:space="preserve">Jul 2026</t>
         </is>
       </c>
-      <c r="B86" s="30">
+      <c r="B86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>282244.39</v>
       </c>
-      <c r="C86" s="30">
+      <c r="C86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>128479.08</v>
       </c>
-      <c r="D86" s="30">
+      <c r="D86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>51623.53</v>
       </c>
-      <c r="E86" s="30">
+      <c r="E86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>15443.78</v>
       </c>
-      <c r="F86" s="30">
+      <c r="F86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>10115.66</v>
       </c>
-      <c r="G86" s="30">
+      <c r="G86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>12181.13</v>
       </c>
-      <c r="H86" s="30">
+      <c r="H86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
         <v>8131.06</v>
       </c>
-      <c r="I86" s="30">
+      <c r="I86" s="8">
         <f>SUM(B86:H86)-SUM(B85:H85)</f>
         <v>2560.57</v>
       </c>
@@ -2937,35 +2937,35 @@
           <t xml:space="preserve">Aug 2026</t>
         </is>
       </c>
-      <c r="B87" s="30">
+      <c r="B87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>283816.94</v>
       </c>
-      <c r="C87" s="30">
+      <c r="C87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>129068.58</v>
       </c>
-      <c r="D87" s="30">
+      <c r="D87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>51899.67</v>
       </c>
-      <c r="E87" s="30">
+      <c r="E87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>15508.26</v>
       </c>
-      <c r="F87" s="30">
+      <c r="F87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>10135.07</v>
       </c>
-      <c r="G87" s="30">
+      <c r="G87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>12211.58</v>
       </c>
-      <c r="H87" s="30">
+      <c r="H87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
         <v>8153.11</v>
       </c>
-      <c r="I87" s="30">
+      <c r="I87" s="8">
         <f>SUM(B87:H87)-SUM(B86:H86)</f>
         <v>2574.59</v>
       </c>
@@ -2976,35 +2976,35 @@
           <t xml:space="preserve">Sep 2026</t>
         </is>
       </c>
-      <c r="B88" s="30">
+      <c r="B88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>285398.74</v>
       </c>
-      <c r="C88" s="30">
+      <c r="C88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>129660.87</v>
       </c>
-      <c r="D88" s="30">
+      <c r="D88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>52177.43</v>
       </c>
-      <c r="E88" s="30">
+      <c r="E88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>15573.01</v>
       </c>
-      <c r="F88" s="30">
+      <c r="F88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>10154.51</v>
       </c>
-      <c r="G88" s="30">
+      <c r="G88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>12242.11</v>
       </c>
-      <c r="H88" s="30">
+      <c r="H88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
         <v>8175.22</v>
       </c>
-      <c r="I88" s="30">
+      <c r="I88" s="8">
         <f>SUM(B88:H88)-SUM(B87:H87)</f>
         <v>2588.68</v>
       </c>
@@ -3015,35 +3015,35 @@
           <t xml:space="preserve">Oct 2026</t>
         </is>
       </c>
-      <c r="B89" s="30">
+      <c r="B89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>286989.84</v>
       </c>
-      <c r="C89" s="30">
+      <c r="C89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>130255.96</v>
       </c>
-      <c r="D89" s="30">
+      <c r="D89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>52456.82</v>
       </c>
-      <c r="E89" s="30">
+      <c r="E89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>15638.03</v>
       </c>
-      <c r="F89" s="30">
+      <c r="F89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>10173.99</v>
       </c>
-      <c r="G89" s="30">
+      <c r="G89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>12272.72</v>
       </c>
-      <c r="H89" s="30">
+      <c r="H89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
         <v>8197.39</v>
       </c>
-      <c r="I89" s="30">
+      <c r="I89" s="8">
         <f>SUM(B89:H89)-SUM(B88:H88)</f>
         <v>2602.86</v>
       </c>
@@ -3054,35 +3054,35 @@
           <t xml:space="preserve">Nov 2026</t>
         </is>
       </c>
-      <c r="B90" s="30">
+      <c r="B90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>288590.3</v>
       </c>
-      <c r="C90" s="30">
+      <c r="C90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>130853.88</v>
       </c>
-      <c r="D90" s="30">
+      <c r="D90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>52737.84</v>
       </c>
-      <c r="E90" s="30">
+      <c r="E90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>15703.32</v>
       </c>
-      <c r="F90" s="30">
+      <c r="F90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>10193.51</v>
       </c>
-      <c r="G90" s="30">
+      <c r="G90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>12303.4</v>
       </c>
-      <c r="H90" s="30">
+      <c r="H90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
         <v>8219.62</v>
       </c>
-      <c r="I90" s="30">
+      <c r="I90" s="8">
         <f>SUM(B90:H90)-SUM(B89:H89)</f>
         <v>2617.12</v>
       </c>
@@ -3093,35 +3093,35 @@
           <t xml:space="preserve">Dec 2026</t>
         </is>
       </c>
-      <c r="B91" s="30">
+      <c r="B91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>290200.18</v>
       </c>
-      <c r="C91" s="30">
+      <c r="C91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>131454.63</v>
       </c>
-      <c r="D91" s="30">
+      <c r="D91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>53020.5</v>
       </c>
-      <c r="E91" s="30">
+      <c r="E91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>15768.88</v>
       </c>
-      <c r="F91" s="30">
+      <c r="F91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>10213.06</v>
       </c>
-      <c r="G91" s="30">
+      <c r="G91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>12334.16</v>
       </c>
-      <c r="H91" s="30">
+      <c r="H91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
         <v>8241.91</v>
       </c>
-      <c r="I91" s="30">
+      <c r="I91" s="8">
         <f>SUM(B91:H91)-SUM(B90:H90)</f>
         <v>2631.46</v>
       </c>
@@ -3132,35 +3132,35 @@
           <t xml:space="preserve">Jan 2027</t>
         </is>
       </c>
-      <c r="B92" s="30">
+      <c r="B92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>291819.54</v>
       </c>
-      <c r="C92" s="30">
+      <c r="C92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>132058.23</v>
       </c>
-      <c r="D92" s="30">
+      <c r="D92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>53304.82</v>
       </c>
-      <c r="E92" s="30">
+      <c r="E92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>15834.72</v>
       </c>
-      <c r="F92" s="30">
+      <c r="F92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>10232.66</v>
       </c>
-      <c r="G92" s="30">
+      <c r="G92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>12364.99</v>
       </c>
-      <c r="H92" s="30">
+      <c r="H92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
         <v>8264.26</v>
       </c>
-      <c r="I92" s="30">
+      <c r="I92" s="8">
         <f>SUM(B92:H92)-SUM(B91:H91)</f>
         <v>2645.89</v>
       </c>
@@ -3171,35 +3171,35 @@
           <t xml:space="preserve">Feb 2027</t>
         </is>
       </c>
-      <c r="B93" s="30">
+      <c r="B93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>293448.43</v>
       </c>
-      <c r="C93" s="30">
+      <c r="C93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>132664.69</v>
       </c>
-      <c r="D93" s="30">
+      <c r="D93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>53590.8</v>
       </c>
-      <c r="E93" s="30">
+      <c r="E93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>15900.83</v>
       </c>
-      <c r="F93" s="30">
+      <c r="F93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>10252.29</v>
       </c>
-      <c r="G93" s="30">
+      <c r="G93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>12395.9</v>
       </c>
-      <c r="H93" s="30">
+      <c r="H93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
         <v>8286.67</v>
       </c>
-      <c r="I93" s="30">
+      <c r="I93" s="8">
         <f>SUM(B93:H93)-SUM(B92:H92)</f>
         <v>2660.4</v>
       </c>
@@ -3210,35 +3210,35 @@
           <t xml:space="preserve">Mar 2027</t>
         </is>
       </c>
-      <c r="B94" s="30">
+      <c r="B94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>295086.93</v>
       </c>
-      <c r="C94" s="30">
+      <c r="C94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>133274.02</v>
       </c>
-      <c r="D94" s="30">
+      <c r="D94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>53878.46</v>
       </c>
-      <c r="E94" s="30">
+      <c r="E94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>15967.21</v>
       </c>
-      <c r="F94" s="30">
+      <c r="F94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>10271.96</v>
       </c>
-      <c r="G94" s="30">
+      <c r="G94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>12426.89</v>
       </c>
-      <c r="H94" s="30">
+      <c r="H94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
         <v>8309.14</v>
       </c>
-      <c r="I94" s="30">
+      <c r="I94" s="8">
         <f>SUM(B94:H94)-SUM(B93:H93)</f>
         <v>2675.0</v>
       </c>
@@ -3249,35 +3249,35 @@
           <t xml:space="preserve">Apr 2027</t>
         </is>
       </c>
-      <c r="B95" s="30">
+      <c r="B95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>296735.08</v>
       </c>
-      <c r="C95" s="30">
+      <c r="C95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>133886.25</v>
       </c>
-      <c r="D95" s="30">
+      <c r="D95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>54167.8</v>
       </c>
-      <c r="E95" s="30">
+      <c r="E95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>16033.88</v>
       </c>
-      <c r="F95" s="30">
+      <c r="F95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>10291.66</v>
       </c>
-      <c r="G95" s="30">
+      <c r="G95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>12457.96</v>
       </c>
-      <c r="H95" s="30">
+      <c r="H95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
         <v>8331.68</v>
       </c>
-      <c r="I95" s="30">
+      <c r="I95" s="8">
         <f>SUM(B95:H95)-SUM(B94:H94)</f>
         <v>2689.69</v>
       </c>
@@ -3288,35 +3288,35 @@
           <t xml:space="preserve">May 2027</t>
         </is>
       </c>
-      <c r="B96" s="30">
+      <c r="B96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>298392.95</v>
       </c>
-      <c r="C96" s="30">
+      <c r="C96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>134501.37</v>
       </c>
-      <c r="D96" s="30">
+      <c r="D96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>54458.84</v>
       </c>
-      <c r="E96" s="30">
+      <c r="E96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>16100.82</v>
       </c>
-      <c r="F96" s="30">
+      <c r="F96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>10311.41</v>
       </c>
-      <c r="G96" s="30">
+      <c r="G96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>12489.11</v>
       </c>
-      <c r="H96" s="30">
+      <c r="H96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
         <v>8354.27</v>
       </c>
-      <c r="I96" s="30">
+      <c r="I96" s="8">
         <f>SUM(B96:H96)-SUM(B95:H95)</f>
         <v>2704.46</v>
       </c>
@@ -3327,35 +3327,35 @@
           <t xml:space="preserve">Jun 2027</t>
         </is>
       </c>
-      <c r="B97" s="30">
+      <c r="B97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>300060.6</v>
       </c>
-      <c r="C97" s="30">
+      <c r="C97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>135119.42</v>
       </c>
-      <c r="D97" s="30">
+      <c r="D97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>54751.59</v>
       </c>
-      <c r="E97" s="30">
+      <c r="E97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>16168.04</v>
       </c>
-      <c r="F97" s="30">
+      <c r="F97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>10331.19</v>
       </c>
-      <c r="G97" s="30">
+      <c r="G97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>12520.33</v>
       </c>
-      <c r="H97" s="30">
+      <c r="H97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
         <v>8376.93</v>
       </c>
-      <c r="I97" s="30">
+      <c r="I97" s="8">
         <f>SUM(B97:H97)-SUM(B96:H96)</f>
         <v>2719.32</v>
       </c>
@@ -3366,35 +3366,35 @@
           <t xml:space="preserve">Jul 2027</t>
         </is>
       </c>
-      <c r="B98" s="30">
+      <c r="B98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>301738.1</v>
       </c>
-      <c r="C98" s="30">
+      <c r="C98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>135740.39</v>
       </c>
-      <c r="D98" s="30">
+      <c r="D98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>55046.05</v>
       </c>
-      <c r="E98" s="30">
+      <c r="E98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>16235.55</v>
       </c>
-      <c r="F98" s="30">
+      <c r="F98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>10351.01</v>
       </c>
-      <c r="G98" s="30">
+      <c r="G98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>12551.63</v>
       </c>
-      <c r="H98" s="30">
+      <c r="H98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
         <v>8399.64</v>
       </c>
-      <c r="I98" s="30">
+      <c r="I98" s="8">
         <f>SUM(B98:H98)-SUM(B97:H97)</f>
         <v>2734.27</v>
       </c>
@@ -3405,35 +3405,35 @@
           <t xml:space="preserve">Aug 2027</t>
         </is>
       </c>
-      <c r="B99" s="30">
+      <c r="B99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>303425.49</v>
       </c>
-      <c r="C99" s="30">
+      <c r="C99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>136364.31</v>
       </c>
-      <c r="D99" s="30">
+      <c r="D99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>55342.24</v>
       </c>
-      <c r="E99" s="30">
+      <c r="E99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>16303.33</v>
       </c>
-      <c r="F99" s="30">
+      <c r="F99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>10370.87</v>
       </c>
-      <c r="G99" s="30">
+      <c r="G99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>12583.01</v>
       </c>
-      <c r="H99" s="30">
+      <c r="H99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
         <v>8422.42</v>
       </c>
-      <c r="I99" s="30">
+      <c r="I99" s="8">
         <f>SUM(B99:H99)-SUM(B98:H98)</f>
         <v>2749.31</v>
       </c>
@@ -3444,35 +3444,35 @@
           <t xml:space="preserve">Sep 2027</t>
         </is>
       </c>
-      <c r="B100" s="30">
+      <c r="B100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>305122.85</v>
       </c>
-      <c r="C100" s="30">
+      <c r="C100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>136991.19</v>
       </c>
-      <c r="D100" s="30">
+      <c r="D100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>55640.17</v>
       </c>
-      <c r="E100" s="30">
+      <c r="E100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>16371.4</v>
       </c>
-      <c r="F100" s="30">
+      <c r="F100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>10390.76</v>
       </c>
-      <c r="G100" s="30">
+      <c r="G100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>12614.47</v>
       </c>
-      <c r="H100" s="30">
+      <c r="H100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
         <v>8445.26</v>
       </c>
-      <c r="I100" s="30">
+      <c r="I100" s="8">
         <f>SUM(B100:H100)-SUM(B99:H99)</f>
         <v>2764.43</v>
       </c>
@@ -3483,35 +3483,35 @@
           <t xml:space="preserve">Oct 2027</t>
         </is>
       </c>
-      <c r="B101" s="30">
+      <c r="B101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>306830.24</v>
       </c>
-      <c r="C101" s="30">
+      <c r="C101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>137621.04</v>
       </c>
-      <c r="D101" s="30">
+      <c r="D101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>55939.85</v>
       </c>
-      <c r="E101" s="30">
+      <c r="E101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>16439.75</v>
       </c>
-      <c r="F101" s="30">
+      <c r="F101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>10410.7</v>
       </c>
-      <c r="G101" s="30">
+      <c r="G101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>12646.0</v>
       </c>
-      <c r="H101" s="30">
+      <c r="H101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
         <v>8468.17</v>
       </c>
-      <c r="I101" s="30">
+      <c r="I101" s="8">
         <f>SUM(B101:H101)-SUM(B100:H100)</f>
         <v>2779.65</v>
       </c>
@@ -3522,35 +3522,35 @@
           <t xml:space="preserve">Nov 2027</t>
         </is>
       </c>
-      <c r="B102" s="30">
+      <c r="B102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>308547.73</v>
       </c>
-      <c r="C102" s="30">
+      <c r="C102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>138253.89</v>
       </c>
-      <c r="D102" s="30">
+      <c r="D102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>56241.29</v>
       </c>
-      <c r="E102" s="30">
+      <c r="E102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>16508.39</v>
       </c>
-      <c r="F102" s="30">
+      <c r="F102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>10430.67</v>
       </c>
-      <c r="G102" s="30">
+      <c r="G102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>12677.62</v>
       </c>
-      <c r="H102" s="30">
+      <c r="H102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
         <v>8491.13</v>
       </c>
-      <c r="I102" s="30">
+      <c r="I102" s="8">
         <f>SUM(B102:H102)-SUM(B101:H101)</f>
         <v>2794.95</v>
       </c>
@@ -3561,35 +3561,35 @@
           <t xml:space="preserve">Dec 2027</t>
         </is>
       </c>
-      <c r="B103" s="30">
+      <c r="B103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=B$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>310275.36</v>
       </c>
-      <c r="C103" s="30">
+      <c r="C103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=C$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>138889.73</v>
       </c>
-      <c r="D103" s="30">
+      <c r="D103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=D$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>56544.5</v>
       </c>
-      <c r="E103" s="30">
+      <c r="E103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>16577.31</v>
       </c>
-      <c r="F103" s="30">
+      <c r="F103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>10450.68</v>
       </c>
-      <c r="G103" s="30">
+      <c r="G103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=G$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>12709.31</v>
       </c>
-      <c r="H103" s="30">
+      <c r="H103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=H$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
         <v>8514.16</v>
       </c>
-      <c r="I103" s="30">
+      <c r="I103" s="8">
         <f>SUM(B103:H103)-SUM(B102:H102)</f>
         <v>2810.35</v>
       </c>

</xml_diff>

<commit_message>
Fix Savings-by-Bank pie (SUMIF used Account col, not Bank); make Monthly Interest a stacked column per bank
- Balance-by-Bank SUMIF criteria range corrected from Balance col B (Account) to col A (Bank); fixes zero balances + empty pie
- Monthly Interest Earned is now a stacked column chart with one segment per bank (7 series), driven by a new per-bank monthly-interest data block
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -1808,7 +1808,7 @@
                   <a:srgbClr val="1F3864"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Monthly Interest Earned</a:t>
+              <a:t>Monthly Interest Earned by Bank</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1820,30 +1820,30 @@
       <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
+        <c:grouping val="stacked"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Dashboard!$I$79</c:f>
+              <c:f>Dashboard!$B$106</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Interest Earned</c:v>
+                  <c:v>Maya</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="548235"/>
+              <a:srgbClr val="4472C4"/>
             </a:solidFill>
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$80:$A$103</c:f>
+              <c:f>Dashboard!$A$107:$A$130</c:f>
               <c:strCache>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
@@ -1923,7 +1923,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$I$80:$I$103</c:f>
+              <c:f>Dashboard!$B$107:$B$130</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
@@ -1931,78 +1931,1166 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2491.7355</c:v>
+                  <c:v>1518.2827</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2505.3423</c:v>
+                  <c:v>1527.1875</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2519.029</c:v>
+                  <c:v>1536.1479</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2532.7962</c:v>
+                  <c:v>1545.1644</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2546.6443</c:v>
+                  <c:v>1554.2372</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2560.5738</c:v>
+                  <c:v>1563.3669</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2574.5853</c:v>
+                  <c:v>1572.5537</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2588.6792</c:v>
+                  <c:v>1581.798</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2602.8562</c:v>
+                  <c:v>1591.1003</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2617.1167</c:v>
+                  <c:v>1600.4609</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2631.4612</c:v>
+                  <c:v>1609.8802</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2645.8903</c:v>
+                  <c:v>1619.3586</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2660.4045</c:v>
+                  <c:v>1628.8965</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2675.0044</c:v>
+                  <c:v>1638.4942</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2689.6904</c:v>
+                  <c:v>1648.1523</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2704.4633</c:v>
+                  <c:v>1657.8711</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2719.3234</c:v>
+                  <c:v>1667.6511</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2734.2713</c:v>
+                  <c:v>1677.4925</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2749.3077</c:v>
+                  <c:v>1687.3959</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2764.433</c:v>
+                  <c:v>1697.3616</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2779.6479</c:v>
+                  <c:v>1707.3902</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2794.9528</c:v>
+                  <c:v>1717.4819</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>2810.3485</c:v>
+                  <c:v>1727.6372</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$C$106</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>UNO</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="ED7D31"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$107:$A$130</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$C$107:$C$130</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>573.0196</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>575.7329</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>578.4593</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>581.1989</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>583.9517</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>586.7178</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>589.4974</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>592.2904</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>595.0969</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>597.9169</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>600.7507</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>603.5981</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>606.4593</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>609.3344</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>612.2234</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>615.1263</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>618.0433</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>620.9745</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>623.9198</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>626.8794</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>629.8533</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>632.8417</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>635.8445</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$D$106</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Tonik</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="70AD47"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$107:$A$130</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$D$107:$D$130</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>266.6667</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>268.2222</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>269.7874</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>271.3623</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>272.9469</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>274.5414</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>276.1457</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>277.76</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>279.3842</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>281.0186</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>282.663</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>284.3177</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>285.9827</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>287.6579</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>289.3436</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>291.0398</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>292.7464</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>294.4637</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>296.1916</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>297.9303</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>299.6798</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>301.4401</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>303.2114</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$E$106</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Banko</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$107:$A$130</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$E$107:$E$130</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>62.887</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>63.1496</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>63.4132</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>63.678</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>63.9439</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>64.2108</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>64.4789</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>64.7481</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>65.0184</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>65.2899</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>65.5625</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>65.8362</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>66.1111</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>66.3871</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>66.6643</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>66.9426</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>67.2221</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>67.5028</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>67.7846</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>68.0676</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>68.3518</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>68.6372</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>68.9237</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$F$106</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CIMB</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7030A0"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$107:$A$130</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$F$107:$F$130</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>19.1844</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>19.2212</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>19.2581</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>19.2951</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>19.3321</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>19.3692</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>19.4063</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>19.4436</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>19.4809</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>19.5182</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>19.5557</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>19.5932</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>19.6308</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>19.6684</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>19.7062</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>19.744</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19.7819</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19.8198</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>19.8578</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>19.8959</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>19.9341</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>19.9723</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>20.0107</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$G$106</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>GoTyme</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="843C0C"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$107:$A$130</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$G$107:$G$130</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>30.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30.075</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30.1502</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>30.2256</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>30.3011</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30.3769</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>30.4528</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>30.529</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>30.6053</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>30.6818</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>30.7585</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>30.8354</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>30.9125</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>30.9898</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>31.0672</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>31.1449</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>31.2228</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>31.3008</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>31.3791</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>31.4575</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>31.5362</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>31.615</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>31.694</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$H$106</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Maribank</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="5B9BD5"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$107:$A$130</c:f>
+              <c:strCache>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>Jan 2026</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb 2026</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar 2026</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr 2026</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May 2026</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun 2026</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul 2026</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug 2026</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep 2026</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct 2026</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov 2026</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec 2026</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Jan 2027</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Feb 2027</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Mar 2027</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Apr 2027</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>May 2027</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>Jun 2027</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>Jul 2027</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>Aug 2027</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>Sep 2027</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>Oct 2027</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>Nov 2027</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>Dec 2027</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$H$107:$H$130</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>21.6951</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>21.7539</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>21.8129</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>21.872</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>21.9314</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>21.9908</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>22.0505</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>22.1103</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>22.1702</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>22.2304</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>22.2906</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>22.3511</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>22.4117</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>22.4725</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>22.5334</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>22.5945</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>22.6558</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>22.7172</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>22.7789</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>22.8406</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22.9026</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>22.9647</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>23.027</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="100"/>
         <c:axId val="333"/>
         <c:axId val="444"/>
       </c:barChart>
@@ -2053,7 +3141,7 @@
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="b"/>
+      <c:legendPos val="r"/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -2474,7 +3562,7 @@
         </is>
       </c>
       <c r="B17" s="29">
-        <f>SUMIF(Balance!$B$6:$B$19,A17,Balance!$F$6:$F$19)</f>
+        <f>SUMIF(Balance!$A$6:$A$19,A17,Balance!$F$6:$F$19)</f>
         <v>273000.0</v>
       </c>
     </row>
@@ -2485,7 +3573,7 @@
         </is>
       </c>
       <c r="B18" s="29">
-        <f>SUMIF(Balance!$B$6:$B$19,A18,Balance!$F$6:$F$19)</f>
+        <f>SUMIF(Balance!$A$6:$A$19,A18,Balance!$F$6:$F$19)</f>
         <v>125000.0</v>
       </c>
     </row>
@@ -2496,7 +3584,7 @@
         </is>
       </c>
       <c r="B19" s="29">
-        <f>SUMIF(Balance!$B$6:$B$19,A19,Balance!$F$6:$F$19)</f>
+        <f>SUMIF(Balance!$A$6:$A$19,A19,Balance!$F$6:$F$19)</f>
         <v>50000.0</v>
       </c>
     </row>
@@ -2507,7 +3595,7 @@
         </is>
       </c>
       <c r="B20" s="29">
-        <f>SUMIF(Balance!$B$6:$B$19,A20,Balance!$F$6:$F$19)</f>
+        <f>SUMIF(Balance!$A$6:$A$19,A20,Balance!$F$6:$F$19)</f>
         <v>15062.5</v>
       </c>
     </row>
@@ -2518,7 +3606,7 @@
         </is>
       </c>
       <c r="B21" s="29">
-        <f>SUMIF(Balance!$B$6:$B$19,A21,Balance!$F$6:$F$19)</f>
+        <f>SUMIF(Balance!$A$6:$A$19,A21,Balance!$F$6:$F$19)</f>
         <v>10000.0</v>
       </c>
     </row>
@@ -2529,7 +3617,7 @@
         </is>
       </c>
       <c r="B22" s="29">
-        <f>SUMIF(Balance!$B$6:$B$19,A22,Balance!$F$6:$F$19)</f>
+        <f>SUMIF(Balance!$A$6:$A$19,A22,Balance!$F$6:$F$19)</f>
         <v>12000.0</v>
       </c>
     </row>
@@ -2540,7 +3628,7 @@
         </is>
       </c>
       <c r="B23" s="29">
-        <f>SUMIF(Balance!$B$6:$B$19,A23,Balance!$F$6:$F$19)</f>
+        <f>SUMIF(Balance!$A$6:$A$19,A23,Balance!$F$6:$F$19)</f>
         <v>8000.0</v>
       </c>
     </row>
@@ -2577,7 +3665,7 @@
     <row r="51" ht="22" customHeight="1">
       <c r="A51" t="inlineStr" s="24">
         <is>
-          <t xml:space="preserve">📊 Monthly Interest Earned</t>
+          <t xml:space="preserve">📊 Monthly Interest Earned by Bank</t>
         </is>
       </c>
       <c r="B51" s="24"/>
@@ -3594,8 +4682,902 @@
         <v>2810.35</v>
       </c>
     </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" t="inlineStr" s="24">
+        <is>
+          <t xml:space="preserve">🗂 Monthly Interest Earned by Bank (auto)</t>
+        </is>
+      </c>
+      <c r="B105" s="24"/>
+      <c r="C105" s="24"/>
+      <c r="D105" s="24"/>
+      <c r="E105" s="24"/>
+      <c r="F105" s="24"/>
+      <c r="G105" s="24"/>
+      <c r="H105" s="24"/>
+      <c r="I105" s="24"/>
+      <c r="J105" s="24"/>
+      <c r="K105" s="24"/>
+      <c r="L105" s="24"/>
+      <c r="M105" s="24"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Month</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Banko</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">CIMB</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">GoTyme</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr" s="22">
+        <is>
+          <t xml:space="preserve">Maribank</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jan 2026</t>
+        </is>
+      </c>
+      <c r="B107" s="8">
+        <v>0</v>
+      </c>
+      <c r="C107" s="8">
+        <v>0</v>
+      </c>
+      <c r="D107" s="8">
+        <v>0</v>
+      </c>
+      <c r="E107" s="8">
+        <v>0</v>
+      </c>
+      <c r="F107" s="8">
+        <v>0</v>
+      </c>
+      <c r="G107" s="8">
+        <v>0</v>
+      </c>
+      <c r="H107" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Feb 2026</t>
+        </is>
+      </c>
+      <c r="B108" s="8">
+        <f>B81-B80</f>
+        <v>1518.28</v>
+      </c>
+      <c r="C108" s="8">
+        <f>C81-C80</f>
+        <v>573.02</v>
+      </c>
+      <c r="D108" s="8">
+        <f>D81-D80</f>
+        <v>266.67</v>
+      </c>
+      <c r="E108" s="8">
+        <f>E81-E80</f>
+        <v>62.89</v>
+      </c>
+      <c r="F108" s="8">
+        <f>F81-F80</f>
+        <v>19.18</v>
+      </c>
+      <c r="G108" s="8">
+        <f>G81-G80</f>
+        <v>30.0</v>
+      </c>
+      <c r="H108" s="8">
+        <f>H81-H80</f>
+        <v>21.7</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Mar 2026</t>
+        </is>
+      </c>
+      <c r="B109" s="8">
+        <f>B82-B81</f>
+        <v>1527.19</v>
+      </c>
+      <c r="C109" s="8">
+        <f>C82-C81</f>
+        <v>575.73</v>
+      </c>
+      <c r="D109" s="8">
+        <f>D82-D81</f>
+        <v>268.22</v>
+      </c>
+      <c r="E109" s="8">
+        <f>E82-E81</f>
+        <v>63.15</v>
+      </c>
+      <c r="F109" s="8">
+        <f>F82-F81</f>
+        <v>19.22</v>
+      </c>
+      <c r="G109" s="8">
+        <f>G82-G81</f>
+        <v>30.07</v>
+      </c>
+      <c r="H109" s="8">
+        <f>H82-H81</f>
+        <v>21.75</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Apr 2026</t>
+        </is>
+      </c>
+      <c r="B110" s="8">
+        <f>B83-B82</f>
+        <v>1536.15</v>
+      </c>
+      <c r="C110" s="8">
+        <f>C83-C82</f>
+        <v>578.46</v>
+      </c>
+      <c r="D110" s="8">
+        <f>D83-D82</f>
+        <v>269.79</v>
+      </c>
+      <c r="E110" s="8">
+        <f>E83-E82</f>
+        <v>63.41</v>
+      </c>
+      <c r="F110" s="8">
+        <f>F83-F82</f>
+        <v>19.26</v>
+      </c>
+      <c r="G110" s="8">
+        <f>G83-G82</f>
+        <v>30.15</v>
+      </c>
+      <c r="H110" s="8">
+        <f>H83-H82</f>
+        <v>21.81</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">May 2026</t>
+        </is>
+      </c>
+      <c r="B111" s="8">
+        <f>B84-B83</f>
+        <v>1545.16</v>
+      </c>
+      <c r="C111" s="8">
+        <f>C84-C83</f>
+        <v>581.2</v>
+      </c>
+      <c r="D111" s="8">
+        <f>D84-D83</f>
+        <v>271.36</v>
+      </c>
+      <c r="E111" s="8">
+        <f>E84-E83</f>
+        <v>63.68</v>
+      </c>
+      <c r="F111" s="8">
+        <f>F84-F83</f>
+        <v>19.3</v>
+      </c>
+      <c r="G111" s="8">
+        <f>G84-G83</f>
+        <v>30.23</v>
+      </c>
+      <c r="H111" s="8">
+        <f>H84-H83</f>
+        <v>21.87</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jun 2026</t>
+        </is>
+      </c>
+      <c r="B112" s="8">
+        <f>B85-B84</f>
+        <v>1554.24</v>
+      </c>
+      <c r="C112" s="8">
+        <f>C85-C84</f>
+        <v>583.95</v>
+      </c>
+      <c r="D112" s="8">
+        <f>D85-D84</f>
+        <v>272.95</v>
+      </c>
+      <c r="E112" s="8">
+        <f>E85-E84</f>
+        <v>63.94</v>
+      </c>
+      <c r="F112" s="8">
+        <f>F85-F84</f>
+        <v>19.33</v>
+      </c>
+      <c r="G112" s="8">
+        <f>G85-G84</f>
+        <v>30.3</v>
+      </c>
+      <c r="H112" s="8">
+        <f>H85-H84</f>
+        <v>21.93</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jul 2026</t>
+        </is>
+      </c>
+      <c r="B113" s="8">
+        <f>B86-B85</f>
+        <v>1563.37</v>
+      </c>
+      <c r="C113" s="8">
+        <f>C86-C85</f>
+        <v>586.72</v>
+      </c>
+      <c r="D113" s="8">
+        <f>D86-D85</f>
+        <v>274.54</v>
+      </c>
+      <c r="E113" s="8">
+        <f>E86-E85</f>
+        <v>64.21</v>
+      </c>
+      <c r="F113" s="8">
+        <f>F86-F85</f>
+        <v>19.37</v>
+      </c>
+      <c r="G113" s="8">
+        <f>G86-G85</f>
+        <v>30.38</v>
+      </c>
+      <c r="H113" s="8">
+        <f>H86-H85</f>
+        <v>21.99</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Aug 2026</t>
+        </is>
+      </c>
+      <c r="B114" s="8">
+        <f>B87-B86</f>
+        <v>1572.55</v>
+      </c>
+      <c r="C114" s="8">
+        <f>C87-C86</f>
+        <v>589.5</v>
+      </c>
+      <c r="D114" s="8">
+        <f>D87-D86</f>
+        <v>276.15</v>
+      </c>
+      <c r="E114" s="8">
+        <f>E87-E86</f>
+        <v>64.48</v>
+      </c>
+      <c r="F114" s="8">
+        <f>F87-F86</f>
+        <v>19.41</v>
+      </c>
+      <c r="G114" s="8">
+        <f>G87-G86</f>
+        <v>30.45</v>
+      </c>
+      <c r="H114" s="8">
+        <f>H87-H86</f>
+        <v>22.05</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Sep 2026</t>
+        </is>
+      </c>
+      <c r="B115" s="8">
+        <f>B88-B87</f>
+        <v>1581.8</v>
+      </c>
+      <c r="C115" s="8">
+        <f>C88-C87</f>
+        <v>592.29</v>
+      </c>
+      <c r="D115" s="8">
+        <f>D88-D87</f>
+        <v>277.76</v>
+      </c>
+      <c r="E115" s="8">
+        <f>E88-E87</f>
+        <v>64.75</v>
+      </c>
+      <c r="F115" s="8">
+        <f>F88-F87</f>
+        <v>19.44</v>
+      </c>
+      <c r="G115" s="8">
+        <f>G88-G87</f>
+        <v>30.53</v>
+      </c>
+      <c r="H115" s="8">
+        <f>H88-H87</f>
+        <v>22.11</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Oct 2026</t>
+        </is>
+      </c>
+      <c r="B116" s="8">
+        <f>B89-B88</f>
+        <v>1591.1</v>
+      </c>
+      <c r="C116" s="8">
+        <f>C89-C88</f>
+        <v>595.1</v>
+      </c>
+      <c r="D116" s="8">
+        <f>D89-D88</f>
+        <v>279.38</v>
+      </c>
+      <c r="E116" s="8">
+        <f>E89-E88</f>
+        <v>65.02</v>
+      </c>
+      <c r="F116" s="8">
+        <f>F89-F88</f>
+        <v>19.48</v>
+      </c>
+      <c r="G116" s="8">
+        <f>G89-G88</f>
+        <v>30.61</v>
+      </c>
+      <c r="H116" s="8">
+        <f>H89-H88</f>
+        <v>22.17</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Nov 2026</t>
+        </is>
+      </c>
+      <c r="B117" s="8">
+        <f>B90-B89</f>
+        <v>1600.46</v>
+      </c>
+      <c r="C117" s="8">
+        <f>C90-C89</f>
+        <v>597.92</v>
+      </c>
+      <c r="D117" s="8">
+        <f>D90-D89</f>
+        <v>281.02</v>
+      </c>
+      <c r="E117" s="8">
+        <f>E90-E89</f>
+        <v>65.29</v>
+      </c>
+      <c r="F117" s="8">
+        <f>F90-F89</f>
+        <v>19.52</v>
+      </c>
+      <c r="G117" s="8">
+        <f>G90-G89</f>
+        <v>30.68</v>
+      </c>
+      <c r="H117" s="8">
+        <f>H90-H89</f>
+        <v>22.23</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Dec 2026</t>
+        </is>
+      </c>
+      <c r="B118" s="8">
+        <f>B91-B90</f>
+        <v>1609.88</v>
+      </c>
+      <c r="C118" s="8">
+        <f>C91-C90</f>
+        <v>600.75</v>
+      </c>
+      <c r="D118" s="8">
+        <f>D91-D90</f>
+        <v>282.66</v>
+      </c>
+      <c r="E118" s="8">
+        <f>E91-E90</f>
+        <v>65.56</v>
+      </c>
+      <c r="F118" s="8">
+        <f>F91-F90</f>
+        <v>19.56</v>
+      </c>
+      <c r="G118" s="8">
+        <f>G91-G90</f>
+        <v>30.76</v>
+      </c>
+      <c r="H118" s="8">
+        <f>H91-H90</f>
+        <v>22.29</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jan 2027</t>
+        </is>
+      </c>
+      <c r="B119" s="8">
+        <f>B92-B91</f>
+        <v>1619.36</v>
+      </c>
+      <c r="C119" s="8">
+        <f>C92-C91</f>
+        <v>603.6</v>
+      </c>
+      <c r="D119" s="8">
+        <f>D92-D91</f>
+        <v>284.32</v>
+      </c>
+      <c r="E119" s="8">
+        <f>E92-E91</f>
+        <v>65.84</v>
+      </c>
+      <c r="F119" s="8">
+        <f>F92-F91</f>
+        <v>19.59</v>
+      </c>
+      <c r="G119" s="8">
+        <f>G92-G91</f>
+        <v>30.84</v>
+      </c>
+      <c r="H119" s="8">
+        <f>H92-H91</f>
+        <v>22.35</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Feb 2027</t>
+        </is>
+      </c>
+      <c r="B120" s="8">
+        <f>B93-B92</f>
+        <v>1628.9</v>
+      </c>
+      <c r="C120" s="8">
+        <f>C93-C92</f>
+        <v>606.46</v>
+      </c>
+      <c r="D120" s="8">
+        <f>D93-D92</f>
+        <v>285.98</v>
+      </c>
+      <c r="E120" s="8">
+        <f>E93-E92</f>
+        <v>66.11</v>
+      </c>
+      <c r="F120" s="8">
+        <f>F93-F92</f>
+        <v>19.63</v>
+      </c>
+      <c r="G120" s="8">
+        <f>G93-G92</f>
+        <v>30.91</v>
+      </c>
+      <c r="H120" s="8">
+        <f>H93-H92</f>
+        <v>22.41</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Mar 2027</t>
+        </is>
+      </c>
+      <c r="B121" s="8">
+        <f>B94-B93</f>
+        <v>1638.49</v>
+      </c>
+      <c r="C121" s="8">
+        <f>C94-C93</f>
+        <v>609.33</v>
+      </c>
+      <c r="D121" s="8">
+        <f>D94-D93</f>
+        <v>287.66</v>
+      </c>
+      <c r="E121" s="8">
+        <f>E94-E93</f>
+        <v>66.39</v>
+      </c>
+      <c r="F121" s="8">
+        <f>F94-F93</f>
+        <v>19.67</v>
+      </c>
+      <c r="G121" s="8">
+        <f>G94-G93</f>
+        <v>30.99</v>
+      </c>
+      <c r="H121" s="8">
+        <f>H94-H93</f>
+        <v>22.47</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Apr 2027</t>
+        </is>
+      </c>
+      <c r="B122" s="8">
+        <f>B95-B94</f>
+        <v>1648.15</v>
+      </c>
+      <c r="C122" s="8">
+        <f>C95-C94</f>
+        <v>612.22</v>
+      </c>
+      <c r="D122" s="8">
+        <f>D95-D94</f>
+        <v>289.34</v>
+      </c>
+      <c r="E122" s="8">
+        <f>E95-E94</f>
+        <v>66.66</v>
+      </c>
+      <c r="F122" s="8">
+        <f>F95-F94</f>
+        <v>19.71</v>
+      </c>
+      <c r="G122" s="8">
+        <f>G95-G94</f>
+        <v>31.07</v>
+      </c>
+      <c r="H122" s="8">
+        <f>H95-H94</f>
+        <v>22.53</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">May 2027</t>
+        </is>
+      </c>
+      <c r="B123" s="8">
+        <f>B96-B95</f>
+        <v>1657.87</v>
+      </c>
+      <c r="C123" s="8">
+        <f>C96-C95</f>
+        <v>615.13</v>
+      </c>
+      <c r="D123" s="8">
+        <f>D96-D95</f>
+        <v>291.04</v>
+      </c>
+      <c r="E123" s="8">
+        <f>E96-E95</f>
+        <v>66.94</v>
+      </c>
+      <c r="F123" s="8">
+        <f>F96-F95</f>
+        <v>19.74</v>
+      </c>
+      <c r="G123" s="8">
+        <f>G96-G95</f>
+        <v>31.14</v>
+      </c>
+      <c r="H123" s="8">
+        <f>H96-H95</f>
+        <v>22.59</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jun 2027</t>
+        </is>
+      </c>
+      <c r="B124" s="8">
+        <f>B97-B96</f>
+        <v>1667.65</v>
+      </c>
+      <c r="C124" s="8">
+        <f>C97-C96</f>
+        <v>618.04</v>
+      </c>
+      <c r="D124" s="8">
+        <f>D97-D96</f>
+        <v>292.75</v>
+      </c>
+      <c r="E124" s="8">
+        <f>E97-E96</f>
+        <v>67.22</v>
+      </c>
+      <c r="F124" s="8">
+        <f>F97-F96</f>
+        <v>19.78</v>
+      </c>
+      <c r="G124" s="8">
+        <f>G97-G96</f>
+        <v>31.22</v>
+      </c>
+      <c r="H124" s="8">
+        <f>H97-H96</f>
+        <v>22.66</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Jul 2027</t>
+        </is>
+      </c>
+      <c r="B125" s="8">
+        <f>B98-B97</f>
+        <v>1677.49</v>
+      </c>
+      <c r="C125" s="8">
+        <f>C98-C97</f>
+        <v>620.97</v>
+      </c>
+      <c r="D125" s="8">
+        <f>D98-D97</f>
+        <v>294.46</v>
+      </c>
+      <c r="E125" s="8">
+        <f>E98-E97</f>
+        <v>67.5</v>
+      </c>
+      <c r="F125" s="8">
+        <f>F98-F97</f>
+        <v>19.82</v>
+      </c>
+      <c r="G125" s="8">
+        <f>G98-G97</f>
+        <v>31.3</v>
+      </c>
+      <c r="H125" s="8">
+        <f>H98-H97</f>
+        <v>22.72</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Aug 2027</t>
+        </is>
+      </c>
+      <c r="B126" s="8">
+        <f>B99-B98</f>
+        <v>1687.4</v>
+      </c>
+      <c r="C126" s="8">
+        <f>C99-C98</f>
+        <v>623.92</v>
+      </c>
+      <c r="D126" s="8">
+        <f>D99-D98</f>
+        <v>296.19</v>
+      </c>
+      <c r="E126" s="8">
+        <f>E99-E98</f>
+        <v>67.78</v>
+      </c>
+      <c r="F126" s="8">
+        <f>F99-F98</f>
+        <v>19.86</v>
+      </c>
+      <c r="G126" s="8">
+        <f>G99-G98</f>
+        <v>31.38</v>
+      </c>
+      <c r="H126" s="8">
+        <f>H99-H98</f>
+        <v>22.78</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Sep 2027</t>
+        </is>
+      </c>
+      <c r="B127" s="8">
+        <f>B100-B99</f>
+        <v>1697.36</v>
+      </c>
+      <c r="C127" s="8">
+        <f>C100-C99</f>
+        <v>626.88</v>
+      </c>
+      <c r="D127" s="8">
+        <f>D100-D99</f>
+        <v>297.93</v>
+      </c>
+      <c r="E127" s="8">
+        <f>E100-E99</f>
+        <v>68.07</v>
+      </c>
+      <c r="F127" s="8">
+        <f>F100-F99</f>
+        <v>19.9</v>
+      </c>
+      <c r="G127" s="8">
+        <f>G100-G99</f>
+        <v>31.46</v>
+      </c>
+      <c r="H127" s="8">
+        <f>H100-H99</f>
+        <v>22.84</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Oct 2027</t>
+        </is>
+      </c>
+      <c r="B128" s="8">
+        <f>B101-B100</f>
+        <v>1707.39</v>
+      </c>
+      <c r="C128" s="8">
+        <f>C101-C100</f>
+        <v>629.85</v>
+      </c>
+      <c r="D128" s="8">
+        <f>D101-D100</f>
+        <v>299.68</v>
+      </c>
+      <c r="E128" s="8">
+        <f>E101-E100</f>
+        <v>68.35</v>
+      </c>
+      <c r="F128" s="8">
+        <f>F101-F100</f>
+        <v>19.93</v>
+      </c>
+      <c r="G128" s="8">
+        <f>G101-G100</f>
+        <v>31.54</v>
+      </c>
+      <c r="H128" s="8">
+        <f>H101-H100</f>
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Nov 2027</t>
+        </is>
+      </c>
+      <c r="B129" s="8">
+        <f>B102-B101</f>
+        <v>1717.48</v>
+      </c>
+      <c r="C129" s="8">
+        <f>C102-C101</f>
+        <v>632.84</v>
+      </c>
+      <c r="D129" s="8">
+        <f>D102-D101</f>
+        <v>301.44</v>
+      </c>
+      <c r="E129" s="8">
+        <f>E102-E101</f>
+        <v>68.64</v>
+      </c>
+      <c r="F129" s="8">
+        <f>F102-F101</f>
+        <v>19.97</v>
+      </c>
+      <c r="G129" s="8">
+        <f>G102-G101</f>
+        <v>31.62</v>
+      </c>
+      <c r="H129" s="8">
+        <f>H102-H101</f>
+        <v>22.96</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Dec 2027</t>
+        </is>
+      </c>
+      <c r="B130" s="8">
+        <f>B103-B102</f>
+        <v>1727.64</v>
+      </c>
+      <c r="C130" s="8">
+        <f>C103-C102</f>
+        <v>635.84</v>
+      </c>
+      <c r="D130" s="8">
+        <f>D103-D102</f>
+        <v>303.21</v>
+      </c>
+      <c r="E130" s="8">
+        <f>E103-E102</f>
+        <v>68.92</v>
+      </c>
+      <c r="F130" s="8">
+        <f>F103-F102</f>
+        <v>20.01</v>
+      </c>
+      <c r="G130" s="8">
+        <f>G103-G102</f>
+        <v>31.69</v>
+      </c>
+      <c r="H130" s="8">
+        <f>H103-H102</f>
+        <v>23.03</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
@@ -3623,6 +5605,7 @@
     <mergeCell ref="A27:M27"/>
     <mergeCell ref="A51:M51"/>
     <mergeCell ref="A77:M77"/>
+    <mergeCell ref="A105:M105"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2:B2" location="Dashboard!A1" display="🏠 Dashboard"/>

</xml_diff>

<commit_message>
Add automatic interest accrual: balances grow on their own via TODAY()
- Interest sheet: new columns Interest Start (earliest deposit), Periods Elapsed
  (days/months to TODAY), Interest to Date, and Balance Today (compounds live)
- Balance sheet: adds Interest to Date + Balance Today columns
- Dashboard: Total Balance Today, Interest Earned to Date, pie & goal use Balance Today
- Removed manual Interest seed transaction (auto-accrual replaces it to avoid double-count)
- Updated formula reference .docx accordingly
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -960,76 +960,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>15062.5</c:v>
+                  <c:v>15000.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15125.387</c:v>
+                  <c:v>15062.6261</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15188.5366</c:v>
+                  <c:v>15125.5137</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15251.9499</c:v>
+                  <c:v>15188.6638</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15315.6279</c:v>
+                  <c:v>15252.0775</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>15379.5717</c:v>
+                  <c:v>15315.7561</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>15443.7826</c:v>
+                  <c:v>15379.7005</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>15508.2615</c:v>
+                  <c:v>15443.9118</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>15573.0096</c:v>
+                  <c:v>15508.3913</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>15638.028</c:v>
+                  <c:v>15573.14</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>15703.3179</c:v>
+                  <c:v>15638.159</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>15768.8804</c:v>
+                  <c:v>15703.4494</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>15834.7167</c:v>
+                  <c:v>15769.0124</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>15900.8278</c:v>
+                  <c:v>15834.8492</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>15967.2149</c:v>
+                  <c:v>15900.9609</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>16033.8792</c:v>
+                  <c:v>15967.3485</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>16100.8218</c:v>
+                  <c:v>16034.0134</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>16168.0439</c:v>
+                  <c:v>16100.9566</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>16235.5466</c:v>
+                  <c:v>16168.1792</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>16303.3312</c:v>
+                  <c:v>16235.6825</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>16371.3988</c:v>
+                  <c:v>16303.4677</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>16439.7506</c:v>
+                  <c:v>16371.5359</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>16508.3877</c:v>
+                  <c:v>16439.8882</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>16577.3115</c:v>
+                  <c:v>16508.5259</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1741,25 +1741,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>273000.0</c:v>
+                  <c:v>274565.82</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>125000.0</c:v>
+                  <c:v>125581.64</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>50000.0</c:v>
+                  <c:v>50266.67</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15062.5</c:v>
+                  <c:v>15070.02</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000.0</c:v>
+                  <c:v>10021.45</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>12000.0</c:v>
+                  <c:v>12030.0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8000.0</c:v>
+                  <c:v>8024.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2474,73 +2474,73 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>62.887</c:v>
+                  <c:v>62.6261</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>63.1496</c:v>
+                  <c:v>62.8876</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>63.4132</c:v>
+                  <c:v>63.1501</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>63.678</c:v>
+                  <c:v>63.4138</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>63.9439</c:v>
+                  <c:v>63.6785</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>64.2108</c:v>
+                  <c:v>63.9444</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>64.4789</c:v>
+                  <c:v>64.2114</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>64.7481</c:v>
+                  <c:v>64.4795</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>65.0184</c:v>
+                  <c:v>64.7487</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>65.2899</c:v>
+                  <c:v>65.019</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>65.5625</c:v>
+                  <c:v>65.2905</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>65.8362</c:v>
+                  <c:v>65.563</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>66.1111</c:v>
+                  <c:v>65.8368</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>66.3871</c:v>
+                  <c:v>66.1116</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>66.6643</c:v>
+                  <c:v>66.3877</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>66.9426</c:v>
+                  <c:v>66.6648</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>67.2221</c:v>
+                  <c:v>66.9432</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>67.5028</c:v>
+                  <c:v>67.2227</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>67.7846</c:v>
+                  <c:v>67.5033</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>68.0676</c:v>
+                  <c:v>67.7852</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>68.3518</c:v>
+                  <c:v>68.0682</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>68.6372</c:v>
+                  <c:v>68.3524</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>68.9237</c:v>
+                  <c:v>68.6377</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3388,15 +3388,15 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" t="inlineStr" s="25">
         <is>
-          <t xml:space="preserve">Total Balance (All Accounts)</t>
+          <t xml:space="preserve">Total Balance Today (incl. interest)</t>
         </is>
       </c>
       <c r="B5" s="25"/>
       <c r="C5" s="25"/>
       <c r="D5" s="25"/>
       <c r="E5" s="26">
-        <f>SUM(Balance!$F$6:$F$19)</f>
-        <v>493062.5</v>
+        <f>SUM(Balance!$H$6:$H$19)</f>
+        <v>495559.84</v>
       </c>
       <c r="F5" s="26"/>
       <c r="G5" s="26"/>
@@ -3422,15 +3422,15 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" t="inlineStr" s="25">
         <is>
-          <t xml:space="preserve">Total Interest Credited</t>
+          <t xml:space="preserve">Interest Earned to Date (auto)</t>
         </is>
       </c>
       <c r="B7" s="25"/>
       <c r="C7" s="25"/>
       <c r="D7" s="25"/>
       <c r="E7" s="26">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$B$6:$B$205,"Interest")</f>
-        <v>62.5</v>
+        <f>SUM(Balance!$G$6:$G$19)</f>
+        <v>2559.84</v>
       </c>
       <c r="F7" s="26"/>
       <c r="G7" s="26"/>
@@ -3492,15 +3492,15 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" t="inlineStr" s="25">
         <is>
-          <t xml:space="preserve">Maya Personal Goal — Current Balance</t>
+          <t xml:space="preserve">Maya Personal Goal — Balance Today</t>
         </is>
       </c>
       <c r="B12" s="25"/>
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
       <c r="E12" s="26">
-        <f>IFERROR(VLOOKUP("Maya - Personal Goal",Balance!$C$6:$F$19,4,FALSE),0)</f>
-        <v>25000.0</v>
+        <f>IFERROR(VLOOKUP("Maya - Personal Goal",Balance!$C$6:$H$19,6,FALSE),0)</f>
+        <v>25116.67</v>
       </c>
       <c r="F12" s="26"/>
       <c r="G12" s="26"/>
@@ -3517,7 +3517,7 @@
       <c r="D13" s="25"/>
       <c r="E13" s="27">
         <f>IFERROR(E12/E11,0)</f>
-        <v>0.25</v>
+        <v>0.2512</v>
       </c>
       <c r="F13" s="27"/>
       <c r="G13" s="27"/>
@@ -3562,8 +3562,8 @@
         </is>
       </c>
       <c r="B17" s="29">
-        <f>SUMIF(Balance!$A$6:$A$19,A17,Balance!$F$6:$F$19)</f>
-        <v>273000.0</v>
+        <f>SUMIF(Balance!$A$6:$A$19,A17,Balance!$H$6:$H$19)</f>
+        <v>274565.82</v>
       </c>
     </row>
     <row r="18">
@@ -3573,8 +3573,8 @@
         </is>
       </c>
       <c r="B18" s="29">
-        <f>SUMIF(Balance!$A$6:$A$19,A18,Balance!$F$6:$F$19)</f>
-        <v>125000.0</v>
+        <f>SUMIF(Balance!$A$6:$A$19,A18,Balance!$H$6:$H$19)</f>
+        <v>125581.64</v>
       </c>
     </row>
     <row r="19">
@@ -3584,8 +3584,8 @@
         </is>
       </c>
       <c r="B19" s="29">
-        <f>SUMIF(Balance!$A$6:$A$19,A19,Balance!$F$6:$F$19)</f>
-        <v>50000.0</v>
+        <f>SUMIF(Balance!$A$6:$A$19,A19,Balance!$H$6:$H$19)</f>
+        <v>50266.67</v>
       </c>
     </row>
     <row r="20">
@@ -3595,8 +3595,8 @@
         </is>
       </c>
       <c r="B20" s="29">
-        <f>SUMIF(Balance!$A$6:$A$19,A20,Balance!$F$6:$F$19)</f>
-        <v>15062.5</v>
+        <f>SUMIF(Balance!$A$6:$A$19,A20,Balance!$H$6:$H$19)</f>
+        <v>15070.02</v>
       </c>
     </row>
     <row r="21">
@@ -3606,8 +3606,8 @@
         </is>
       </c>
       <c r="B21" s="29">
-        <f>SUMIF(Balance!$A$6:$A$19,A21,Balance!$F$6:$F$19)</f>
-        <v>10000.0</v>
+        <f>SUMIF(Balance!$A$6:$A$19,A21,Balance!$H$6:$H$19)</f>
+        <v>10021.45</v>
       </c>
     </row>
     <row r="22">
@@ -3617,8 +3617,8 @@
         </is>
       </c>
       <c r="B22" s="29">
-        <f>SUMIF(Balance!$A$6:$A$19,A22,Balance!$F$6:$F$19)</f>
-        <v>12000.0</v>
+        <f>SUMIF(Balance!$A$6:$A$19,A22,Balance!$H$6:$H$19)</f>
+        <v>12030.0</v>
       </c>
     </row>
     <row r="23">
@@ -3628,8 +3628,8 @@
         </is>
       </c>
       <c r="B23" s="29">
-        <f>SUMIF(Balance!$A$6:$A$19,A23,Balance!$F$6:$F$19)</f>
-        <v>8000.0</v>
+        <f>SUMIF(Balance!$A$6:$A$19,A23,Balance!$H$6:$H$19)</f>
+        <v>8024.25</v>
       </c>
     </row>
     <row r="24">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="B24" s="16">
         <f>SUM(B17:B23)</f>
-        <v>493062.5</v>
+        <v>495559.84</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="E80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
-        <v>15062.5</v>
+        <v>15000.0</v>
       </c>
       <c r="F80" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^0)</f>
@@ -3805,7 +3805,7 @@
       </c>
       <c r="E81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
-        <v>15125.39</v>
+        <v>15062.63</v>
       </c>
       <c r="F81" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^1)</f>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="I81" s="8">
         <f>SUM(B81:H81)-SUM(B80:H80)</f>
-        <v>2491.74</v>
+        <v>2491.47</v>
       </c>
     </row>
     <row r="82">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="E82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
-        <v>15188.54</v>
+        <v>15125.51</v>
       </c>
       <c r="F82" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^2)</f>
@@ -3860,7 +3860,7 @@
       </c>
       <c r="I82" s="8">
         <f>SUM(B82:H82)-SUM(B81:H81)</f>
-        <v>2505.34</v>
+        <v>2505.08</v>
       </c>
     </row>
     <row r="83">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="E83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
-        <v>15251.95</v>
+        <v>15188.66</v>
       </c>
       <c r="F83" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^3)</f>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="I83" s="8">
         <f>SUM(B83:H83)-SUM(B82:H82)</f>
-        <v>2519.03</v>
+        <v>2518.77</v>
       </c>
     </row>
     <row r="84">
@@ -3922,7 +3922,7 @@
       </c>
       <c r="E84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
-        <v>15315.63</v>
+        <v>15252.08</v>
       </c>
       <c r="F84" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^4)</f>
@@ -3938,7 +3938,7 @@
       </c>
       <c r="I84" s="8">
         <f>SUM(B84:H84)-SUM(B83:H83)</f>
-        <v>2532.8</v>
+        <v>2532.53</v>
       </c>
     </row>
     <row r="85">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="E85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
-        <v>15379.57</v>
+        <v>15315.76</v>
       </c>
       <c r="F85" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^5)</f>
@@ -3977,7 +3977,7 @@
       </c>
       <c r="I85" s="8">
         <f>SUM(B85:H85)-SUM(B84:H84)</f>
-        <v>2546.64</v>
+        <v>2546.38</v>
       </c>
     </row>
     <row r="86">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="E86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
-        <v>15443.78</v>
+        <v>15379.7</v>
       </c>
       <c r="F86" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^6)</f>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="I86" s="8">
         <f>SUM(B86:H86)-SUM(B85:H85)</f>
-        <v>2560.57</v>
+        <v>2560.31</v>
       </c>
     </row>
     <row r="87">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="E87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
-        <v>15508.26</v>
+        <v>15443.91</v>
       </c>
       <c r="F87" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^7)</f>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="I87" s="8">
         <f>SUM(B87:H87)-SUM(B86:H86)</f>
-        <v>2574.59</v>
+        <v>2574.32</v>
       </c>
     </row>
     <row r="88">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="E88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
-        <v>15573.01</v>
+        <v>15508.39</v>
       </c>
       <c r="F88" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^8)</f>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="I88" s="8">
         <f>SUM(B88:H88)-SUM(B87:H87)</f>
-        <v>2588.68</v>
+        <v>2588.41</v>
       </c>
     </row>
     <row r="89">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="E89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
-        <v>15638.03</v>
+        <v>15573.14</v>
       </c>
       <c r="F89" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^9)</f>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="I89" s="8">
         <f>SUM(B89:H89)-SUM(B88:H88)</f>
-        <v>2602.86</v>
+        <v>2602.59</v>
       </c>
     </row>
     <row r="90">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="E90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
-        <v>15703.32</v>
+        <v>15638.16</v>
       </c>
       <c r="F90" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^10)</f>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="I90" s="8">
         <f>SUM(B90:H90)-SUM(B89:H89)</f>
-        <v>2617.12</v>
+        <v>2616.85</v>
       </c>
     </row>
     <row r="91">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="E91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
-        <v>15768.88</v>
+        <v>15703.45</v>
       </c>
       <c r="F91" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^11)</f>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="I91" s="8">
         <f>SUM(B91:H91)-SUM(B90:H90)</f>
-        <v>2631.46</v>
+        <v>2631.19</v>
       </c>
     </row>
     <row r="92">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="E92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
-        <v>15834.72</v>
+        <v>15769.01</v>
       </c>
       <c r="F92" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^12)</f>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="I92" s="8">
         <f>SUM(B92:H92)-SUM(B91:H91)</f>
-        <v>2645.89</v>
+        <v>2645.62</v>
       </c>
     </row>
     <row r="93">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="E93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
-        <v>15900.83</v>
+        <v>15834.85</v>
       </c>
       <c r="F93" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^13)</f>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="I93" s="8">
         <f>SUM(B93:H93)-SUM(B92:H92)</f>
-        <v>2660.4</v>
+        <v>2660.13</v>
       </c>
     </row>
     <row r="94">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="E94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
-        <v>15967.21</v>
+        <v>15900.96</v>
       </c>
       <c r="F94" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^14)</f>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="I94" s="8">
         <f>SUM(B94:H94)-SUM(B93:H93)</f>
-        <v>2675.0</v>
+        <v>2674.73</v>
       </c>
     </row>
     <row r="95">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="E95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
-        <v>16033.88</v>
+        <v>15967.35</v>
       </c>
       <c r="F95" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^15)</f>
@@ -4367,7 +4367,7 @@
       </c>
       <c r="I95" s="8">
         <f>SUM(B95:H95)-SUM(B94:H94)</f>
-        <v>2689.69</v>
+        <v>2689.41</v>
       </c>
     </row>
     <row r="96">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="E96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
-        <v>16100.82</v>
+        <v>16034.01</v>
       </c>
       <c r="F96" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^16)</f>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="I96" s="8">
         <f>SUM(B96:H96)-SUM(B95:H95)</f>
-        <v>2704.46</v>
+        <v>2704.19</v>
       </c>
     </row>
     <row r="97">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="E97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
-        <v>16168.04</v>
+        <v>16100.96</v>
       </c>
       <c r="F97" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^17)</f>
@@ -4445,7 +4445,7 @@
       </c>
       <c r="I97" s="8">
         <f>SUM(B97:H97)-SUM(B96:H96)</f>
-        <v>2719.32</v>
+        <v>2719.04</v>
       </c>
     </row>
     <row r="98">
@@ -4468,7 +4468,7 @@
       </c>
       <c r="E98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
-        <v>16235.55</v>
+        <v>16168.18</v>
       </c>
       <c r="F98" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^18)</f>
@@ -4484,7 +4484,7 @@
       </c>
       <c r="I98" s="8">
         <f>SUM(B98:H98)-SUM(B97:H97)</f>
-        <v>2734.27</v>
+        <v>2733.99</v>
       </c>
     </row>
     <row r="99">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="E99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
-        <v>16303.33</v>
+        <v>16235.68</v>
       </c>
       <c r="F99" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^19)</f>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="I99" s="8">
         <f>SUM(B99:H99)-SUM(B98:H98)</f>
-        <v>2749.31</v>
+        <v>2749.03</v>
       </c>
     </row>
     <row r="100">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="E100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
-        <v>16371.4</v>
+        <v>16303.47</v>
       </c>
       <c r="F100" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^20)</f>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="I100" s="8">
         <f>SUM(B100:H100)-SUM(B99:H99)</f>
-        <v>2764.43</v>
+        <v>2764.15</v>
       </c>
     </row>
     <row r="101">
@@ -4585,7 +4585,7 @@
       </c>
       <c r="E101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
-        <v>16439.75</v>
+        <v>16371.54</v>
       </c>
       <c r="F101" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^21)</f>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="I101" s="8">
         <f>SUM(B101:H101)-SUM(B100:H100)</f>
-        <v>2779.65</v>
+        <v>2779.36</v>
       </c>
     </row>
     <row r="102">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="E102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
-        <v>16508.39</v>
+        <v>16439.89</v>
       </c>
       <c r="F102" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^22)</f>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="I102" s="8">
         <f>SUM(B102:H102)-SUM(B101:H101)</f>
-        <v>2794.95</v>
+        <v>2794.67</v>
       </c>
     </row>
     <row r="103">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="E103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=E$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
-        <v>16577.31</v>
+        <v>16508.53</v>
       </c>
       <c r="F103" s="8">
         <f>SUMPRODUCT((Interest!$A$6:$A$19=F$79)*Interest!$G$6:$G$19*Interest!$M$6:$M$19^23)</f>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="I103" s="8">
         <f>SUM(B103:H103)-SUM(B102:H102)</f>
-        <v>2810.35</v>
+        <v>2810.06</v>
       </c>
     </row>
     <row r="105" ht="22" customHeight="1">
@@ -4791,7 +4791,7 @@
       </c>
       <c r="E108" s="8">
         <f>E81-E80</f>
-        <v>62.89</v>
+        <v>62.63</v>
       </c>
       <c r="F108" s="8">
         <f>F81-F80</f>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="E109" s="8">
         <f>E82-E81</f>
-        <v>63.15</v>
+        <v>62.89</v>
       </c>
       <c r="F109" s="8">
         <f>F82-F81</f>
@@ -4861,7 +4861,7 @@
       </c>
       <c r="E110" s="8">
         <f>E83-E82</f>
-        <v>63.41</v>
+        <v>63.15</v>
       </c>
       <c r="F110" s="8">
         <f>F83-F82</f>
@@ -4896,7 +4896,7 @@
       </c>
       <c r="E111" s="8">
         <f>E84-E83</f>
-        <v>63.68</v>
+        <v>63.41</v>
       </c>
       <c r="F111" s="8">
         <f>F84-F83</f>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="E112" s="8">
         <f>E85-E84</f>
-        <v>63.94</v>
+        <v>63.68</v>
       </c>
       <c r="F112" s="8">
         <f>F85-F84</f>
@@ -4966,7 +4966,7 @@
       </c>
       <c r="E113" s="8">
         <f>E86-E85</f>
-        <v>64.21</v>
+        <v>63.94</v>
       </c>
       <c r="F113" s="8">
         <f>F86-F85</f>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="E114" s="8">
         <f>E87-E86</f>
-        <v>64.48</v>
+        <v>64.21</v>
       </c>
       <c r="F114" s="8">
         <f>F87-F86</f>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="E115" s="8">
         <f>E88-E87</f>
-        <v>64.75</v>
+        <v>64.48</v>
       </c>
       <c r="F115" s="8">
         <f>F88-F87</f>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="E116" s="8">
         <f>E89-E88</f>
-        <v>65.02</v>
+        <v>64.75</v>
       </c>
       <c r="F116" s="8">
         <f>F89-F88</f>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="E117" s="8">
         <f>E90-E89</f>
-        <v>65.29</v>
+        <v>65.02</v>
       </c>
       <c r="F117" s="8">
         <f>F90-F89</f>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="E118" s="8">
         <f>E91-E90</f>
-        <v>65.56</v>
+        <v>65.29</v>
       </c>
       <c r="F118" s="8">
         <f>F91-F90</f>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="E119" s="8">
         <f>E92-E91</f>
-        <v>65.84</v>
+        <v>65.56</v>
       </c>
       <c r="F119" s="8">
         <f>F92-F91</f>
@@ -5211,7 +5211,7 @@
       </c>
       <c r="E120" s="8">
         <f>E93-E92</f>
-        <v>66.11</v>
+        <v>65.84</v>
       </c>
       <c r="F120" s="8">
         <f>F93-F92</f>
@@ -5246,7 +5246,7 @@
       </c>
       <c r="E121" s="8">
         <f>E94-E93</f>
-        <v>66.39</v>
+        <v>66.11</v>
       </c>
       <c r="F121" s="8">
         <f>F94-F93</f>
@@ -5281,7 +5281,7 @@
       </c>
       <c r="E122" s="8">
         <f>E95-E94</f>
-        <v>66.66</v>
+        <v>66.39</v>
       </c>
       <c r="F122" s="8">
         <f>F95-F94</f>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="E123" s="8">
         <f>E96-E95</f>
-        <v>66.94</v>
+        <v>66.66</v>
       </c>
       <c r="F123" s="8">
         <f>F96-F95</f>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="E124" s="8">
         <f>E97-E96</f>
-        <v>67.22</v>
+        <v>66.94</v>
       </c>
       <c r="F124" s="8">
         <f>F97-F96</f>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="E125" s="8">
         <f>E98-E97</f>
-        <v>67.5</v>
+        <v>67.22</v>
       </c>
       <c r="F125" s="8">
         <f>F98-F97</f>
@@ -5421,7 +5421,7 @@
       </c>
       <c r="E126" s="8">
         <f>E99-E98</f>
-        <v>67.78</v>
+        <v>67.5</v>
       </c>
       <c r="F126" s="8">
         <f>F99-F98</f>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="E127" s="8">
         <f>E100-E99</f>
-        <v>68.07</v>
+        <v>67.79</v>
       </c>
       <c r="F127" s="8">
         <f>F100-F99</f>
@@ -5491,7 +5491,7 @@
       </c>
       <c r="E128" s="8">
         <f>E101-E100</f>
-        <v>68.35</v>
+        <v>68.07</v>
       </c>
       <c r="F128" s="8">
         <f>F101-F100</f>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="E129" s="8">
         <f>E102-E101</f>
-        <v>68.64</v>
+        <v>68.35</v>
       </c>
       <c r="F129" s="8">
         <f>F102-F101</f>
@@ -5561,7 +5561,7 @@
       </c>
       <c r="E130" s="8">
         <f>E103-E102</f>
-        <v>68.92</v>
+        <v>68.64</v>
       </c>
       <c r="F130" s="8">
         <f>F103-F102</f>
@@ -6290,55 +6290,27 @@
     </row>
     <row r="7">
       <c r="A7" s="20">
-        <v>46193</v>
+        <v>46198</v>
       </c>
       <c r="B7" t="inlineStr" s="21">
         <is>
-          <t xml:space="preserve">Interest</t>
+          <t xml:space="preserve">Transfer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="21">
         <is>
-          <t xml:space="preserve">Banko</t>
+          <t xml:space="preserve">UNO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="21">
         <is>
-          <t xml:space="preserve">Banko - Savings</t>
+          <t xml:space="preserve">UNO - Digi Savings</t>
         </is>
       </c>
       <c r="E7" s="19">
-        <v>62.5</v>
+        <v>5000</v>
       </c>
       <c r="F7" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">Interest posting (example)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20">
-        <v>46198</v>
-      </c>
-      <c r="B8" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">Transfer</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">UNO</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">UNO - Digi Savings</t>
-        </is>
-      </c>
-      <c r="E8" s="19">
-        <v>5000</v>
-      </c>
-      <c r="F8" t="inlineStr" s="21">
         <is>
           <t xml:space="preserve">Transfer in (example)</t>
         </is>
@@ -6379,10 +6351,10 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
   </cols>
@@ -6444,7 +6416,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Current balance per account = Deposits + Net Transactions. Projected columns include compounding interest from the Interest tab.</t>
+          <t xml:space="preserve">Balance Today grows automatically with interest each day/month. Current Balance = Deposits + Net Transactions (money you moved); Balance Today adds the interest accrued up to today.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -6512,16 +6484,24 @@
       </c>
       <c r="G5" t="inlineStr" s="6">
         <is>
+          <t xml:space="preserve">Interest to Date</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Balance Today</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr" s="6">
+        <is>
           <t xml:space="preserve">Interest (1 Yr)</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr" s="6">
+      <c r="J5" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Proj. Balance (1 Yr)</t>
         </is>
       </c>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
@@ -6554,16 +6534,22 @@
         <f>D6+E6</f>
         <v>48000.0</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="23">
+        <f>IFERROR(VLOOKUP(C6,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>449.15</v>
+      </c>
+      <c r="H6" s="23">
+        <f>IFERROR(VLOOKUP(C6,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>48449.15</v>
+      </c>
+      <c r="I6" s="8">
         <f>IFERROR(VLOOKUP(C6,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>5047.48</v>
       </c>
-      <c r="H6" s="8">
-        <f>F6+G6</f>
+      <c r="J6" s="8">
+        <f>F6+I6</f>
         <v>53047.48</v>
       </c>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
       <c r="K6" s="21"/>
       <c r="L6" s="21"/>
       <c r="M6" s="21"/>
@@ -6596,16 +6582,22 @@
         <f>D7+E7</f>
         <v>100000.0</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="23">
+        <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>500.0</v>
+      </c>
+      <c r="H7" s="23">
+        <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>100500.0</v>
+      </c>
+      <c r="I7" s="8">
         <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>6167.78</v>
       </c>
-      <c r="H7" s="8">
-        <f>F7+G7</f>
+      <c r="J7" s="8">
+        <f>F7+I7</f>
         <v>106167.78</v>
       </c>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
       <c r="K7" s="21"/>
       <c r="L7" s="21"/>
       <c r="M7" s="21"/>
@@ -6638,16 +6630,22 @@
         <f>D8+E8</f>
         <v>100000.0</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="23">
+        <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>500.0</v>
+      </c>
+      <c r="H8" s="23">
+        <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>100500.0</v>
+      </c>
+      <c r="I8" s="8">
         <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>6167.78</v>
       </c>
-      <c r="H8" s="8">
-        <f>F8+G8</f>
+      <c r="J8" s="8">
+        <f>F8+I8</f>
         <v>106167.78</v>
       </c>
-      <c r="I8" s="21"/>
-      <c r="J8" s="21"/>
       <c r="K8" s="21"/>
       <c r="L8" s="21"/>
       <c r="M8" s="21"/>
@@ -6680,16 +6678,22 @@
         <f>D9+E9</f>
         <v>25000.0</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="23">
+        <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>116.67</v>
+      </c>
+      <c r="H9" s="23">
+        <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>25116.67</v>
+      </c>
+      <c r="I9" s="8">
         <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>1436.5</v>
       </c>
-      <c r="H9" s="8">
-        <f>F9+G9</f>
+      <c r="J9" s="8">
+        <f>F9+I9</f>
         <v>26436.5</v>
       </c>
-      <c r="I9" s="21"/>
-      <c r="J9" s="21"/>
       <c r="K9" s="21"/>
       <c r="L9" s="21"/>
       <c r="M9" s="21"/>
@@ -6722,16 +6726,22 @@
         <f>D10+E10</f>
         <v>25000.0</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="23">
+        <f>IFERROR(VLOOKUP(C10,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>81.64</v>
+      </c>
+      <c r="H10" s="23">
+        <f>IFERROR(VLOOKUP(C10,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>25081.64</v>
+      </c>
+      <c r="I10" s="8">
         <f>IFERROR(VLOOKUP(C10,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>890.45</v>
       </c>
-      <c r="H10" s="8">
-        <f>F10+G10</f>
+      <c r="J10" s="8">
+        <f>F10+I10</f>
         <v>25890.45</v>
       </c>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
       <c r="K10" s="21"/>
       <c r="L10" s="21"/>
       <c r="M10" s="21"/>
@@ -6764,16 +6774,22 @@
         <f>D11+E11</f>
         <v>50000.0</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="23">
+        <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>250.0</v>
+      </c>
+      <c r="H11" s="23">
+        <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>50250.0</v>
+      </c>
+      <c r="I11" s="8">
         <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>3083.89</v>
       </c>
-      <c r="H11" s="8">
-        <f>F11+G11</f>
+      <c r="J11" s="8">
+        <f>F11+I11</f>
         <v>53083.89</v>
       </c>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
       <c r="K11" s="21"/>
       <c r="L11" s="21"/>
       <c r="M11" s="21"/>
@@ -6806,16 +6822,22 @@
         <f>D12+E12</f>
         <v>50000.0</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="23">
+        <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>250.0</v>
+      </c>
+      <c r="H12" s="23">
+        <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>50250.0</v>
+      </c>
+      <c r="I12" s="8">
         <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>3083.89</v>
       </c>
-      <c r="H12" s="8">
-        <f>F12+G12</f>
+      <c r="J12" s="8">
+        <f>F12+I12</f>
         <v>53083.89</v>
       </c>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
       <c r="K12" s="21"/>
       <c r="L12" s="21"/>
       <c r="M12" s="21"/>
@@ -6848,16 +6870,22 @@
         <f>D13+E13</f>
         <v>10000.0</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="23">
+        <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>33.33</v>
+      </c>
+      <c r="H13" s="23">
+        <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>10033.33</v>
+      </c>
+      <c r="I13" s="8">
         <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>407.42</v>
       </c>
-      <c r="H13" s="8">
-        <f>F13+G13</f>
+      <c r="J13" s="8">
+        <f>F13+I13</f>
         <v>10407.42</v>
       </c>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
       <c r="K13" s="21"/>
       <c r="L13" s="21"/>
       <c r="M13" s="21"/>
@@ -6890,16 +6918,22 @@
         <f>D14+E14</f>
         <v>10000.0</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="23">
+        <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>33.33</v>
+      </c>
+      <c r="H14" s="23">
+        <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>10033.33</v>
+      </c>
+      <c r="I14" s="8">
         <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>407.42</v>
       </c>
-      <c r="H14" s="8">
-        <f>F14+G14</f>
+      <c r="J14" s="8">
+        <f>F14+I14</f>
         <v>10407.42</v>
       </c>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21"/>
       <c r="K14" s="21"/>
       <c r="L14" s="21"/>
       <c r="M14" s="21"/>
@@ -6932,16 +6966,22 @@
         <f>D15+E15</f>
         <v>30000.0</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="23">
+        <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>200.0</v>
+      </c>
+      <c r="H15" s="23">
+        <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>30200.0</v>
+      </c>
+      <c r="I15" s="8">
         <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>2489.99</v>
       </c>
-      <c r="H15" s="8">
-        <f>F15+G15</f>
+      <c r="J15" s="8">
+        <f>F15+I15</f>
         <v>32489.99</v>
       </c>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
       <c r="K15" s="21"/>
       <c r="L15" s="21"/>
       <c r="M15" s="21"/>
@@ -6968,22 +7008,28 @@
       </c>
       <c r="E16" s="8">
         <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C16)</f>
-        <v>62.5</v>
+        <v>0.0</v>
       </c>
       <c r="F16" s="8">
         <f>D16+E16</f>
-        <v>15062.5</v>
-      </c>
-      <c r="G16" s="8">
+        <v>15000.0</v>
+      </c>
+      <c r="G16" s="23">
+        <f>IFERROR(VLOOKUP(C16,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>70.02</v>
+      </c>
+      <c r="H16" s="23">
+        <f>IFERROR(VLOOKUP(C16,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>15070.02</v>
+      </c>
+      <c r="I16" s="8">
         <f>IFERROR(VLOOKUP(C16,Interest!$D$6:$L$19,9,FALSE),0)</f>
-        <v>772.22</v>
-      </c>
-      <c r="H16" s="8">
-        <f>F16+G16</f>
-        <v>15834.72</v>
-      </c>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
+        <v>769.01</v>
+      </c>
+      <c r="J16" s="8">
+        <f>F16+I16</f>
+        <v>15769.01</v>
+      </c>
       <c r="K16" s="21"/>
       <c r="L16" s="21"/>
       <c r="M16" s="21"/>
@@ -7016,16 +7062,22 @@
         <f>D17+E17</f>
         <v>10000.0</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="23">
+        <f>IFERROR(VLOOKUP(C17,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>21.45</v>
+      </c>
+      <c r="H17" s="23">
+        <f>IFERROR(VLOOKUP(C17,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>10021.45</v>
+      </c>
+      <c r="I17" s="8">
         <f>IFERROR(VLOOKUP(C17,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>232.66</v>
       </c>
-      <c r="H17" s="8">
-        <f>F17+G17</f>
+      <c r="J17" s="8">
+        <f>F17+I17</f>
         <v>10232.66</v>
       </c>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
       <c r="K17" s="21"/>
       <c r="L17" s="21"/>
       <c r="M17" s="21"/>
@@ -7058,16 +7110,22 @@
         <f>D18+E18</f>
         <v>12000.0</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="23">
+        <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>30.0</v>
+      </c>
+      <c r="H18" s="23">
+        <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>12030.0</v>
+      </c>
+      <c r="I18" s="8">
         <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>364.99</v>
       </c>
-      <c r="H18" s="8">
-        <f>F18+G18</f>
+      <c r="J18" s="8">
+        <f>F18+I18</f>
         <v>12364.99</v>
       </c>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
       <c r="K18" s="21"/>
       <c r="L18" s="21"/>
       <c r="M18" s="21"/>
@@ -7100,16 +7158,22 @@
         <f>D19+E19</f>
         <v>8000.0</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="23">
+        <f>IFERROR(VLOOKUP(C19,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>24.25</v>
+      </c>
+      <c r="H19" s="23">
+        <f>IFERROR(VLOOKUP(C19,Interest!$D$6:$Q$19,14,FALSE),0)</f>
+        <v>8024.25</v>
+      </c>
+      <c r="I19" s="8">
         <f>IFERROR(VLOOKUP(C19,Interest!$D$6:$L$19,9,FALSE),0)</f>
         <v>264.26</v>
       </c>
-      <c r="H19" s="8">
-        <f>F19+G19</f>
+      <c r="J19" s="8">
+        <f>F19+I19</f>
         <v>8264.26</v>
       </c>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21"/>
       <c r="K19" s="21"/>
       <c r="L19" s="21"/>
       <c r="M19" s="21"/>
@@ -7128,22 +7192,28 @@
       </c>
       <c r="E20" s="16">
         <f>SUM(E6:E19)</f>
-        <v>3062.5</v>
+        <v>3000.0</v>
       </c>
       <c r="F20" s="16">
         <f>SUM(F6:F19)</f>
-        <v>493062.5</v>
+        <v>493000.0</v>
       </c>
       <c r="G20" s="16">
         <f>SUM(G6:G19)</f>
-        <v>30816.71</v>
+        <v>2559.84</v>
       </c>
       <c r="H20" s="16">
         <f>SUM(H6:H19)</f>
-        <v>523879.21</v>
-      </c>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
+        <v>495559.84</v>
+      </c>
+      <c r="I20" s="16">
+        <f>SUM(I6:I19)</f>
+        <v>30813.51</v>
+      </c>
+      <c r="J20" s="16">
+        <f>SUM(J6:J19)</f>
+        <v>523813.51</v>
+      </c>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
       <c r="M20" s="16"/>
@@ -7179,13 +7249,17 @@
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="11" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="13" customWidth="1"/>
+    <col min="15" max="15" width="12" customWidth="1"/>
+    <col min="16" max="16" width="16" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7206,6 +7280,10 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" t="inlineStr" s="2">
@@ -7241,11 +7319,15 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Interest rates &amp; auto-calculated earnings. Daily accounts compound daily (rate/365); monthly accounts compound monthly (rate/12). Maya Savings overridden to 10%.</t>
+          <t xml:space="preserve">Interest auto-calculates and GROWS ON ITS OWN. 'Balance Today' accrues from each account's first deposit date up to today() every time you open the file - daily accounts step up each day, monthly accounts each month. Maya Savings = 10%.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -7260,11 +7342,15 @@
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">📈 Interest Rates &amp; Earnings</t>
+          <t xml:space="preserve">📈 Interest Rates, Earnings &amp; Live Balance</t>
         </is>
       </c>
       <c r="B4" s="4"/>
@@ -7279,6 +7365,10 @@
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" t="inlineStr" s="6">
@@ -7344,6 +7434,26 @@
       <c r="M5" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Monthly Factor</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Interest Start</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Periods Elapsed</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Interest to Date</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Balance Today</t>
         </is>
       </c>
     </row>
@@ -7404,6 +7514,22 @@
         <f>IF(F6="Daily",(1+E6/365)^(365/12),1+E6/12)</f>
         <v>1.008367</v>
       </c>
+      <c r="N6" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D6)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D6))</f>
+        <v>46174</v>
+      </c>
+      <c r="O6" s="10">
+        <f>IF(N6="",0,IF(F6="Daily",MAX(0,TODAY()-N6),MAX(0,DATEDIF(N6,TODAY(),"m"))))</f>
+        <v>34</v>
+      </c>
+      <c r="P6" s="8">
+        <f>G6*((1+H6)^O6-1)</f>
+        <v>449.15</v>
+      </c>
+      <c r="Q6" s="8">
+        <f>G6+P6</f>
+        <v>48449.15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="7">
@@ -7462,6 +7588,22 @@
         <f>IF(F7="Daily",(1+E7/365)^(365/12),1+E7/12)</f>
         <v>1.005</v>
       </c>
+      <c r="N7" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D7)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D7))</f>
+        <v>46174</v>
+      </c>
+      <c r="O7" s="10">
+        <f>IF(N7="",0,IF(F7="Daily",MAX(0,TODAY()-N7),MAX(0,DATEDIF(N7,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P7" s="8">
+        <f>G7*((1+H7)^O7-1)</f>
+        <v>500.0</v>
+      </c>
+      <c r="Q7" s="8">
+        <f>G7+P7</f>
+        <v>100500.0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="7">
@@ -7520,6 +7662,22 @@
         <f>IF(F8="Daily",(1+E8/365)^(365/12),1+E8/12)</f>
         <v>1.005</v>
       </c>
+      <c r="N8" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D8)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D8))</f>
+        <v>46174</v>
+      </c>
+      <c r="O8" s="10">
+        <f>IF(N8="",0,IF(F8="Daily",MAX(0,TODAY()-N8),MAX(0,DATEDIF(N8,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P8" s="8">
+        <f>G8*((1+H8)^O8-1)</f>
+        <v>500.0</v>
+      </c>
+      <c r="Q8" s="8">
+        <f>G8+P8</f>
+        <v>100500.0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="7">
@@ -7578,6 +7736,22 @@
         <f>IF(F9="Daily",(1+E9/365)^(365/12),1+E9/12)</f>
         <v>1.00466667</v>
       </c>
+      <c r="N9" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D9)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D9))</f>
+        <v>46174</v>
+      </c>
+      <c r="O9" s="10">
+        <f>IF(N9="",0,IF(F9="Daily",MAX(0,TODAY()-N9),MAX(0,DATEDIF(N9,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P9" s="8">
+        <f>G9*((1+H9)^O9-1)</f>
+        <v>116.67</v>
+      </c>
+      <c r="Q9" s="8">
+        <f>G9+P9</f>
+        <v>25116.67</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="7">
@@ -7636,6 +7810,22 @@
         <f>IF(F10="Daily",(1+E10/365)^(365/12),1+E10/12)</f>
         <v>1.00292078</v>
       </c>
+      <c r="N10" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D10)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D10))</f>
+        <v>46174</v>
+      </c>
+      <c r="O10" s="10">
+        <f>IF(N10="",0,IF(F10="Daily",MAX(0,TODAY()-N10),MAX(0,DATEDIF(N10,TODAY(),"m"))))</f>
+        <v>34</v>
+      </c>
+      <c r="P10" s="8">
+        <f>G10*((1+H10)^O10-1)</f>
+        <v>81.64</v>
+      </c>
+      <c r="Q10" s="8">
+        <f>G10+P10</f>
+        <v>25081.64</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="7">
@@ -7694,6 +7884,22 @@
         <f>IF(F11="Daily",(1+E11/365)^(365/12),1+E11/12)</f>
         <v>1.005</v>
       </c>
+      <c r="N11" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D11)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D11))</f>
+        <v>46174</v>
+      </c>
+      <c r="O11" s="10">
+        <f>IF(N11="",0,IF(F11="Daily",MAX(0,TODAY()-N11),MAX(0,DATEDIF(N11,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P11" s="8">
+        <f>G11*((1+H11)^O11-1)</f>
+        <v>250.0</v>
+      </c>
+      <c r="Q11" s="8">
+        <f>G11+P11</f>
+        <v>50250.0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="7">
@@ -7752,6 +7958,22 @@
         <f>IF(F12="Daily",(1+E12/365)^(365/12),1+E12/12)</f>
         <v>1.005</v>
       </c>
+      <c r="N12" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D12)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D12))</f>
+        <v>46174</v>
+      </c>
+      <c r="O12" s="10">
+        <f>IF(N12="",0,IF(F12="Daily",MAX(0,TODAY()-N12),MAX(0,DATEDIF(N12,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P12" s="8">
+        <f>G12*((1+H12)^O12-1)</f>
+        <v>250.0</v>
+      </c>
+      <c r="Q12" s="8">
+        <f>G12+P12</f>
+        <v>50250.0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="7">
@@ -7810,6 +8032,22 @@
         <f>IF(F13="Daily",(1+E13/365)^(365/12),1+E13/12)</f>
         <v>1.00333333</v>
       </c>
+      <c r="N13" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D13)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D13))</f>
+        <v>46174</v>
+      </c>
+      <c r="O13" s="10">
+        <f>IF(N13="",0,IF(F13="Daily",MAX(0,TODAY()-N13),MAX(0,DATEDIF(N13,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P13" s="8">
+        <f>G13*((1+H13)^O13-1)</f>
+        <v>33.33</v>
+      </c>
+      <c r="Q13" s="8">
+        <f>G13+P13</f>
+        <v>10033.33</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="7">
@@ -7868,6 +8106,22 @@
         <f>IF(F14="Daily",(1+E14/365)^(365/12),1+E14/12)</f>
         <v>1.00333333</v>
       </c>
+      <c r="N14" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D14)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D14))</f>
+        <v>46174</v>
+      </c>
+      <c r="O14" s="10">
+        <f>IF(N14="",0,IF(F14="Daily",MAX(0,TODAY()-N14),MAX(0,DATEDIF(N14,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P14" s="8">
+        <f>G14*((1+H14)^O14-1)</f>
+        <v>33.33</v>
+      </c>
+      <c r="Q14" s="8">
+        <f>G14+P14</f>
+        <v>10033.33</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr" s="7">
@@ -7926,6 +8180,22 @@
         <f>IF(F15="Daily",(1+E15/365)^(365/12),1+E15/12)</f>
         <v>1.00666667</v>
       </c>
+      <c r="N15" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D15)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D15))</f>
+        <v>46174</v>
+      </c>
+      <c r="O15" s="10">
+        <f>IF(N15="",0,IF(F15="Daily",MAX(0,TODAY()-N15),MAX(0,DATEDIF(N15,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P15" s="8">
+        <f>G15*((1+H15)^O15-1)</f>
+        <v>200.0</v>
+      </c>
+      <c r="Q15" s="8">
+        <f>G15+P15</f>
+        <v>30200.0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="7">
@@ -7958,7 +8228,7 @@
       </c>
       <c r="G16" s="8">
         <f>IFERROR(VLOOKUP(D16,Balance!$C$6:$H$19,4,FALSE),0)</f>
-        <v>15062.5</v>
+        <v>15000.0</v>
       </c>
       <c r="H16" s="9">
         <f>IF(F16="Daily",E16/365,E16/12)</f>
@@ -7966,7 +8236,7 @@
       </c>
       <c r="I16" s="8">
         <f>G16*H16</f>
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="J16" s="10">
         <f>IF(F16="Daily",365,12)</f>
@@ -7974,16 +8244,32 @@
       </c>
       <c r="K16" s="8">
         <f>G16*(1+H16)^J16</f>
-        <v>15834.72</v>
+        <v>15769.01</v>
       </c>
       <c r="L16" s="8">
         <f>K16-G16</f>
-        <v>772.22</v>
+        <v>769.01</v>
       </c>
       <c r="M16" s="9">
         <f>IF(F16="Daily",(1+E16/365)^(365/12),1+E16/12)</f>
         <v>1.00417507</v>
       </c>
+      <c r="N16" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D16)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D16))</f>
+        <v>46174</v>
+      </c>
+      <c r="O16" s="10">
+        <f>IF(N16="",0,IF(F16="Daily",MAX(0,TODAY()-N16),MAX(0,DATEDIF(N16,TODAY(),"m"))))</f>
+        <v>34</v>
+      </c>
+      <c r="P16" s="8">
+        <f>G16*((1+H16)^O16-1)</f>
+        <v>70.02</v>
+      </c>
+      <c r="Q16" s="8">
+        <f>G16+P16</f>
+        <v>15070.02</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="7">
@@ -8042,6 +8328,22 @@
         <f>IF(F17="Daily",(1+E17/365)^(365/12),1+E17/12)</f>
         <v>1.00191844</v>
       </c>
+      <c r="N17" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D17)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D17))</f>
+        <v>46174</v>
+      </c>
+      <c r="O17" s="10">
+        <f>IF(N17="",0,IF(F17="Daily",MAX(0,TODAY()-N17),MAX(0,DATEDIF(N17,TODAY(),"m"))))</f>
+        <v>34</v>
+      </c>
+      <c r="P17" s="8">
+        <f>G17*((1+H17)^O17-1)</f>
+        <v>21.45</v>
+      </c>
+      <c r="Q17" s="8">
+        <f>G17+P17</f>
+        <v>10021.45</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="7">
@@ -8100,6 +8402,22 @@
         <f>IF(F18="Daily",(1+E18/365)^(365/12),1+E18/12)</f>
         <v>1.0025</v>
       </c>
+      <c r="N18" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D18)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D18))</f>
+        <v>46174</v>
+      </c>
+      <c r="O18" s="10">
+        <f>IF(N18="",0,IF(F18="Daily",MAX(0,TODAY()-N18),MAX(0,DATEDIF(N18,TODAY(),"m"))))</f>
+        <v>1</v>
+      </c>
+      <c r="P18" s="8">
+        <f>G18*((1+H18)^O18-1)</f>
+        <v>30.0</v>
+      </c>
+      <c r="Q18" s="8">
+        <f>G18+P18</f>
+        <v>12030.0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="7">
@@ -8157,6 +8475,22 @@
       <c r="M19" s="9">
         <f>IF(F19="Daily",(1+E19/365)^(365/12),1+E19/12)</f>
         <v>1.00271188</v>
+      </c>
+      <c r="N19" s="11">
+        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D19)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D19))</f>
+        <v>46174</v>
+      </c>
+      <c r="O19" s="10">
+        <f>IF(N19="",0,IF(F19="Daily",MAX(0,TODAY()-N19),MAX(0,DATEDIF(N19,TODAY(),"m"))))</f>
+        <v>34</v>
+      </c>
+      <c r="P19" s="8">
+        <f>G19*((1+H19)^O19-1)</f>
+        <v>24.25</v>
+      </c>
+      <c r="Q19" s="8">
+        <f>G19+P19</f>
+        <v>8024.25</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -8172,34 +8506,44 @@
       <c r="F20" s="15"/>
       <c r="G20" s="16">
         <f>SUM(G6:G19)</f>
-        <v>493062.5</v>
+        <v>493000.0</v>
       </c>
       <c r="H20" s="15"/>
       <c r="I20" s="16">
         <f>SUM(I6:I19)</f>
-        <v>1932.29</v>
+        <v>1932.28</v>
       </c>
       <c r="J20" s="15"/>
       <c r="K20" s="16">
         <f>SUM(K6:K19)</f>
-        <v>523879.21</v>
+        <v>523813.51</v>
       </c>
       <c r="L20" s="16">
         <f>SUM(L6:L19)</f>
-        <v>30816.71</v>
+        <v>30813.51</v>
       </c>
       <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="16">
+        <f>SUM(P6:P19)</f>
+        <v>2559.84</v>
+      </c>
+      <c r="Q20" s="16">
+        <f>SUM(Q6:Q19)</f>
+        <v>495559.84</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="A3:Q3"/>
+    <mergeCell ref="A4:Q4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2:B2" location="Dashboard!A1" display="🏠 Dashboard"/>

</xml_diff>

<commit_message>
Fix Balance Today/Interest to Date showing 0: replace MINIFS (Excel 2019+) with AGGREGATE (Excel 2010+)
- MINIFS in the Interest Start column errored (#NAME?) on Excel 2016/older,
  cascading to 0 via IFERROR on Interest to Date and Balance Today
- Use AGGREGATE(15,6,...) to find earliest deposit date + ISNUMBER guard
- Updated formula reference .docx
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -7515,11 +7515,11 @@
         <v>1.008367</v>
       </c>
       <c r="N6" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D6)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D6))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D6),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O6" s="10">
-        <f>IF(N6="",0,IF(F6="Daily",MAX(0,TODAY()-N6),MAX(0,DATEDIF(N6,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N6),IF(F6="Daily",MAX(0,TODAY()-N6),MAX(0,DATEDIF(N6,TODAY(),"m"))),0)</f>
         <v>34</v>
       </c>
       <c r="P6" s="8">
@@ -7589,11 +7589,11 @@
         <v>1.005</v>
       </c>
       <c r="N7" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D7)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D7))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D7),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O7" s="10">
-        <f>IF(N7="",0,IF(F7="Daily",MAX(0,TODAY()-N7),MAX(0,DATEDIF(N7,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N7),IF(F7="Daily",MAX(0,TODAY()-N7),MAX(0,DATEDIF(N7,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P7" s="8">
@@ -7663,11 +7663,11 @@
         <v>1.005</v>
       </c>
       <c r="N8" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D8)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D8))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D8),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O8" s="10">
-        <f>IF(N8="",0,IF(F8="Daily",MAX(0,TODAY()-N8),MAX(0,DATEDIF(N8,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N8),IF(F8="Daily",MAX(0,TODAY()-N8),MAX(0,DATEDIF(N8,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P8" s="8">
@@ -7737,11 +7737,11 @@
         <v>1.00466667</v>
       </c>
       <c r="N9" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D9)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D9))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D9),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O9" s="10">
-        <f>IF(N9="",0,IF(F9="Daily",MAX(0,TODAY()-N9),MAX(0,DATEDIF(N9,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N9),IF(F9="Daily",MAX(0,TODAY()-N9),MAX(0,DATEDIF(N9,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P9" s="8">
@@ -7811,11 +7811,11 @@
         <v>1.00292078</v>
       </c>
       <c r="N10" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D10)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D10))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D10),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O10" s="10">
-        <f>IF(N10="",0,IF(F10="Daily",MAX(0,TODAY()-N10),MAX(0,DATEDIF(N10,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N10),IF(F10="Daily",MAX(0,TODAY()-N10),MAX(0,DATEDIF(N10,TODAY(),"m"))),0)</f>
         <v>34</v>
       </c>
       <c r="P10" s="8">
@@ -7885,11 +7885,11 @@
         <v>1.005</v>
       </c>
       <c r="N11" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D11)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D11))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D11),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O11" s="10">
-        <f>IF(N11="",0,IF(F11="Daily",MAX(0,TODAY()-N11),MAX(0,DATEDIF(N11,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N11),IF(F11="Daily",MAX(0,TODAY()-N11),MAX(0,DATEDIF(N11,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P11" s="8">
@@ -7959,11 +7959,11 @@
         <v>1.005</v>
       </c>
       <c r="N12" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D12)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D12))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D12),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O12" s="10">
-        <f>IF(N12="",0,IF(F12="Daily",MAX(0,TODAY()-N12),MAX(0,DATEDIF(N12,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N12),IF(F12="Daily",MAX(0,TODAY()-N12),MAX(0,DATEDIF(N12,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P12" s="8">
@@ -8033,11 +8033,11 @@
         <v>1.00333333</v>
       </c>
       <c r="N13" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D13)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D13))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D13),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O13" s="10">
-        <f>IF(N13="",0,IF(F13="Daily",MAX(0,TODAY()-N13),MAX(0,DATEDIF(N13,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N13),IF(F13="Daily",MAX(0,TODAY()-N13),MAX(0,DATEDIF(N13,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P13" s="8">
@@ -8107,11 +8107,11 @@
         <v>1.00333333</v>
       </c>
       <c r="N14" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D14)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D14))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D14),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O14" s="10">
-        <f>IF(N14="",0,IF(F14="Daily",MAX(0,TODAY()-N14),MAX(0,DATEDIF(N14,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N14),IF(F14="Daily",MAX(0,TODAY()-N14),MAX(0,DATEDIF(N14,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P14" s="8">
@@ -8181,11 +8181,11 @@
         <v>1.00666667</v>
       </c>
       <c r="N15" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D15)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D15))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D15),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O15" s="10">
-        <f>IF(N15="",0,IF(F15="Daily",MAX(0,TODAY()-N15),MAX(0,DATEDIF(N15,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N15),IF(F15="Daily",MAX(0,TODAY()-N15),MAX(0,DATEDIF(N15,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P15" s="8">
@@ -8255,11 +8255,11 @@
         <v>1.00417507</v>
       </c>
       <c r="N16" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D16)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D16))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D16),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O16" s="10">
-        <f>IF(N16="",0,IF(F16="Daily",MAX(0,TODAY()-N16),MAX(0,DATEDIF(N16,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N16),IF(F16="Daily",MAX(0,TODAY()-N16),MAX(0,DATEDIF(N16,TODAY(),"m"))),0)</f>
         <v>34</v>
       </c>
       <c r="P16" s="8">
@@ -8329,11 +8329,11 @@
         <v>1.00191844</v>
       </c>
       <c r="N17" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D17)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D17))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D17),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O17" s="10">
-        <f>IF(N17="",0,IF(F17="Daily",MAX(0,TODAY()-N17),MAX(0,DATEDIF(N17,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N17),IF(F17="Daily",MAX(0,TODAY()-N17),MAX(0,DATEDIF(N17,TODAY(),"m"))),0)</f>
         <v>34</v>
       </c>
       <c r="P17" s="8">
@@ -8403,11 +8403,11 @@
         <v>1.0025</v>
       </c>
       <c r="N18" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D18)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D18))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D18),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O18" s="10">
-        <f>IF(N18="",0,IF(F18="Daily",MAX(0,TODAY()-N18),MAX(0,DATEDIF(N18,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N18),IF(F18="Daily",MAX(0,TODAY()-N18),MAX(0,DATEDIF(N18,TODAY(),"m"))),0)</f>
         <v>1</v>
       </c>
       <c r="P18" s="8">
@@ -8477,11 +8477,11 @@
         <v>1.00271188</v>
       </c>
       <c r="N19" s="11">
-        <f>IF(COUNTIFS(Deposit!$C$6:$C$205,D19)=0,"",MINIFS(Deposit!$A$6:$A$205,Deposit!$C$6:$C$205,D19))</f>
+        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D19),1),"")</f>
         <v>46174</v>
       </c>
       <c r="O19" s="10">
-        <f>IF(N19="",0,IF(F19="Daily",MAX(0,TODAY()-N19),MAX(0,DATEDIF(N19,TODAY(),"m"))))</f>
+        <f>IF(ISNUMBER(N19),IF(F19="Daily",MAX(0,TODAY()-N19),MAX(0,DATEDIF(N19,TODAY(),"m"))),0)</f>
         <v>34</v>
       </c>
       <c r="P19" s="8">

</xml_diff>

<commit_message>
Make Interest Start an editable date value (drop AGGREGATE); accrual now uses only universal functions
- AGGREGATE array lookup returned no match on the user's Excel, leaving Periods Elapsed = 0
- Interest Start is now a plain, editable date (yellow), pre-filled with first deposit date
- Periods Elapsed / Interest to Date / Balance Today use only TODAY, DATEDIF, IF, MAX, ISNUMBER
- Updated formula reference .docx
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -245,6 +245,9 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7327,7 +7330,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Interest auto-calculates and GROWS ON ITS OWN. 'Balance Today' accrues from each account's first deposit date up to today() every time you open the file - daily accounts step up each day, monthly accounts each month. Maya Savings = 10%.</t>
+          <t xml:space="preserve">Interest auto-calculates and GROWS ON ITS OWN. 'Balance Today' accrues from the yellow 'Interest Start' date up to TODAY() every time you open the file - daily accounts step up each day, monthly accounts each month. Interest Start is pre-filled with your first deposit date; edit it if an account started elsewhere. Maya Savings = 10%.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -7514,8 +7517,7 @@
         <f>IF(F6="Daily",(1+E6/365)^(365/12),1+E6/12)</f>
         <v>1.008367</v>
       </c>
-      <c r="N6" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D6),1),"")</f>
+      <c r="N6" s="31">
         <v>46174</v>
       </c>
       <c r="O6" s="10">
@@ -7588,8 +7590,7 @@
         <f>IF(F7="Daily",(1+E7/365)^(365/12),1+E7/12)</f>
         <v>1.005</v>
       </c>
-      <c r="N7" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D7),1),"")</f>
+      <c r="N7" s="31">
         <v>46174</v>
       </c>
       <c r="O7" s="10">
@@ -7662,8 +7663,7 @@
         <f>IF(F8="Daily",(1+E8/365)^(365/12),1+E8/12)</f>
         <v>1.005</v>
       </c>
-      <c r="N8" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D8),1),"")</f>
+      <c r="N8" s="31">
         <v>46174</v>
       </c>
       <c r="O8" s="10">
@@ -7736,8 +7736,7 @@
         <f>IF(F9="Daily",(1+E9/365)^(365/12),1+E9/12)</f>
         <v>1.00466667</v>
       </c>
-      <c r="N9" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D9),1),"")</f>
+      <c r="N9" s="31">
         <v>46174</v>
       </c>
       <c r="O9" s="10">
@@ -7810,8 +7809,7 @@
         <f>IF(F10="Daily",(1+E10/365)^(365/12),1+E10/12)</f>
         <v>1.00292078</v>
       </c>
-      <c r="N10" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D10),1),"")</f>
+      <c r="N10" s="31">
         <v>46174</v>
       </c>
       <c r="O10" s="10">
@@ -7884,8 +7882,7 @@
         <f>IF(F11="Daily",(1+E11/365)^(365/12),1+E11/12)</f>
         <v>1.005</v>
       </c>
-      <c r="N11" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D11),1),"")</f>
+      <c r="N11" s="31">
         <v>46174</v>
       </c>
       <c r="O11" s="10">
@@ -7958,8 +7955,7 @@
         <f>IF(F12="Daily",(1+E12/365)^(365/12),1+E12/12)</f>
         <v>1.005</v>
       </c>
-      <c r="N12" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D12),1),"")</f>
+      <c r="N12" s="31">
         <v>46174</v>
       </c>
       <c r="O12" s="10">
@@ -8032,8 +8028,7 @@
         <f>IF(F13="Daily",(1+E13/365)^(365/12),1+E13/12)</f>
         <v>1.00333333</v>
       </c>
-      <c r="N13" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D13),1),"")</f>
+      <c r="N13" s="31">
         <v>46174</v>
       </c>
       <c r="O13" s="10">
@@ -8106,8 +8101,7 @@
         <f>IF(F14="Daily",(1+E14/365)^(365/12),1+E14/12)</f>
         <v>1.00333333</v>
       </c>
-      <c r="N14" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D14),1),"")</f>
+      <c r="N14" s="31">
         <v>46174</v>
       </c>
       <c r="O14" s="10">
@@ -8180,8 +8174,7 @@
         <f>IF(F15="Daily",(1+E15/365)^(365/12),1+E15/12)</f>
         <v>1.00666667</v>
       </c>
-      <c r="N15" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D15),1),"")</f>
+      <c r="N15" s="31">
         <v>46174</v>
       </c>
       <c r="O15" s="10">
@@ -8254,8 +8247,7 @@
         <f>IF(F16="Daily",(1+E16/365)^(365/12),1+E16/12)</f>
         <v>1.00417507</v>
       </c>
-      <c r="N16" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D16),1),"")</f>
+      <c r="N16" s="31">
         <v>46174</v>
       </c>
       <c r="O16" s="10">
@@ -8328,8 +8320,7 @@
         <f>IF(F17="Daily",(1+E17/365)^(365/12),1+E17/12)</f>
         <v>1.00191844</v>
       </c>
-      <c r="N17" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D17),1),"")</f>
+      <c r="N17" s="31">
         <v>46174</v>
       </c>
       <c r="O17" s="10">
@@ -8402,8 +8393,7 @@
         <f>IF(F18="Daily",(1+E18/365)^(365/12),1+E18/12)</f>
         <v>1.0025</v>
       </c>
-      <c r="N18" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D18),1),"")</f>
+      <c r="N18" s="31">
         <v>46174</v>
       </c>
       <c r="O18" s="10">
@@ -8476,8 +8466,7 @@
         <f>IF(F19="Daily",(1+E19/365)^(365/12),1+E19/12)</f>
         <v>1.00271188</v>
       </c>
-      <c r="N19" s="11">
-        <f>IFERROR(AGGREGATE(15,6,Deposit!$A$6:$A$205/(Deposit!$C$6:$C$205=D19),1),"")</f>
+      <c r="N19" s="31">
         <v>46174</v>
       </c>
       <c r="O19" s="10">

</xml_diff>

<commit_message>
User-friendly upgrades: dropdown menus, goal progress bar, live 'as of' date
- Deposit/Transactions: drop-down lists (Bank, Account, Type) via named ranges
  BankList/AccountList + input hints -> no more typos that break balance matching
- Dashboard: green data-bar on Personal Goal progress; live 'Figures as of <date>' stamp
- worksheet() now supports data validations + conditional formatting (correct schema order)
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -8,6 +8,10 @@
     <sheet name="Balance" sheetId="4" r:id="rId4"/>
     <sheet name="Interest" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="BankList">Dashboard!$A$17:$A$23</definedName>
+    <definedName name="AccountList">Interest!$D$6:$D$19</definedName>
+  </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -154,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -227,6 +231,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3369,7 +3376,7 @@
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
     </row>
-    <row r="4" ht="22" customHeight="1">
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" t="inlineStr" s="24">
         <is>
           <t xml:space="preserve">🔑 Key Metrics</t>
@@ -3382,79 +3389,81 @@
       <c r="F4" s="24"/>
       <c r="G4" s="24"/>
       <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="24"/>
+      <c r="I4" s="25">
+        <f>"Figures as of "&amp;TEXT(TODAY(),"mmm d, yyyy")</f>
+      </c>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" t="inlineStr" s="25">
+      <c r="A5" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve">Total Balance Today (incl. interest)</t>
         </is>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="26">
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="27">
         <f>SUM(Balance!$H$6:$H$19)</f>
         <v>495559.84</v>
       </c>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" t="inlineStr" s="25">
+      <c r="A6" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve">Total Deposited (All-Time)</t>
         </is>
       </c>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="26">
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="27">
         <f>SUM(Balance!$D$6:$D$19)</f>
         <v>490000.0</v>
       </c>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" t="inlineStr" s="25">
+      <c r="A7" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve">Interest Earned to Date (auto)</t>
         </is>
       </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="26">
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="27">
         <f>SUM(Balance!$G$6:$G$19)</f>
         <v>2559.84</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" t="inlineStr" s="25">
+      <c r="A8" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve">Total Withdrawn</t>
         </is>
       </c>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="26">
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="27">
         <f>-SUMIFS(Transactions!$E$6:$E$205,Transactions!$B$6:$B$205,"Withdrawal")</f>
         <v>2000</v>
       </c>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
     </row>
     <row r="9" ht="6" customHeight="1"/>
     <row r="10" ht="22" customHeight="1">
@@ -3477,54 +3486,54 @@
       <c r="M10" s="24"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" t="inlineStr" s="25">
+      <c r="A11" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve">Your Savings Goal Target</t>
         </is>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="28">
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="29">
         <v>100000</v>
       </c>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" t="inlineStr" s="25">
+      <c r="A12" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve">Maya Personal Goal — Balance Today</t>
         </is>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="26">
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="27">
         <f>IFERROR(VLOOKUP("Maya - Personal Goal",Balance!$C$6:$H$19,6,FALSE),0)</f>
         <v>25116.67</v>
       </c>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" t="inlineStr" s="25">
+      <c r="A13" t="inlineStr" s="26">
         <is>
           <t xml:space="preserve">Progress Toward Goal</t>
         </is>
       </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="27">
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="28">
         <f>IFERROR(E12/E11,0)</f>
         <v>0.2512</v>
       </c>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
     </row>
     <row r="14" ht="6" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -3564,7 +3573,7 @@
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="B17" s="29">
+      <c r="B17" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A17,Balance!$H$6:$H$19)</f>
         <v>274565.82</v>
       </c>
@@ -3575,7 +3584,7 @@
           <t xml:space="preserve">UNO</t>
         </is>
       </c>
-      <c r="B18" s="29">
+      <c r="B18" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A18,Balance!$H$6:$H$19)</f>
         <v>125581.64</v>
       </c>
@@ -3586,7 +3595,7 @@
           <t xml:space="preserve">Tonik</t>
         </is>
       </c>
-      <c r="B19" s="29">
+      <c r="B19" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A19,Balance!$H$6:$H$19)</f>
         <v>50266.67</v>
       </c>
@@ -3597,7 +3606,7 @@
           <t xml:space="preserve">Banko</t>
         </is>
       </c>
-      <c r="B20" s="29">
+      <c r="B20" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A20,Balance!$H$6:$H$19)</f>
         <v>15070.02</v>
       </c>
@@ -3608,7 +3617,7 @@
           <t xml:space="preserve">CIMB</t>
         </is>
       </c>
-      <c r="B21" s="29">
+      <c r="B21" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A21,Balance!$H$6:$H$19)</f>
         <v>10021.45</v>
       </c>
@@ -3619,7 +3628,7 @@
           <t xml:space="preserve">GoTyme</t>
         </is>
       </c>
-      <c r="B22" s="29">
+      <c r="B22" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A22,Balance!$H$6:$H$19)</f>
         <v>12030.0</v>
       </c>
@@ -3630,7 +3639,7 @@
           <t xml:space="preserve">Maribank</t>
         </is>
       </c>
-      <c r="B23" s="29">
+      <c r="B23" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A23,Balance!$H$6:$H$19)</f>
         <v>8024.25</v>
       </c>
@@ -5580,7 +5589,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="29">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
@@ -5588,7 +5597,8 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="I4:M4"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="E5:H5"/>
     <mergeCell ref="A6:D6"/>
@@ -5610,6 +5620,15 @@
     <mergeCell ref="A77:M77"/>
     <mergeCell ref="A105:M105"/>
   </mergeCells>
+  <conditionalFormatting sqref="E13">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A2:B2" location="Dashboard!A1" display="🏠 Dashboard"/>
     <hyperlink ref="C2:D2" location="Deposit!A1" display="➕ Deposit"/>
@@ -6100,6 +6119,14 @@
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="A4:M4"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="B6:B205">
+      <formula1>BankList</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick an account" prompt="Choose the account from the drop-down list so the balance matches correctly." sqref="C6:C205">
+      <formula1>AccountList</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="A2:B2" location="Dashboard!A1" display="🏠 Dashboard"/>
     <hyperlink ref="C2:D2" location="Deposit!A1" display="➕ Deposit"/>
@@ -6330,6 +6357,17 @@
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="A4:M4"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically - no need to record it here.)" sqref="B6:B205">
+      <formula1>"Deposit,Withdrawal,Transfer,Adjustment,Fee"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="C6:C205">
+      <formula1>BankList</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick an account" prompt="Choose the account from the drop-down list." sqref="D6:D205">
+      <formula1>AccountList</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="A2:B2" location="Dashboard!A1" display="🏠 Dashboard"/>
     <hyperlink ref="C2:D2" location="Deposit!A1" display="➕ Deposit"/>
@@ -7517,7 +7555,7 @@
         <f>IF(F6="Daily",(1+E6/365)^(365/12),1+E6/12)</f>
         <v>1.008367</v>
       </c>
-      <c r="N6" s="31">
+      <c r="N6" s="32">
         <v>46174</v>
       </c>
       <c r="O6" s="10">
@@ -7590,7 +7628,7 @@
         <f>IF(F7="Daily",(1+E7/365)^(365/12),1+E7/12)</f>
         <v>1.005</v>
       </c>
-      <c r="N7" s="31">
+      <c r="N7" s="32">
         <v>46174</v>
       </c>
       <c r="O7" s="10">
@@ -7663,7 +7701,7 @@
         <f>IF(F8="Daily",(1+E8/365)^(365/12),1+E8/12)</f>
         <v>1.005</v>
       </c>
-      <c r="N8" s="31">
+      <c r="N8" s="32">
         <v>46174</v>
       </c>
       <c r="O8" s="10">
@@ -7736,7 +7774,7 @@
         <f>IF(F9="Daily",(1+E9/365)^(365/12),1+E9/12)</f>
         <v>1.00466667</v>
       </c>
-      <c r="N9" s="31">
+      <c r="N9" s="32">
         <v>46174</v>
       </c>
       <c r="O9" s="10">
@@ -7809,7 +7847,7 @@
         <f>IF(F10="Daily",(1+E10/365)^(365/12),1+E10/12)</f>
         <v>1.00292078</v>
       </c>
-      <c r="N10" s="31">
+      <c r="N10" s="32">
         <v>46174</v>
       </c>
       <c r="O10" s="10">
@@ -7882,7 +7920,7 @@
         <f>IF(F11="Daily",(1+E11/365)^(365/12),1+E11/12)</f>
         <v>1.005</v>
       </c>
-      <c r="N11" s="31">
+      <c r="N11" s="32">
         <v>46174</v>
       </c>
       <c r="O11" s="10">
@@ -7955,7 +7993,7 @@
         <f>IF(F12="Daily",(1+E12/365)^(365/12),1+E12/12)</f>
         <v>1.005</v>
       </c>
-      <c r="N12" s="31">
+      <c r="N12" s="32">
         <v>46174</v>
       </c>
       <c r="O12" s="10">
@@ -8028,7 +8066,7 @@
         <f>IF(F13="Daily",(1+E13/365)^(365/12),1+E13/12)</f>
         <v>1.00333333</v>
       </c>
-      <c r="N13" s="31">
+      <c r="N13" s="32">
         <v>46174</v>
       </c>
       <c r="O13" s="10">
@@ -8101,7 +8139,7 @@
         <f>IF(F14="Daily",(1+E14/365)^(365/12),1+E14/12)</f>
         <v>1.00333333</v>
       </c>
-      <c r="N14" s="31">
+      <c r="N14" s="32">
         <v>46174</v>
       </c>
       <c r="O14" s="10">
@@ -8174,7 +8212,7 @@
         <f>IF(F15="Daily",(1+E15/365)^(365/12),1+E15/12)</f>
         <v>1.00666667</v>
       </c>
-      <c r="N15" s="31">
+      <c r="N15" s="32">
         <v>46174</v>
       </c>
       <c r="O15" s="10">
@@ -8247,7 +8285,7 @@
         <f>IF(F16="Daily",(1+E16/365)^(365/12),1+E16/12)</f>
         <v>1.00417507</v>
       </c>
-      <c r="N16" s="31">
+      <c r="N16" s="32">
         <v>46174</v>
       </c>
       <c r="O16" s="10">
@@ -8320,7 +8358,7 @@
         <f>IF(F17="Daily",(1+E17/365)^(365/12),1+E17/12)</f>
         <v>1.00191844</v>
       </c>
-      <c r="N17" s="31">
+      <c r="N17" s="32">
         <v>46174</v>
       </c>
       <c r="O17" s="10">
@@ -8393,7 +8431,7 @@
         <f>IF(F18="Daily",(1+E18/365)^(365/12),1+E18/12)</f>
         <v>1.0025</v>
       </c>
-      <c r="N18" s="31">
+      <c r="N18" s="32">
         <v>46174</v>
       </c>
       <c r="O18" s="10">
@@ -8466,7 +8504,7 @@
         <f>IF(F19="Daily",(1+E19/365)^(365/12),1+E19/12)</f>
         <v>1.00271188</v>
       </c>
-      <c r="N19" s="31">
+      <c r="N19" s="32">
         <v>46174</v>
       </c>
       <c r="O19" s="10">

</xml_diff>

<commit_message>
Fix Interest nav buttons: hide internal calc columns so the sheet fits on screen (no horizontal scroll)
- Hides Periodic Rate, Periods/Yr, Monthly Factor, Periods Elapsed (kept for calcs)
- Interest sheet now fits without horizontal scrolling, so the top nav bar stays visible/clickable
- Formulas and charts unaffected (hidden columns still compute)
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -7288,18 +7288,18 @@
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="8" max="8" width="11" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="10" max="10" width="10" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="13" max="13" width="12" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="13" customWidth="1"/>
-    <col min="15" max="15" width="12" customWidth="1"/>
+    <col min="15" max="15" width="12" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Polish Dashboard charts: distinct bank palette, peso-formatted axes, gridlines, rotated month labels, bottom legend
- Savings Growth (line): thicker rounded lines, subtle gridlines, currency y-axis, rotated 24-month labels, bottom legend
- Monthly Interest (stacked column): consistent colors, white segment separators, tighter gap, currency y-axis, gridlines, rotated labels
- Shared 7-color bank palette across both charts
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -265,6 +265,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -313,10 +314,11 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575">
+            <a:ln w="22225" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="4472C4"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
           <c:marker>
@@ -500,10 +502,11 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575">
+            <a:ln w="22225" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="ED7D31"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
           <c:marker>
@@ -687,10 +690,11 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575">
+            <a:ln w="22225" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="70AD47"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
           <c:marker>
@@ -874,10 +878,11 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575">
+            <a:ln w="22225" cap="rnd">
               <a:solidFill>
-                <a:srgbClr val="C00000"/>
+                <a:srgbClr val="FFC000"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
           <c:marker>
@@ -1061,10 +1066,11 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575">
+            <a:ln w="22225" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="7030A0"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
           <c:marker>
@@ -1248,10 +1254,11 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575">
+            <a:ln w="22225" cap="rnd">
               <a:solidFill>
-                <a:srgbClr val="843C0C"/>
+                <a:srgbClr val="C00000"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
           <c:marker>
@@ -1435,10 +1442,11 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575">
+            <a:ln w="22225" cap="rnd">
               <a:solidFill>
-                <a:srgbClr val="5B9BD5"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
+              <a:round/>
             </a:ln>
           </c:spPr>
           <c:marker>
@@ -1622,8 +1630,21 @@
           <c:tx>
             <c:rich>
               <a:bodyPr/>
+              <a:lstStyle/>
               <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="595959"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US" sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="595959"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t>Month</a:t>
                 </a:r>
               </a:p>
@@ -1631,7 +1652,21 @@
           </c:tx>
           <c:overlay val="0"/>
         </c:title>
+        <c:txPr>
+          <a:bodyPr rot="-2700000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
         <c:crossAx val="222"/>
+        <c:lblOffset val="100"/>
+        <c:tickLblSkip val="1"/>
+        <c:tickMarkSkip val="1"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="222"/>
@@ -1640,25 +1675,47 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="E7E7E7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
               <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
               <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="595959"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
                 <a:r>
-                  <a:t>Cumulative Balance (PHP)</a:t>
+                  <a:rPr lang="en-US" sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="595959"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Cumulative Balance</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
           <c:overlay val="0"/>
         </c:title>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:numFmt formatCode="[$₱-3409]#,##0" sourceLinked="0"/>
         <c:crossAx val="111"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
+      <c:legendPos val="b"/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -1798,6 +1855,7 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -1850,6 +1908,11 @@
             <a:solidFill>
               <a:srgbClr val="4472C4"/>
             </a:solidFill>
+            <a:ln w="3175">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:cat>
             <c:strRef>
@@ -2031,6 +2094,11 @@
             <a:solidFill>
               <a:srgbClr val="ED7D31"/>
             </a:solidFill>
+            <a:ln w="3175">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:cat>
             <c:strRef>
@@ -2212,6 +2280,11 @@
             <a:solidFill>
               <a:srgbClr val="70AD47"/>
             </a:solidFill>
+            <a:ln w="3175">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:cat>
             <c:strRef>
@@ -2391,8 +2464,13 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="C00000"/>
+              <a:srgbClr val="FFC000"/>
             </a:solidFill>
+            <a:ln w="3175">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:cat>
             <c:strRef>
@@ -2574,6 +2652,11 @@
             <a:solidFill>
               <a:srgbClr val="7030A0"/>
             </a:solidFill>
+            <a:ln w="3175">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:cat>
             <c:strRef>
@@ -2753,8 +2836,13 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="843C0C"/>
+              <a:srgbClr val="C00000"/>
             </a:solidFill>
+            <a:ln w="3175">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:cat>
             <c:strRef>
@@ -2934,8 +3022,13 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="5B9BD5"/>
+              <a:srgbClr val="595959"/>
             </a:solidFill>
+            <a:ln w="3175">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:cat>
             <c:strRef>
@@ -3099,7 +3192,7 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="60"/>
+        <c:gapWidth val="40"/>
         <c:overlap val="100"/>
         <c:axId val="333"/>
         <c:axId val="444"/>
@@ -3115,8 +3208,21 @@
           <c:tx>
             <c:rich>
               <a:bodyPr/>
+              <a:lstStyle/>
               <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="595959"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
                 <a:r>
+                  <a:rPr lang="en-US" sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="595959"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t>Month</a:t>
                 </a:r>
               </a:p>
@@ -3124,7 +3230,21 @@
           </c:tx>
           <c:overlay val="0"/>
         </c:title>
+        <c:txPr>
+          <a:bodyPr rot="-2700000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
         <c:crossAx val="444"/>
+        <c:lblOffset val="100"/>
+        <c:tickLblSkip val="1"/>
+        <c:tickMarkSkip val="1"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="444"/>
@@ -3133,25 +3253,47 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="E7E7E7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
               <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
               <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="595959"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
                 <a:r>
-                  <a:t>Interest (PHP)</a:t>
+                  <a:rPr lang="en-US" sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="595959"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Interest Earned</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
           <c:overlay val="0"/>
         </c:title>
-        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:numFmt formatCode="[$₱-3409]#,##0" sourceLinked="0"/>
         <c:crossAx val="333"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
+      <c:legendPos val="b"/>
       <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>

</xml_diff>

<commit_message>
Post interest earned as auto transactions and fold it into Current Balance
- Transactions tab: new auto-posted Interest ledger (one line per account, Date=TODAY,
  Amount=interest earned to date) beside the manual log; read-only, totals row
- Balance tab: relabeled so Current Balance = Principal (Deposits+Net Tx) + Interest Earned
- Ledger reads from Interest sheet (based on principal only) -> no double-count, no circular ref
- Dashboard labels updated; formula .docx updated
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -3543,7 +3543,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" t="inlineStr" s="26">
         <is>
-          <t xml:space="preserve">Total Balance Today (incl. interest)</t>
+          <t xml:space="preserve">Total Current Balance (incl. interest)</t>
         </is>
       </c>
       <c r="B5" s="26"/>
@@ -3647,7 +3647,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" t="inlineStr" s="26">
         <is>
-          <t xml:space="preserve">Maya Personal Goal — Balance Today</t>
+          <t xml:space="preserve">Maya Personal Goal — Current Balance</t>
         </is>
       </c>
       <c r="B12" s="26"/>
@@ -6287,19 +6287,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13" style="20" customWidth="1"/>
-    <col min="2" max="2" width="14" style="21" customWidth="1"/>
-    <col min="3" max="3" width="12" style="21" customWidth="1"/>
-    <col min="4" max="4" width="24" style="21" customWidth="1"/>
-    <col min="5" max="5" width="15" style="19" customWidth="1"/>
-    <col min="6" max="6" width="28" style="21" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="1" max="1" width="12" style="20" customWidth="1"/>
+    <col min="2" max="2" width="12" style="21" customWidth="1"/>
+    <col min="3" max="3" width="10" style="21" customWidth="1"/>
+    <col min="4" max="4" width="18" style="21" customWidth="1"/>
+    <col min="5" max="5" width="13" style="19" customWidth="1"/>
+    <col min="6" max="6" width="15" style="21" customWidth="1"/>
+    <col min="7" max="7" width="3" customWidth="1"/>
+    <col min="8" max="8" width="11" style="20" customWidth="1"/>
+    <col min="9" max="9" width="9" style="21" customWidth="1"/>
+    <col min="10" max="10" width="9" style="21" customWidth="1"/>
+    <col min="11" max="11" width="18" style="21" customWidth="1"/>
+    <col min="12" max="12" width="13" style="19" customWidth="1"/>
+    <col min="13" max="13" width="16" style="21" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6359,7 +6359,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">All money movements: deposits, withdrawals, transfers and interest postings. Use negative amounts for money out. Filter by any column.</t>
+          <t xml:space="preserve">LEFT = money you move (deposits/withdrawals/transfers) - use the filters; use negative amounts for money out. RIGHT = interest earned, posted automatically and already included in your Current Balance (do not edit).</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -6375,10 +6375,10 @@
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
     </row>
-    <row r="4" ht="22" customHeight="1">
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">🔄 Transaction Log  (use the filter arrows to search / sort)</t>
+          <t xml:space="preserve">🔄 Transaction Log  (money you move)</t>
         </is>
       </c>
       <c r="B4" s="4"/>
@@ -6387,7 +6387,11 @@
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="H4" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">🪙 Interest Earned  (auto-posted — do not edit)</t>
+        </is>
+      </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -6425,13 +6429,37 @@
           <t xml:space="preserve">Notes</t>
         </is>
       </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
+      <c r="G5" s="0"/>
+      <c r="H5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Type</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Bank</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Account</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Amount</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20">
@@ -6460,6 +6488,34 @@
           <t xml:space="preserve">ATM withdrawal (example)</t>
         </is>
       </c>
+      <c r="H6" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I6" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Savings</t>
+        </is>
+      </c>
+      <c r="L6" s="23">
+        <f>IFERROR(VLOOKUP(K6,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>449.15</v>
+      </c>
+      <c r="M6" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20">
@@ -6488,9 +6544,408 @@
           <t xml:space="preserve">Transfer in (example)</t>
         </is>
       </c>
+      <c r="H7" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I7" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Time Deposit 1</t>
+        </is>
+      </c>
+      <c r="L7" s="23">
+        <f>IFERROR(VLOOKUP(K7,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>500.0</v>
+      </c>
+      <c r="M7" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="H8" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I8" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Time Deposit 2</t>
+        </is>
+      </c>
+      <c r="L8" s="23">
+        <f>IFERROR(VLOOKUP(K8,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>500.0</v>
+      </c>
+      <c r="M8" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="H9" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I9" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Personal Goal</t>
+        </is>
+      </c>
+      <c r="L9" s="23">
+        <f>IFERROR(VLOOKUP(K9,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>116.67</v>
+      </c>
+      <c r="M9" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="H10" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I10" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO - Digi Savings</t>
+        </is>
+      </c>
+      <c r="L10" s="23">
+        <f>IFERROR(VLOOKUP(K10,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>81.64</v>
+      </c>
+      <c r="M10" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="H11" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I11" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO - Time Deposit 1</t>
+        </is>
+      </c>
+      <c r="L11" s="23">
+        <f>IFERROR(VLOOKUP(K11,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>250.0</v>
+      </c>
+      <c r="M11" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="H12" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I12" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO - Time Deposit 2</t>
+        </is>
+      </c>
+      <c r="L12" s="23">
+        <f>IFERROR(VLOOKUP(K12,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>250.0</v>
+      </c>
+      <c r="M12" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="H13" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I13" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Stash 1</t>
+        </is>
+      </c>
+      <c r="L13" s="23">
+        <f>IFERROR(VLOOKUP(K13,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>33.33</v>
+      </c>
+      <c r="M13" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="H14" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I14" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Stash 2</t>
+        </is>
+      </c>
+      <c r="L14" s="23">
+        <f>IFERROR(VLOOKUP(K14,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>33.33</v>
+      </c>
+      <c r="M14" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="H15" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Time Deposit</t>
+        </is>
+      </c>
+      <c r="L15" s="23">
+        <f>IFERROR(VLOOKUP(K15,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>200.0</v>
+      </c>
+      <c r="M15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="H16" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I16" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Banko</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Banko - Savings</t>
+        </is>
+      </c>
+      <c r="L16" s="23">
+        <f>IFERROR(VLOOKUP(K16,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>70.02</v>
+      </c>
+      <c r="M16" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="H17" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">CIMB</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">CIMB - Savings</t>
+        </is>
+      </c>
+      <c r="L17" s="23">
+        <f>IFERROR(VLOOKUP(K17,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>21.45</v>
+      </c>
+      <c r="M17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="H18" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">GoTyme</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">GoTyme - GoSave</t>
+        </is>
+      </c>
+      <c r="L18" s="23">
+        <f>IFERROR(VLOOKUP(K18,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>30.0</v>
+      </c>
+      <c r="M18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="H19" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="I19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maribank</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maribank - Savings</t>
+        </is>
+      </c>
+      <c r="L19" s="23">
+        <f>IFERROR(VLOOKUP(K19,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>24.25</v>
+      </c>
+      <c r="M19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="K20" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve">Total interest</t>
+        </is>
+      </c>
+      <c r="L20" s="16">
+        <f>SUM(L6:L19)</f>
+        <v>2559.84</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
@@ -6498,10 +6953,11 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="H4:M4"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically - no need to record it here.)" sqref="B6:B205">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically on the right - no need to record it here.)" sqref="B6:B205">
       <formula1>"Deposit,Withdrawal,Transfer,Adjustment,Fee"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="C6:C205">
@@ -6600,7 +7056,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Balance Today grows automatically with interest each day/month. Current Balance = Deposits + Net Transactions (money you moved); Balance Today adds the interest accrued up to today.</t>
+          <t xml:space="preserve">Current Balance = Principal (Deposits + Net Transactions) + Interest Earned. Interest is posted automatically on the Transactions tab and grows each day/month, so Current Balance rises on its own.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -6663,17 +7119,17 @@
       </c>
       <c r="F5" t="inlineStr" s="6">
         <is>
+          <t xml:space="preserve">Principal</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Interest Earned</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr" s="6">
+        <is>
           <t xml:space="preserve">Current Balance</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Interest to Date</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Balance Today</t>
         </is>
       </c>
       <c r="I5" t="inlineStr" s="6">

</xml_diff>

<commit_message>
Fix Transactions layout: stack auto-interest ledger BELOW the log (no shared rows)
- Interest ledger moved from beside the table (shared rows 6-19) to rows 49-62
  so filtering/sorting the manual log no longer hides or scrambles it
- Manual table trimmed to 40 rows (A5:F45) - cleaner, no giant empty striped block
- Balance & Dashboard now use structured refs SUMIFS(tblTransactions[...]) so they
  sum only the manual log, never the auto-interest ledger (no double-count/loop)
- Updated formula .docx
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -3412,8 +3412,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblTransactions" displayName="tblTransactions" ref="A5:F205" totalsRowShown="0">
-  <autoFilter ref="A5:F205"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblTransactions" displayName="tblTransactions" ref="A5:F45" totalsRowShown="0">
+  <autoFilter ref="A5:F45"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Type"/>
@@ -3601,7 +3601,7 @@
       <c r="C8" s="26"/>
       <c r="D8" s="26"/>
       <c r="E8" s="27">
-        <f>-SUMIFS(Transactions!$E$6:$E$205,Transactions!$B$6:$B$205,"Withdrawal")</f>
+        <f>-SUMIFS(tblTransactions[Amount],tblTransactions[Type],"Withdrawal")</f>
         <v>2000</v>
       </c>
       <c r="F8" s="27"/>
@@ -6287,19 +6287,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" style="20" customWidth="1"/>
-    <col min="2" max="2" width="12" style="21" customWidth="1"/>
-    <col min="3" max="3" width="10" style="21" customWidth="1"/>
-    <col min="4" max="4" width="18" style="21" customWidth="1"/>
-    <col min="5" max="5" width="13" style="19" customWidth="1"/>
-    <col min="6" max="6" width="15" style="21" customWidth="1"/>
-    <col min="7" max="7" width="3" customWidth="1"/>
-    <col min="8" max="8" width="11" style="20" customWidth="1"/>
-    <col min="9" max="9" width="9" style="21" customWidth="1"/>
-    <col min="10" max="10" width="9" style="21" customWidth="1"/>
-    <col min="11" max="11" width="18" style="21" customWidth="1"/>
-    <col min="12" max="12" width="13" style="19" customWidth="1"/>
-    <col min="13" max="13" width="16" style="21" customWidth="1"/>
+    <col min="1" max="1" width="13" style="20" customWidth="1"/>
+    <col min="2" max="2" width="14" style="21" customWidth="1"/>
+    <col min="3" max="3" width="12" style="21" customWidth="1"/>
+    <col min="4" max="4" width="24" style="21" customWidth="1"/>
+    <col min="5" max="5" width="15" style="19" customWidth="1"/>
+    <col min="6" max="6" width="28" style="21" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6359,7 +6359,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">LEFT = money you move (deposits/withdrawals/transfers) - use the filters; use negative amounts for money out. RIGHT = interest earned, posted automatically and already included in your Current Balance (do not edit).</t>
+          <t xml:space="preserve">Log money you move here (deposits/withdrawals/transfers) - use negative amounts for money out, and the filter arrows to search. Interest earned is listed automatically further down and is already included in your Current Balance - do not edit it.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -6375,10 +6375,10 @@
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
     </row>
-    <row r="4" ht="20" customHeight="1">
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">🔄 Transaction Log  (money you move)</t>
+          <t xml:space="preserve">🔄 Transaction Log  (money you move — use the filters)</t>
         </is>
       </c>
       <c r="B4" s="4"/>
@@ -6387,11 +6387,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
-      <c r="H4" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">🪙 Interest Earned  (auto-posted — do not edit)</t>
-        </is>
-      </c>
+      <c r="H4" s="4"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -6429,37 +6425,6 @@
           <t xml:space="preserve">Notes</t>
         </is>
       </c>
-      <c r="G5" s="0"/>
-      <c r="H5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Date</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Type</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Bank</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Account</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Amount</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Notes</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="20">
@@ -6488,34 +6453,6 @@
           <t xml:space="preserve">ATM withdrawal (example)</t>
         </is>
       </c>
-      <c r="H6" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="I6" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya - Savings</t>
-        </is>
-      </c>
-      <c r="L6" s="23">
-        <f>IFERROR(VLOOKUP(K6,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>449.15</v>
-      </c>
-      <c r="M6" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="20">
@@ -6544,404 +6481,507 @@
           <t xml:space="preserve">Transfer in (example)</t>
         </is>
       </c>
-      <c r="H7" s="11">
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">🪙 Interest Earned  (auto-posted — do not edit)</t>
+        </is>
+      </c>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47" s="4"/>
+      <c r="J47" s="4"/>
+      <c r="K47" s="4"/>
+      <c r="L47" s="4"/>
+      <c r="M47" s="4"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Type</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Bank</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Account</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Amount</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I7" t="inlineStr" s="7">
+      <c r="B49" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr" s="7">
+      <c r="C49" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya - Time Deposit 1</t>
-        </is>
-      </c>
-      <c r="L7" s="23">
-        <f>IFERROR(VLOOKUP(K7,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>500.0</v>
-      </c>
-      <c r="M7" t="inlineStr" s="7">
+      <c r="D49" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Savings</t>
+        </is>
+      </c>
+      <c r="E49" s="23">
+        <f>IFERROR(VLOOKUP(D49,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>449.15</v>
+      </c>
+      <c r="F49" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="H8" s="11">
+    <row r="50">
+      <c r="A50" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I8" t="inlineStr" s="7">
+      <c r="B50" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr" s="7">
+      <c r="C50" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya - Time Deposit 2</t>
-        </is>
-      </c>
-      <c r="L8" s="23">
-        <f>IFERROR(VLOOKUP(K8,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="D50" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Time Deposit 1</t>
+        </is>
+      </c>
+      <c r="E50" s="23">
+        <f>IFERROR(VLOOKUP(D50,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>500.0</v>
       </c>
-      <c r="M8" t="inlineStr" s="7">
+      <c r="F50" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="H9" s="11">
+    <row r="51">
+      <c r="A51" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I9" t="inlineStr" s="7">
+      <c r="B51" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr" s="7">
+      <c r="C51" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya - Personal Goal</t>
-        </is>
-      </c>
-      <c r="L9" s="23">
-        <f>IFERROR(VLOOKUP(K9,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>116.67</v>
-      </c>
-      <c r="M9" t="inlineStr" s="7">
+      <c r="D51" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Time Deposit 2</t>
+        </is>
+      </c>
+      <c r="E51" s="23">
+        <f>IFERROR(VLOOKUP(D51,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>500.0</v>
+      </c>
+      <c r="F51" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="H10" s="11">
+    <row r="52">
+      <c r="A52" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I10" t="inlineStr" s="7">
+      <c r="B52" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO - Digi Savings</t>
-        </is>
-      </c>
-      <c r="L10" s="23">
-        <f>IFERROR(VLOOKUP(K10,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>81.64</v>
-      </c>
-      <c r="M10" t="inlineStr" s="7">
+      <c r="C52" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Personal Goal</t>
+        </is>
+      </c>
+      <c r="E52" s="23">
+        <f>IFERROR(VLOOKUP(D52,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>116.67</v>
+      </c>
+      <c r="F52" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="H11" s="11">
+    <row r="53">
+      <c r="A53" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I11" t="inlineStr" s="7">
+      <c r="B53" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr" s="7">
+      <c r="C53" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO - Time Deposit 1</t>
-        </is>
-      </c>
-      <c r="L11" s="23">
-        <f>IFERROR(VLOOKUP(K11,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>250.0</v>
-      </c>
-      <c r="M11" t="inlineStr" s="7">
+      <c r="D53" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO - Digi Savings</t>
+        </is>
+      </c>
+      <c r="E53" s="23">
+        <f>IFERROR(VLOOKUP(D53,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>81.64</v>
+      </c>
+      <c r="F53" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="H12" s="11">
+    <row r="54">
+      <c r="A54" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I12" t="inlineStr" s="7">
+      <c r="B54" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr" s="7">
+      <c r="C54" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO - Time Deposit 2</t>
-        </is>
-      </c>
-      <c r="L12" s="23">
-        <f>IFERROR(VLOOKUP(K12,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="D54" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO - Time Deposit 1</t>
+        </is>
+      </c>
+      <c r="E54" s="23">
+        <f>IFERROR(VLOOKUP(D54,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>250.0</v>
       </c>
-      <c r="M12" t="inlineStr" s="7">
+      <c r="F54" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="H13" s="11">
+    <row r="55">
+      <c r="A55" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I13" t="inlineStr" s="7">
+      <c r="B55" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik - Stash 1</t>
-        </is>
-      </c>
-      <c r="L13" s="23">
-        <f>IFERROR(VLOOKUP(K13,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.33</v>
-      </c>
-      <c r="M13" t="inlineStr" s="7">
+      <c r="C55" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO - Time Deposit 2</t>
+        </is>
+      </c>
+      <c r="E55" s="23">
+        <f>IFERROR(VLOOKUP(D55,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>250.0</v>
+      </c>
+      <c r="F55" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="H14" s="11">
+    <row r="56">
+      <c r="A56" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I14" t="inlineStr" s="7">
+      <c r="B56" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr" s="7">
+      <c r="C56" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Tonik</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik - Stash 2</t>
-        </is>
-      </c>
-      <c r="L14" s="23">
-        <f>IFERROR(VLOOKUP(K14,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="D56" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Stash 1</t>
+        </is>
+      </c>
+      <c r="E56" s="23">
+        <f>IFERROR(VLOOKUP(D56,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>33.33</v>
       </c>
-      <c r="M14" t="inlineStr" s="7">
+      <c r="F56" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="H15" s="11">
+    <row r="57">
+      <c r="A57" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I15" t="inlineStr" s="7">
+      <c r="B57" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr" s="7">
+      <c r="C57" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Tonik</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik - Time Deposit</t>
-        </is>
-      </c>
-      <c r="L15" s="23">
-        <f>IFERROR(VLOOKUP(K15,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>200.0</v>
-      </c>
-      <c r="M15" t="inlineStr" s="7">
+      <c r="D57" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Stash 2</t>
+        </is>
+      </c>
+      <c r="E57" s="23">
+        <f>IFERROR(VLOOKUP(D57,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>33.33</v>
+      </c>
+      <c r="F57" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="H16" s="11">
+    <row r="58">
+      <c r="A58" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I16" t="inlineStr" s="7">
+      <c r="B58" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Banko</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Banko - Savings</t>
-        </is>
-      </c>
-      <c r="L16" s="23">
-        <f>IFERROR(VLOOKUP(K16,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>70.02</v>
-      </c>
-      <c r="M16" t="inlineStr" s="7">
+      <c r="C58" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Time Deposit</t>
+        </is>
+      </c>
+      <c r="E58" s="23">
+        <f>IFERROR(VLOOKUP(D58,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>200.0</v>
+      </c>
+      <c r="F58" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="H17" s="11">
+    <row r="59">
+      <c r="A59" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I17" t="inlineStr" s="7">
+      <c r="B59" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CIMB</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CIMB - Savings</t>
-        </is>
-      </c>
-      <c r="L17" s="23">
-        <f>IFERROR(VLOOKUP(K17,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>21.45</v>
-      </c>
-      <c r="M17" t="inlineStr" s="7">
+      <c r="C59" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Banko</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Banko - Savings</t>
+        </is>
+      </c>
+      <c r="E59" s="23">
+        <f>IFERROR(VLOOKUP(D59,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>70.02</v>
+      </c>
+      <c r="F59" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="H18" s="11">
+    <row r="60">
+      <c r="A60" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I18" t="inlineStr" s="7">
+      <c r="B60" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">GoTyme</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">GoTyme - GoSave</t>
-        </is>
-      </c>
-      <c r="L18" s="23">
-        <f>IFERROR(VLOOKUP(K18,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>30.0</v>
-      </c>
-      <c r="M18" t="inlineStr" s="7">
+      <c r="C60" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">CIMB</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">CIMB - Savings</t>
+        </is>
+      </c>
+      <c r="E60" s="23">
+        <f>IFERROR(VLOOKUP(D60,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>21.45</v>
+      </c>
+      <c r="F60" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="H19" s="11">
+    <row r="61">
+      <c r="A61" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="I19" t="inlineStr" s="7">
+      <c r="B61" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr" s="7">
+      <c r="C61" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">GoTyme</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">GoTyme - GoSave</t>
+        </is>
+      </c>
+      <c r="E61" s="23">
+        <f>IFERROR(VLOOKUP(D61,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>30.0</v>
+      </c>
+      <c r="F61" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B62" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maribank</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr" s="7">
+      <c r="D62" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maribank - Savings</t>
         </is>
       </c>
-      <c r="L19" s="23">
-        <f>IFERROR(VLOOKUP(K19,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E62" s="23">
+        <f>IFERROR(VLOOKUP(D62,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>24.25</v>
       </c>
-      <c r="M19" t="inlineStr" s="7">
+      <c r="F62" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="K20" t="inlineStr" s="15">
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr" s="15">
         <is>
           <t xml:space="preserve">Total interest</t>
         </is>
       </c>
-      <c r="L20" s="16">
-        <f>SUM(L6:L19)</f>
+      <c r="E63" s="16">
+        <f>SUM(E49:E62)</f>
         <v>2559.84</v>
+      </c>
+      <c r="F63" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -6953,17 +6993,17 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="H4:M4"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="A47:M47"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically on the right - no need to record it here.)" sqref="B6:B205">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically below - no need to record it here.)" sqref="B6:B45">
       <formula1>"Deposit,Withdrawal,Transfer,Adjustment,Fee"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="C6:C205">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="C6:C45">
       <formula1>BankList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick an account" prompt="Choose the account from the drop-down list." sqref="D6:D205">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick an account" prompt="Choose the account from the drop-down list." sqref="D6:D45">
       <formula1>AccountList</formula1>
     </dataValidation>
   </dataValidations>
@@ -7167,7 +7207,7 @@
         <v>50000.0</v>
       </c>
       <c r="E6" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C6)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C6)</f>
         <v>-2000.0</v>
       </c>
       <c r="F6" s="8">
@@ -7215,7 +7255,7 @@
         <v>100000.0</v>
       </c>
       <c r="E7" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C7)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C7)</f>
         <v>0.0</v>
       </c>
       <c r="F7" s="8">
@@ -7263,7 +7303,7 @@
         <v>100000.0</v>
       </c>
       <c r="E8" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C8)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C8)</f>
         <v>0.0</v>
       </c>
       <c r="F8" s="8">
@@ -7311,7 +7351,7 @@
         <v>25000.0</v>
       </c>
       <c r="E9" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C9)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C9)</f>
         <v>0.0</v>
       </c>
       <c r="F9" s="8">
@@ -7359,7 +7399,7 @@
         <v>20000.0</v>
       </c>
       <c r="E10" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C10)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C10)</f>
         <v>5000.0</v>
       </c>
       <c r="F10" s="8">
@@ -7407,7 +7447,7 @@
         <v>50000.0</v>
       </c>
       <c r="E11" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C11)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C11)</f>
         <v>0.0</v>
       </c>
       <c r="F11" s="8">
@@ -7455,7 +7495,7 @@
         <v>50000.0</v>
       </c>
       <c r="E12" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C12)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C12)</f>
         <v>0.0</v>
       </c>
       <c r="F12" s="8">
@@ -7503,7 +7543,7 @@
         <v>10000.0</v>
       </c>
       <c r="E13" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C13)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C13)</f>
         <v>0.0</v>
       </c>
       <c r="F13" s="8">
@@ -7551,7 +7591,7 @@
         <v>10000.0</v>
       </c>
       <c r="E14" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C14)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C14)</f>
         <v>0.0</v>
       </c>
       <c r="F14" s="8">
@@ -7599,7 +7639,7 @@
         <v>30000.0</v>
       </c>
       <c r="E15" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C15)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C15)</f>
         <v>0.0</v>
       </c>
       <c r="F15" s="8">
@@ -7647,7 +7687,7 @@
         <v>15000.0</v>
       </c>
       <c r="E16" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C16)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C16)</f>
         <v>0.0</v>
       </c>
       <c r="F16" s="8">
@@ -7695,7 +7735,7 @@
         <v>10000.0</v>
       </c>
       <c r="E17" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C17)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C17)</f>
         <v>0.0</v>
       </c>
       <c r="F17" s="8">
@@ -7743,7 +7783,7 @@
         <v>12000.0</v>
       </c>
       <c r="E18" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C18)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C18)</f>
         <v>0.0</v>
       </c>
       <c r="F18" s="8">
@@ -7791,7 +7831,7 @@
         <v>8000.0</v>
       </c>
       <c r="E19" s="8">
-        <f>SUMIFS(Transactions!$E$6:$E$205,Transactions!$D$6:$D$205,C19)</f>
+        <f>SUMIFS(tblTransactions[Amount],tblTransactions[Account],C19)</f>
         <v>0.0</v>
       </c>
       <c r="F19" s="8">

</xml_diff>

<commit_message>
Remove misleading Interest/Period total (it mixed per-day and per-month figures)
Per-row Interest/Period values are correct (1 day for daily accounts, 1 month for
monthly), but their sum mixes time units, so the total is dropped. True accrued
total remains in the Interest to Date column.
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -9175,10 +9175,7 @@
         <v>493000.0</v>
       </c>
       <c r="H20" s="15"/>
-      <c r="I20" s="16">
-        <f>SUM(I6:I19)</f>
-        <v>1932.28</v>
-      </c>
+      <c r="I20" s="15"/>
       <c r="J20" s="15"/>
       <c r="K20" s="16">
         <f>SUM(K6:K19)</f>

</xml_diff>

<commit_message>
Change Interest/Period to Interest/Day (per-day for all accounts)
- Column now = Current Balance x Annual Rate / 365 for every account (daily & monthly)
- Consistent per-day basis, so the column total is meaningful again (restored)
- Compounding/accrual (Interest to Date, Balance Today) unchanged
- Updated formula .docx
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -8093,7 +8093,7 @@
       </c>
       <c r="I5" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Interest / Period</t>
+          <t xml:space="preserve">Interest / Day</t>
         </is>
       </c>
       <c r="J5" t="inlineStr" s="6">
@@ -8175,7 +8175,7 @@
         <v>0.00027397</v>
       </c>
       <c r="I6" s="8">
-        <f>G6*H6</f>
+        <f>G6*E6/365</f>
         <v>13.15</v>
       </c>
       <c r="J6" s="10">
@@ -8248,8 +8248,8 @@
         <v>0.005</v>
       </c>
       <c r="I7" s="8">
-        <f>G7*H7</f>
-        <v>500.0</v>
+        <f>G7*E7/365</f>
+        <v>16.44</v>
       </c>
       <c r="J7" s="10">
         <f>IF(F7="Daily",365,12)</f>
@@ -8321,8 +8321,8 @@
         <v>0.005</v>
       </c>
       <c r="I8" s="8">
-        <f>G8*H8</f>
-        <v>500.0</v>
+        <f>G8*E8/365</f>
+        <v>16.44</v>
       </c>
       <c r="J8" s="10">
         <f>IF(F8="Daily",365,12)</f>
@@ -8394,8 +8394,8 @@
         <v>0.00466667</v>
       </c>
       <c r="I9" s="8">
-        <f>G9*H9</f>
-        <v>116.67</v>
+        <f>G9*E9/365</f>
+        <v>3.84</v>
       </c>
       <c r="J9" s="10">
         <f>IF(F9="Daily",365,12)</f>
@@ -8467,7 +8467,7 @@
         <v>9.589e-05</v>
       </c>
       <c r="I10" s="8">
-        <f>G10*H10</f>
+        <f>G10*E10/365</f>
         <v>2.4</v>
       </c>
       <c r="J10" s="10">
@@ -8540,8 +8540,8 @@
         <v>0.005</v>
       </c>
       <c r="I11" s="8">
-        <f>G11*H11</f>
-        <v>250.0</v>
+        <f>G11*E11/365</f>
+        <v>8.22</v>
       </c>
       <c r="J11" s="10">
         <f>IF(F11="Daily",365,12)</f>
@@ -8613,8 +8613,8 @@
         <v>0.005</v>
       </c>
       <c r="I12" s="8">
-        <f>G12*H12</f>
-        <v>250.0</v>
+        <f>G12*E12/365</f>
+        <v>8.22</v>
       </c>
       <c r="J12" s="10">
         <f>IF(F12="Daily",365,12)</f>
@@ -8686,8 +8686,8 @@
         <v>0.00333333</v>
       </c>
       <c r="I13" s="8">
-        <f>G13*H13</f>
-        <v>33.33</v>
+        <f>G13*E13/365</f>
+        <v>1.1</v>
       </c>
       <c r="J13" s="10">
         <f>IF(F13="Daily",365,12)</f>
@@ -8759,8 +8759,8 @@
         <v>0.00333333</v>
       </c>
       <c r="I14" s="8">
-        <f>G14*H14</f>
-        <v>33.33</v>
+        <f>G14*E14/365</f>
+        <v>1.1</v>
       </c>
       <c r="J14" s="10">
         <f>IF(F14="Daily",365,12)</f>
@@ -8832,8 +8832,8 @@
         <v>0.00666667</v>
       </c>
       <c r="I15" s="8">
-        <f>G15*H15</f>
-        <v>200.0</v>
+        <f>G15*E15/365</f>
+        <v>6.58</v>
       </c>
       <c r="J15" s="10">
         <f>IF(F15="Daily",365,12)</f>
@@ -8905,7 +8905,7 @@
         <v>0.00013699</v>
       </c>
       <c r="I16" s="8">
-        <f>G16*H16</f>
+        <f>G16*E16/365</f>
         <v>2.05</v>
       </c>
       <c r="J16" s="10">
@@ -8978,7 +8978,7 @@
         <v>6.301e-05</v>
       </c>
       <c r="I17" s="8">
-        <f>G17*H17</f>
+        <f>G17*E17/365</f>
         <v>0.63</v>
       </c>
       <c r="J17" s="10">
@@ -9051,8 +9051,8 @@
         <v>0.0025</v>
       </c>
       <c r="I18" s="8">
-        <f>G18*H18</f>
-        <v>30.0</v>
+        <f>G18*E18/365</f>
+        <v>0.99</v>
       </c>
       <c r="J18" s="10">
         <f>IF(F18="Daily",365,12)</f>
@@ -9124,7 +9124,7 @@
         <v>8.904e-05</v>
       </c>
       <c r="I19" s="8">
-        <f>G19*H19</f>
+        <f>G19*E19/365</f>
         <v>0.71</v>
       </c>
       <c r="J19" s="10">
@@ -9175,7 +9175,10 @@
         <v>493000.0</v>
       </c>
       <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
+      <c r="I20" s="16">
+        <f>SUM(I6:I19)</f>
+        <v>81.87</v>
+      </c>
       <c r="J20" s="15"/>
       <c r="K20" s="16">
         <f>SUM(K6:K19)</f>

</xml_diff>

<commit_message>
Add Interest/Month column beside Interest/Day; label both as (est.)
- New 'Interest / Month (est.)' column (J) = Balance x Rate/12, right next to 'Interest / Day (est.)'
- Moved the Periods/Yr helper to hidden column R (Proj Balance now uses ^R); no cross-sheet
  VLOOKUP positions changed (P/Q/L/M unchanged) -> zero risk to Balance/Transactions/Dashboard
- Both rate columns visible & adjacent; sheet still fits on screen (visible width 198)
- Updated formula .docx
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -7926,13 +7926,13 @@
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="8" width="11" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="10" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
     <col min="13" max="13" width="12" hidden="1" customWidth="1"/>
@@ -7940,6 +7940,7 @@
     <col min="15" max="15" width="12" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
     <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="10" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7964,6 +7965,7 @@
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" t="inlineStr" s="2">
@@ -8003,6 +8005,7 @@
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
@@ -8026,6 +8029,7 @@
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" t="inlineStr" s="4">
@@ -8049,6 +8053,7 @@
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" t="inlineStr" s="6">
@@ -8093,47 +8098,52 @@
       </c>
       <c r="I5" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Interest / Day</t>
+          <t xml:space="preserve">Interest / Day (est.)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr" s="6">
         <is>
+          <t xml:space="preserve">Interest / Month (est.)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Proj. Balance (1 Yr)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Interest (1 Yr)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Monthly Factor</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Interest Start</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Periods Elapsed</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Interest to Date</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Balance Today</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr" s="6">
+        <is>
           <t xml:space="preserve">Periods / Yr</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Proj. Balance (1 Yr)</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Interest (1 Yr)</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Monthly Factor</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Interest Start</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Periods Elapsed</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Interest to Date</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Balance Today</t>
         </is>
       </c>
     </row>
@@ -8178,12 +8188,12 @@
         <f>G6*E6/365</f>
         <v>13.15</v>
       </c>
-      <c r="J6" s="10">
-        <f>IF(F6="Daily",365,12)</f>
-        <v>365</v>
+      <c r="J6" s="8">
+        <f>G6*E6/12</f>
+        <v>400.0</v>
       </c>
       <c r="K6" s="8">
-        <f>G6*(1+H6)^J6</f>
+        <f>G6*(1+H6)^R6</f>
         <v>53047.48</v>
       </c>
       <c r="L6" s="8">
@@ -8209,6 +8219,10 @@
         <f>G6+P6</f>
         <v>48449.15</v>
       </c>
+      <c r="R6" s="10">
+        <f>IF(F6="Daily",365,12)</f>
+        <v>365</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="7">
@@ -8251,12 +8265,12 @@
         <f>G7*E7/365</f>
         <v>16.44</v>
       </c>
-      <c r="J7" s="10">
-        <f>IF(F7="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J7" s="8">
+        <f>G7*E7/12</f>
+        <v>500.0</v>
       </c>
       <c r="K7" s="8">
-        <f>G7*(1+H7)^J7</f>
+        <f>G7*(1+H7)^R7</f>
         <v>106167.78</v>
       </c>
       <c r="L7" s="8">
@@ -8282,6 +8296,10 @@
         <f>G7+P7</f>
         <v>100500.0</v>
       </c>
+      <c r="R7" s="10">
+        <f>IF(F7="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="7">
@@ -8324,12 +8342,12 @@
         <f>G8*E8/365</f>
         <v>16.44</v>
       </c>
-      <c r="J8" s="10">
-        <f>IF(F8="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J8" s="8">
+        <f>G8*E8/12</f>
+        <v>500.0</v>
       </c>
       <c r="K8" s="8">
-        <f>G8*(1+H8)^J8</f>
+        <f>G8*(1+H8)^R8</f>
         <v>106167.78</v>
       </c>
       <c r="L8" s="8">
@@ -8355,6 +8373,10 @@
         <f>G8+P8</f>
         <v>100500.0</v>
       </c>
+      <c r="R8" s="10">
+        <f>IF(F8="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="7">
@@ -8397,12 +8419,12 @@
         <f>G9*E9/365</f>
         <v>3.84</v>
       </c>
-      <c r="J9" s="10">
-        <f>IF(F9="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J9" s="8">
+        <f>G9*E9/12</f>
+        <v>116.67</v>
       </c>
       <c r="K9" s="8">
-        <f>G9*(1+H9)^J9</f>
+        <f>G9*(1+H9)^R9</f>
         <v>26436.5</v>
       </c>
       <c r="L9" s="8">
@@ -8428,6 +8450,10 @@
         <f>G9+P9</f>
         <v>25116.67</v>
       </c>
+      <c r="R9" s="10">
+        <f>IF(F9="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="7">
@@ -8470,12 +8496,12 @@
         <f>G10*E10/365</f>
         <v>2.4</v>
       </c>
-      <c r="J10" s="10">
-        <f>IF(F10="Daily",365,12)</f>
-        <v>365</v>
+      <c r="J10" s="8">
+        <f>G10*E10/12</f>
+        <v>72.92</v>
       </c>
       <c r="K10" s="8">
-        <f>G10*(1+H10)^J10</f>
+        <f>G10*(1+H10)^R10</f>
         <v>25890.45</v>
       </c>
       <c r="L10" s="8">
@@ -8501,6 +8527,10 @@
         <f>G10+P10</f>
         <v>25081.64</v>
       </c>
+      <c r="R10" s="10">
+        <f>IF(F10="Daily",365,12)</f>
+        <v>365</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="7">
@@ -8543,12 +8573,12 @@
         <f>G11*E11/365</f>
         <v>8.22</v>
       </c>
-      <c r="J11" s="10">
-        <f>IF(F11="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J11" s="8">
+        <f>G11*E11/12</f>
+        <v>250.0</v>
       </c>
       <c r="K11" s="8">
-        <f>G11*(1+H11)^J11</f>
+        <f>G11*(1+H11)^R11</f>
         <v>53083.89</v>
       </c>
       <c r="L11" s="8">
@@ -8574,6 +8604,10 @@
         <f>G11+P11</f>
         <v>50250.0</v>
       </c>
+      <c r="R11" s="10">
+        <f>IF(F11="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="7">
@@ -8616,12 +8650,12 @@
         <f>G12*E12/365</f>
         <v>8.22</v>
       </c>
-      <c r="J12" s="10">
-        <f>IF(F12="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J12" s="8">
+        <f>G12*E12/12</f>
+        <v>250.0</v>
       </c>
       <c r="K12" s="8">
-        <f>G12*(1+H12)^J12</f>
+        <f>G12*(1+H12)^R12</f>
         <v>53083.89</v>
       </c>
       <c r="L12" s="8">
@@ -8647,6 +8681,10 @@
         <f>G12+P12</f>
         <v>50250.0</v>
       </c>
+      <c r="R12" s="10">
+        <f>IF(F12="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="7">
@@ -8689,12 +8727,12 @@
         <f>G13*E13/365</f>
         <v>1.1</v>
       </c>
-      <c r="J13" s="10">
-        <f>IF(F13="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J13" s="8">
+        <f>G13*E13/12</f>
+        <v>33.33</v>
       </c>
       <c r="K13" s="8">
-        <f>G13*(1+H13)^J13</f>
+        <f>G13*(1+H13)^R13</f>
         <v>10407.42</v>
       </c>
       <c r="L13" s="8">
@@ -8720,6 +8758,10 @@
         <f>G13+P13</f>
         <v>10033.33</v>
       </c>
+      <c r="R13" s="10">
+        <f>IF(F13="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="7">
@@ -8762,12 +8804,12 @@
         <f>G14*E14/365</f>
         <v>1.1</v>
       </c>
-      <c r="J14" s="10">
-        <f>IF(F14="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J14" s="8">
+        <f>G14*E14/12</f>
+        <v>33.33</v>
       </c>
       <c r="K14" s="8">
-        <f>G14*(1+H14)^J14</f>
+        <f>G14*(1+H14)^R14</f>
         <v>10407.42</v>
       </c>
       <c r="L14" s="8">
@@ -8793,6 +8835,10 @@
         <f>G14+P14</f>
         <v>10033.33</v>
       </c>
+      <c r="R14" s="10">
+        <f>IF(F14="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr" s="7">
@@ -8835,12 +8881,12 @@
         <f>G15*E15/365</f>
         <v>6.58</v>
       </c>
-      <c r="J15" s="10">
-        <f>IF(F15="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J15" s="8">
+        <f>G15*E15/12</f>
+        <v>200.0</v>
       </c>
       <c r="K15" s="8">
-        <f>G15*(1+H15)^J15</f>
+        <f>G15*(1+H15)^R15</f>
         <v>32489.99</v>
       </c>
       <c r="L15" s="8">
@@ -8866,6 +8912,10 @@
         <f>G15+P15</f>
         <v>30200.0</v>
       </c>
+      <c r="R15" s="10">
+        <f>IF(F15="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="7">
@@ -8908,12 +8958,12 @@
         <f>G16*E16/365</f>
         <v>2.05</v>
       </c>
-      <c r="J16" s="10">
-        <f>IF(F16="Daily",365,12)</f>
-        <v>365</v>
+      <c r="J16" s="8">
+        <f>G16*E16/12</f>
+        <v>62.5</v>
       </c>
       <c r="K16" s="8">
-        <f>G16*(1+H16)^J16</f>
+        <f>G16*(1+H16)^R16</f>
         <v>15769.01</v>
       </c>
       <c r="L16" s="8">
@@ -8939,6 +8989,10 @@
         <f>G16+P16</f>
         <v>15070.02</v>
       </c>
+      <c r="R16" s="10">
+        <f>IF(F16="Daily",365,12)</f>
+        <v>365</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="7">
@@ -8981,12 +9035,12 @@
         <f>G17*E17/365</f>
         <v>0.63</v>
       </c>
-      <c r="J17" s="10">
-        <f>IF(F17="Daily",365,12)</f>
-        <v>365</v>
+      <c r="J17" s="8">
+        <f>G17*E17/12</f>
+        <v>19.17</v>
       </c>
       <c r="K17" s="8">
-        <f>G17*(1+H17)^J17</f>
+        <f>G17*(1+H17)^R17</f>
         <v>10232.66</v>
       </c>
       <c r="L17" s="8">
@@ -9012,6 +9066,10 @@
         <f>G17+P17</f>
         <v>10021.45</v>
       </c>
+      <c r="R17" s="10">
+        <f>IF(F17="Daily",365,12)</f>
+        <v>365</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="7">
@@ -9054,12 +9112,12 @@
         <f>G18*E18/365</f>
         <v>0.99</v>
       </c>
-      <c r="J18" s="10">
-        <f>IF(F18="Daily",365,12)</f>
-        <v>12</v>
+      <c r="J18" s="8">
+        <f>G18*E18/12</f>
+        <v>30.0</v>
       </c>
       <c r="K18" s="8">
-        <f>G18*(1+H18)^J18</f>
+        <f>G18*(1+H18)^R18</f>
         <v>12364.99</v>
       </c>
       <c r="L18" s="8">
@@ -9085,6 +9143,10 @@
         <f>G18+P18</f>
         <v>12030.0</v>
       </c>
+      <c r="R18" s="10">
+        <f>IF(F18="Daily",365,12)</f>
+        <v>12</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="7">
@@ -9127,12 +9189,12 @@
         <f>G19*E19/365</f>
         <v>0.71</v>
       </c>
-      <c r="J19" s="10">
-        <f>IF(F19="Daily",365,12)</f>
-        <v>365</v>
+      <c r="J19" s="8">
+        <f>G19*E19/12</f>
+        <v>21.67</v>
       </c>
       <c r="K19" s="8">
-        <f>G19*(1+H19)^J19</f>
+        <f>G19*(1+H19)^R19</f>
         <v>8264.26</v>
       </c>
       <c r="L19" s="8">
@@ -9157,6 +9219,10 @@
       <c r="Q19" s="8">
         <f>G19+P19</f>
         <v>8024.25</v>
+      </c>
+      <c r="R19" s="10">
+        <f>IF(F19="Daily",365,12)</f>
+        <v>365</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -9179,7 +9245,10 @@
         <f>SUM(I6:I19)</f>
         <v>81.87</v>
       </c>
-      <c r="J20" s="15"/>
+      <c r="J20" s="16">
+        <f>SUM(J6:J19)</f>
+        <v>2489.59</v>
+      </c>
       <c r="K20" s="16">
         <f>SUM(K6:K19)</f>
         <v>523813.51</v>
@@ -9199,17 +9268,18 @@
         <f>SUM(Q6:Q19)</f>
         <v>495559.84</v>
       </c>
+      <c r="R20" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:R1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="A3:Q3"/>
-    <mergeCell ref="A4:Q4"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A4:R4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2:B2" location="Dashboard!A1" display="🏠 Dashboard"/>

</xml_diff>

<commit_message>
Make auto-interest ledger visible: shrink log to 20 rows so interest sits just below it (rows 22-38)
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -3412,8 +3412,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblTransactions" displayName="tblTransactions" ref="A5:F45" totalsRowShown="0">
-  <autoFilter ref="A5:F45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblTransactions" displayName="tblTransactions" ref="A5:F20" totalsRowShown="0">
+  <autoFilter ref="A5:F20"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Type"/>
@@ -6482,503 +6482,503 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" t="inlineStr" s="4">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">🪙 Interest Earned  (auto-posted — do not edit)</t>
         </is>
       </c>
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="4"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="4"/>
-      <c r="M47" s="4"/>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" t="inlineStr" s="6">
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Date</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr" s="6">
+      <c r="B23" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Type</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr" s="6">
+      <c r="C23" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Bank</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr" s="6">
+      <c r="D23" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Account</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr" s="6">
+      <c r="E23" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Amount</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr" s="6">
+      <c r="F23" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="11">
+    <row r="24">
+      <c r="A24" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B49" t="inlineStr" s="7">
+      <c r="B24" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr" s="7">
+      <c r="C24" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr" s="7">
+      <c r="D24" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya - Savings</t>
         </is>
       </c>
-      <c r="E49" s="23">
-        <f>IFERROR(VLOOKUP(D49,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E24" s="23">
+        <f>IFERROR(VLOOKUP(D24,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>449.15</v>
       </c>
-      <c r="F49" t="inlineStr" s="7">
+      <c r="F24" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="11">
+    <row r="25">
+      <c r="A25" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B50" t="inlineStr" s="7">
+      <c r="B25" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr" s="7">
+      <c r="C25" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr" s="7">
+      <c r="D25" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya - Time Deposit 1</t>
         </is>
       </c>
-      <c r="E50" s="23">
-        <f>IFERROR(VLOOKUP(D50,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E25" s="23">
+        <f>IFERROR(VLOOKUP(D25,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>500.0</v>
       </c>
-      <c r="F50" t="inlineStr" s="7">
+      <c r="F25" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="11">
+    <row r="26">
+      <c r="A26" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B51" t="inlineStr" s="7">
+      <c r="B26" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr" s="7">
+      <c r="C26" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr" s="7">
+      <c r="D26" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya - Time Deposit 2</t>
         </is>
       </c>
-      <c r="E51" s="23">
-        <f>IFERROR(VLOOKUP(D51,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E26" s="23">
+        <f>IFERROR(VLOOKUP(D26,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>500.0</v>
       </c>
-      <c r="F51" t="inlineStr" s="7">
+      <c r="F26" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="11">
+    <row r="27">
+      <c r="A27" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B52" t="inlineStr" s="7">
+      <c r="B27" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr" s="7">
+      <c r="C27" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr" s="7">
+      <c r="D27" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya - Personal Goal</t>
         </is>
       </c>
-      <c r="E52" s="23">
-        <f>IFERROR(VLOOKUP(D52,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E27" s="23">
+        <f>IFERROR(VLOOKUP(D27,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>116.67</v>
       </c>
-      <c r="F52" t="inlineStr" s="7">
+      <c r="F27" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="11">
+    <row r="28">
+      <c r="A28" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B53" t="inlineStr" s="7">
+      <c r="B28" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr" s="7">
+      <c r="C28" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr" s="7">
+      <c r="D28" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO - Digi Savings</t>
         </is>
       </c>
-      <c r="E53" s="23">
-        <f>IFERROR(VLOOKUP(D53,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E28" s="23">
+        <f>IFERROR(VLOOKUP(D28,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>81.64</v>
       </c>
-      <c r="F53" t="inlineStr" s="7">
+      <c r="F28" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="11">
+    <row r="29">
+      <c r="A29" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B54" t="inlineStr" s="7">
+      <c r="B29" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr" s="7">
+      <c r="C29" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr" s="7">
+      <c r="D29" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO - Time Deposit 1</t>
         </is>
       </c>
-      <c r="E54" s="23">
-        <f>IFERROR(VLOOKUP(D54,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E29" s="23">
+        <f>IFERROR(VLOOKUP(D29,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>250.0</v>
       </c>
-      <c r="F54" t="inlineStr" s="7">
+      <c r="F29" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="11">
+    <row r="30">
+      <c r="A30" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B55" t="inlineStr" s="7">
+      <c r="B30" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr" s="7">
+      <c r="C30" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr" s="7">
+      <c r="D30" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO - Time Deposit 2</t>
         </is>
       </c>
-      <c r="E55" s="23">
-        <f>IFERROR(VLOOKUP(D55,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E30" s="23">
+        <f>IFERROR(VLOOKUP(D30,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>250.0</v>
       </c>
-      <c r="F55" t="inlineStr" s="7">
+      <c r="F30" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="11">
+    <row r="31">
+      <c r="A31" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B56" t="inlineStr" s="7">
+      <c r="B31" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr" s="7">
+      <c r="C31" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Tonik</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr" s="7">
+      <c r="D31" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Tonik - Stash 1</t>
         </is>
       </c>
-      <c r="E56" s="23">
-        <f>IFERROR(VLOOKUP(D56,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E31" s="23">
+        <f>IFERROR(VLOOKUP(D31,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>33.33</v>
       </c>
-      <c r="F56" t="inlineStr" s="7">
+      <c r="F31" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="11">
+    <row r="32">
+      <c r="A32" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B57" t="inlineStr" s="7">
+      <c r="B32" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr" s="7">
+      <c r="C32" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Tonik</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr" s="7">
+      <c r="D32" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Tonik - Stash 2</t>
         </is>
       </c>
-      <c r="E57" s="23">
-        <f>IFERROR(VLOOKUP(D57,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E32" s="23">
+        <f>IFERROR(VLOOKUP(D32,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>33.33</v>
       </c>
-      <c r="F57" t="inlineStr" s="7">
+      <c r="F32" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="11">
+    <row r="33">
+      <c r="A33" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B58" t="inlineStr" s="7">
+      <c r="B33" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr" s="7">
+      <c r="C33" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Tonik</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr" s="7">
+      <c r="D33" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Tonik - Time Deposit</t>
         </is>
       </c>
-      <c r="E58" s="23">
-        <f>IFERROR(VLOOKUP(D58,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E33" s="23">
+        <f>IFERROR(VLOOKUP(D33,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>200.0</v>
       </c>
-      <c r="F58" t="inlineStr" s="7">
+      <c r="F33" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="11">
+    <row r="34">
+      <c r="A34" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B59" t="inlineStr" s="7">
+      <c r="B34" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr" s="7">
+      <c r="C34" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Banko</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr" s="7">
+      <c r="D34" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Banko - Savings</t>
         </is>
       </c>
-      <c r="E59" s="23">
-        <f>IFERROR(VLOOKUP(D59,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E34" s="23">
+        <f>IFERROR(VLOOKUP(D34,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>70.02</v>
       </c>
-      <c r="F59" t="inlineStr" s="7">
+      <c r="F34" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="11">
+    <row r="35">
+      <c r="A35" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B60" t="inlineStr" s="7">
+      <c r="B35" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr" s="7">
+      <c r="C35" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">CIMB</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr" s="7">
+      <c r="D35" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">CIMB - Savings</t>
         </is>
       </c>
-      <c r="E60" s="23">
-        <f>IFERROR(VLOOKUP(D60,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E35" s="23">
+        <f>IFERROR(VLOOKUP(D35,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>21.45</v>
       </c>
-      <c r="F60" t="inlineStr" s="7">
+      <c r="F35" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="11">
+    <row r="36">
+      <c r="A36" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B61" t="inlineStr" s="7">
+      <c r="B36" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr" s="7">
+      <c r="C36" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">GoTyme</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr" s="7">
+      <c r="D36" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">GoTyme - GoSave</t>
         </is>
       </c>
-      <c r="E61" s="23">
-        <f>IFERROR(VLOOKUP(D61,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E36" s="23">
+        <f>IFERROR(VLOOKUP(D36,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>30.0</v>
       </c>
-      <c r="F61" t="inlineStr" s="7">
+      <c r="F36" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="11">
+    <row r="37">
+      <c r="A37" s="11">
         <f>TODAY()</f>
         <v>46208</v>
       </c>
-      <c r="B62" t="inlineStr" s="7">
+      <c r="B37" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr" s="7">
+      <c r="C37" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maribank</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr" s="7">
+      <c r="D37" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maribank - Savings</t>
         </is>
       </c>
-      <c r="E62" s="23">
-        <f>IFERROR(VLOOKUP(D62,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+      <c r="E37" s="23">
+        <f>IFERROR(VLOOKUP(D37,Interest!$D$6:$Q$19,13,FALSE),0)</f>
         <v>24.25</v>
       </c>
-      <c r="F62" t="inlineStr" s="7">
+      <c r="F37" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" t="inlineStr" s="15">
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" t="inlineStr" s="15">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="B63" t="inlineStr" s="15">
+      <c r="B38" t="inlineStr" s="15">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="C63" t="inlineStr" s="15">
+      <c r="C38" t="inlineStr" s="15">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="D63" t="inlineStr" s="15">
+      <c r="D38" t="inlineStr" s="15">
         <is>
           <t xml:space="preserve">Total interest</t>
         </is>
       </c>
-      <c r="E63" s="16">
-        <f>SUM(E49:E62)</f>
+      <c r="E38" s="16">
+        <f>SUM(E24:E37)</f>
         <v>2559.84</v>
       </c>
-      <c r="F63" t="inlineStr" s="15">
+      <c r="F38" t="inlineStr" s="15">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6994,16 +6994,16 @@
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A47:M47"/>
+    <mergeCell ref="A22:M22"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically below - no need to record it here.)" sqref="B6:B45">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically below - no need to record it here.)" sqref="B6:B20">
       <formula1>"Deposit,Withdrawal,Transfer,Adjustment,Fee"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="C6:C45">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="C6:C20">
       <formula1>BankList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick an account" prompt="Choose the account from the drop-down list." sqref="D6:D45">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick an account" prompt="Choose the account from the drop-down list." sqref="D6:D20">
       <formula1>AccountList</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Move interest ledger ABOVE the transaction log so the log grows freely (no collision/cleanup)
- Interest Earned (auto-posted) now at top (rows 4-20); Transaction Log below (from row 22)
- Log has nothing beneath it -> it auto-extends downward indefinitely as you add rows; no manual cleanup
- Filtering/sorting the log still can't touch interest (separate rows above)
- Balance keeps structured-ref SUMIFS so it auto-adjusts to any log size
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -3412,8 +3412,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblTransactions" displayName="tblTransactions" ref="A5:F20" totalsRowShown="0">
-  <autoFilter ref="A5:F20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblTransactions" displayName="tblTransactions" ref="A23:F62" totalsRowShown="0">
+  <autoFilter ref="A23:F62"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Type"/>
@@ -6359,7 +6359,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Log money you move here (deposits/withdrawals/transfers) - use negative amounts for money out, and the filter arrows to search. Interest earned is listed automatically further down and is already included in your Current Balance - do not edit it.</t>
+          <t xml:space="preserve">Interest earned is shown at the TOP (auto-posted, read-only) and is already included in your Current Balance. Log the money you move (deposits/withdrawals/transfers) in the Transaction Log below - use negative amounts for money out and the filter arrows to search. The log can grow as long as you need (nothing sits beneath it).</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -6378,7 +6378,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">🔄 Transaction Log  (money you move — use the filters)</t>
+          <t xml:space="preserve">🪙 Interest Earned  (auto-posted — do not edit)</t>
         </is>
       </c>
       <c r="B4" s="4"/>
@@ -6427,65 +6427,460 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20">
-        <v>46188</v>
-      </c>
-      <c r="B6" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">Withdrawal</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr" s="21">
+      <c r="A6" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B6" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="21">
+      <c r="D6" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Maya - Savings</t>
         </is>
       </c>
-      <c r="E6" s="19">
-        <v>-2000</v>
-      </c>
-      <c r="F6" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">ATM withdrawal (example)</t>
+      <c r="E6" s="23">
+        <f>IFERROR(VLOOKUP(D6,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>449.15</v>
+      </c>
+      <c r="F6" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20">
-        <v>46198</v>
-      </c>
-      <c r="B7" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">Transfer</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr" s="21">
+      <c r="A7" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B7" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Time Deposit 1</t>
+        </is>
+      </c>
+      <c r="E7" s="23">
+        <f>IFERROR(VLOOKUP(D7,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>500.0</v>
+      </c>
+      <c r="F7" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B8" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Time Deposit 2</t>
+        </is>
+      </c>
+      <c r="E8" s="23">
+        <f>IFERROR(VLOOKUP(D8,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>500.0</v>
+      </c>
+      <c r="F8" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B9" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maya - Personal Goal</t>
+        </is>
+      </c>
+      <c r="E9" s="23">
+        <f>IFERROR(VLOOKUP(D9,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>116.67</v>
+      </c>
+      <c r="F9" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B10" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="21">
+      <c r="D10" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">UNO - Digi Savings</t>
         </is>
       </c>
-      <c r="E7" s="19">
-        <v>5000</v>
-      </c>
-      <c r="F7" t="inlineStr" s="21">
-        <is>
-          <t xml:space="preserve">Transfer in (example)</t>
+      <c r="E10" s="23">
+        <f>IFERROR(VLOOKUP(D10,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>81.64</v>
+      </c>
+      <c r="F10" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B11" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO - Time Deposit 1</t>
+        </is>
+      </c>
+      <c r="E11" s="23">
+        <f>IFERROR(VLOOKUP(D11,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>250.0</v>
+      </c>
+      <c r="F11" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B12" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">UNO - Time Deposit 2</t>
+        </is>
+      </c>
+      <c r="E12" s="23">
+        <f>IFERROR(VLOOKUP(D12,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>250.0</v>
+      </c>
+      <c r="F12" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B13" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Stash 1</t>
+        </is>
+      </c>
+      <c r="E13" s="23">
+        <f>IFERROR(VLOOKUP(D13,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>33.33</v>
+      </c>
+      <c r="F13" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B14" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Stash 2</t>
+        </is>
+      </c>
+      <c r="E14" s="23">
+        <f>IFERROR(VLOOKUP(D14,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>33.33</v>
+      </c>
+      <c r="F14" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Tonik - Time Deposit</t>
+        </is>
+      </c>
+      <c r="E15" s="23">
+        <f>IFERROR(VLOOKUP(D15,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>200.0</v>
+      </c>
+      <c r="F15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B16" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Banko</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Banko - Savings</t>
+        </is>
+      </c>
+      <c r="E16" s="23">
+        <f>IFERROR(VLOOKUP(D16,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>70.02</v>
+      </c>
+      <c r="F16" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">CIMB</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">CIMB - Savings</t>
+        </is>
+      </c>
+      <c r="E17" s="23">
+        <f>IFERROR(VLOOKUP(D17,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>21.45</v>
+      </c>
+      <c r="F17" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">GoTyme</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">GoTyme - GoSave</t>
+        </is>
+      </c>
+      <c r="E18" s="23">
+        <f>IFERROR(VLOOKUP(D18,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>30.0</v>
+      </c>
+      <c r="F18" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11">
+        <f>TODAY()</f>
+        <v>46208</v>
+      </c>
+      <c r="B19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maribank</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Maribank - Savings</t>
+        </is>
+      </c>
+      <c r="E19" s="23">
+        <f>IFERROR(VLOOKUP(D19,Interest!$D$6:$Q$19,13,FALSE),0)</f>
+        <v>24.25</v>
+      </c>
+      <c r="F19" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Interest earned to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve">Total interest</t>
+        </is>
+      </c>
+      <c r="E20" s="16">
+        <f>SUM(E6:E19)</f>
+        <v>2559.84</v>
+      </c>
+      <c r="F20" t="inlineStr" s="15">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">🪙 Interest Earned  (auto-posted — do not edit)</t>
+          <t xml:space="preserve">🔄 Transaction Log  (money you move — use the filters)</t>
         </is>
       </c>
       <c r="B22" s="4"/>
@@ -6534,453 +6929,58 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B24" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr" s="7">
+      <c r="A24" s="20">
+        <v>46188</v>
+      </c>
+      <c r="B24" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">Withdrawal</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr" s="21">
         <is>
           <t xml:space="preserve">Maya</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr" s="7">
+      <c r="D24" t="inlineStr" s="21">
         <is>
           <t xml:space="preserve">Maya - Savings</t>
         </is>
       </c>
-      <c r="E24" s="23">
-        <f>IFERROR(VLOOKUP(D24,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>449.15</v>
-      </c>
-      <c r="F24" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
+      <c r="E24" s="19">
+        <v>-2000</v>
+      </c>
+      <c r="F24" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">ATM withdrawal (example)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B25" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya - Time Deposit 1</t>
-        </is>
-      </c>
-      <c r="E25" s="23">
-        <f>IFERROR(VLOOKUP(D25,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>500.0</v>
-      </c>
-      <c r="F25" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B26" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya - Time Deposit 2</t>
-        </is>
-      </c>
-      <c r="E26" s="23">
-        <f>IFERROR(VLOOKUP(D26,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>500.0</v>
-      </c>
-      <c r="F26" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B27" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maya - Personal Goal</t>
-        </is>
-      </c>
-      <c r="E27" s="23">
-        <f>IFERROR(VLOOKUP(D27,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>116.67</v>
-      </c>
-      <c r="F27" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B28" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr" s="7">
+      <c r="A25" s="20">
+        <v>46198</v>
+      </c>
+      <c r="B25" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">Transfer</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr" s="21">
         <is>
           <t xml:space="preserve">UNO</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr" s="7">
+      <c r="D25" t="inlineStr" s="21">
         <is>
           <t xml:space="preserve">UNO - Digi Savings</t>
         </is>
       </c>
-      <c r="E28" s="23">
-        <f>IFERROR(VLOOKUP(D28,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>81.64</v>
-      </c>
-      <c r="F28" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B29" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO - Time Deposit 1</t>
-        </is>
-      </c>
-      <c r="E29" s="23">
-        <f>IFERROR(VLOOKUP(D29,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>250.0</v>
-      </c>
-      <c r="F29" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B30" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">UNO - Time Deposit 2</t>
-        </is>
-      </c>
-      <c r="E30" s="23">
-        <f>IFERROR(VLOOKUP(D30,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>250.0</v>
-      </c>
-      <c r="F30" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B31" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik - Stash 1</t>
-        </is>
-      </c>
-      <c r="E31" s="23">
-        <f>IFERROR(VLOOKUP(D31,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.33</v>
-      </c>
-      <c r="F31" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B32" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik - Stash 2</t>
-        </is>
-      </c>
-      <c r="E32" s="23">
-        <f>IFERROR(VLOOKUP(D32,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.33</v>
-      </c>
-      <c r="F32" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B33" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Tonik - Time Deposit</t>
-        </is>
-      </c>
-      <c r="E33" s="23">
-        <f>IFERROR(VLOOKUP(D33,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>200.0</v>
-      </c>
-      <c r="F33" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B34" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Banko</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Banko - Savings</t>
-        </is>
-      </c>
-      <c r="E34" s="23">
-        <f>IFERROR(VLOOKUP(D34,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>70.02</v>
-      </c>
-      <c r="F34" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B35" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CIMB</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CIMB - Savings</t>
-        </is>
-      </c>
-      <c r="E35" s="23">
-        <f>IFERROR(VLOOKUP(D35,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>21.45</v>
-      </c>
-      <c r="F35" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B36" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">GoTyme</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">GoTyme - GoSave</t>
-        </is>
-      </c>
-      <c r="E36" s="23">
-        <f>IFERROR(VLOOKUP(D36,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>30.0</v>
-      </c>
-      <c r="F36" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="11">
-        <f>TODAY()</f>
-        <v>46208</v>
-      </c>
-      <c r="B37" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maribank</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Maribank - Savings</t>
-        </is>
-      </c>
-      <c r="E37" s="23">
-        <f>IFERROR(VLOOKUP(D37,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>24.25</v>
-      </c>
-      <c r="F37" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Interest earned to date</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" t="inlineStr" s="15">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr" s="15">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr" s="15">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr" s="15">
-        <is>
-          <t xml:space="preserve">Total interest</t>
-        </is>
-      </c>
-      <c r="E38" s="16">
-        <f>SUM(E24:E37)</f>
-        <v>2559.84</v>
-      </c>
-      <c r="F38" t="inlineStr" s="15">
-        <is>
-          <t xml:space="preserve"/>
+      <c r="E25" s="19">
+        <v>5000</v>
+      </c>
+      <c r="F25" t="inlineStr" s="21">
+        <is>
+          <t xml:space="preserve">Transfer in (example)</t>
         </is>
       </c>
     </row>
@@ -6997,13 +6997,13 @@
     <mergeCell ref="A22:M22"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically below - no need to record it here.)" sqref="B6:B20">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a type" prompt="Choose the transaction type. (Interest is added automatically at the top - no need to record it here.)" sqref="B24:B62">
       <formula1>"Deposit,Withdrawal,Transfer,Adjustment,Fee"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="C6:C20">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick a bank" prompt="Choose the bank from the drop-down list." sqref="C24:C62">
       <formula1>BankList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick an account" prompt="Choose the account from the drop-down list." sqref="D6:D20">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pick an account" prompt="Choose the account from the drop-down list." sqref="D24:D62">
       <formula1>AccountList</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Accrue interest DAILY for every account (was monthly for monthly accounts)
- Interest to Date / Balance Today now use days-elapsed and daily compounding (rate/365) for all accounts
- Monthly-interest accounts no longer sit at a flat monthly figure; they grow every day
- Renamed helper 'Periods Elapsed' -> 'Days Elapsed'; updated subtitles + formula .docx
- Models how banks compute interest on the daily balance
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -1808,13 +1808,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>274565.82</c:v>
+                  <c:v>274700.74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>125581.64</c:v>
+                  <c:v>125642.06</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>50266.67</c:v>
+                  <c:v>50299.03</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>15070.02</c:v>
@@ -1823,7 +1823,7 @@
                   <c:v>10021.45</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>12030.0</c:v>
+                  <c:v>12033.58</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>8024.25</c:v>
@@ -3551,7 +3551,7 @@
       <c r="D5" s="26"/>
       <c r="E5" s="27">
         <f>SUM(Balance!$H$6:$H$19)</f>
-        <v>495559.84</v>
+        <v>495791.13</v>
       </c>
       <c r="F5" s="27"/>
       <c r="G5" s="27"/>
@@ -3585,7 +3585,7 @@
       <c r="D7" s="26"/>
       <c r="E7" s="27">
         <f>SUM(Balance!$G$6:$G$19)</f>
-        <v>2559.84</v>
+        <v>2791.13</v>
       </c>
       <c r="F7" s="27"/>
       <c r="G7" s="27"/>
@@ -3655,7 +3655,7 @@
       <c r="D12" s="26"/>
       <c r="E12" s="27">
         <f>IFERROR(VLOOKUP("Maya - Personal Goal",Balance!$C$6:$H$19,6,FALSE),0)</f>
-        <v>25116.67</v>
+        <v>25130.74</v>
       </c>
       <c r="F12" s="27"/>
       <c r="G12" s="27"/>
@@ -3672,7 +3672,7 @@
       <c r="D13" s="26"/>
       <c r="E13" s="28">
         <f>IFERROR(E12/E11,0)</f>
-        <v>0.2512</v>
+        <v>0.2513</v>
       </c>
       <c r="F13" s="28"/>
       <c r="G13" s="28"/>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B17" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A17,Balance!$H$6:$H$19)</f>
-        <v>274565.82</v>
+        <v>274700.74</v>
       </c>
     </row>
     <row r="18">
@@ -3729,7 +3729,7 @@
       </c>
       <c r="B18" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A18,Balance!$H$6:$H$19)</f>
-        <v>125581.64</v>
+        <v>125642.06</v>
       </c>
     </row>
     <row r="19">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="B19" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A19,Balance!$H$6:$H$19)</f>
-        <v>50266.67</v>
+        <v>50299.03</v>
       </c>
     </row>
     <row r="20">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="B22" s="30">
         <f>SUMIF(Balance!$A$6:$A$19,A22,Balance!$H$6:$H$19)</f>
-        <v>12030.0</v>
+        <v>12033.58</v>
       </c>
     </row>
     <row r="23">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="B24" s="16">
         <f>SUM(B17:B23)</f>
-        <v>495559.84</v>
+        <v>495791.13</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="E7" s="23">
         <f>IFERROR(VLOOKUP(D7,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>500.0</v>
+        <v>560.42</v>
       </c>
       <c r="F7" t="inlineStr" s="7">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="E8" s="23">
         <f>IFERROR(VLOOKUP(D8,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>500.0</v>
+        <v>560.42</v>
       </c>
       <c r="F8" t="inlineStr" s="7">
         <is>
@@ -6538,7 +6538,7 @@
       </c>
       <c r="E9" s="23">
         <f>IFERROR(VLOOKUP(D9,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>116.67</v>
+        <v>130.74</v>
       </c>
       <c r="F9" t="inlineStr" s="7">
         <is>
@@ -6598,7 +6598,7 @@
       </c>
       <c r="E11" s="23">
         <f>IFERROR(VLOOKUP(D11,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>250.0</v>
+        <v>280.21</v>
       </c>
       <c r="F11" t="inlineStr" s="7">
         <is>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="E12" s="23">
         <f>IFERROR(VLOOKUP(D12,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>250.0</v>
+        <v>280.21</v>
       </c>
       <c r="F12" t="inlineStr" s="7">
         <is>
@@ -6658,7 +6658,7 @@
       </c>
       <c r="E13" s="23">
         <f>IFERROR(VLOOKUP(D13,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.33</v>
+        <v>37.33</v>
       </c>
       <c r="F13" t="inlineStr" s="7">
         <is>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="E14" s="23">
         <f>IFERROR(VLOOKUP(D14,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.33</v>
+        <v>37.33</v>
       </c>
       <c r="F14" t="inlineStr" s="7">
         <is>
@@ -6718,7 +6718,7 @@
       </c>
       <c r="E15" s="23">
         <f>IFERROR(VLOOKUP(D15,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>200.0</v>
+        <v>224.37</v>
       </c>
       <c r="F15" t="inlineStr" s="7">
         <is>
@@ -6808,7 +6808,7 @@
       </c>
       <c r="E18" s="23">
         <f>IFERROR(VLOOKUP(D18,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>30.0</v>
+        <v>33.58</v>
       </c>
       <c r="F18" t="inlineStr" s="7">
         <is>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="E20" s="16">
         <f>SUM(E6:E19)</f>
-        <v>2559.84</v>
+        <v>2791.13</v>
       </c>
       <c r="F20" t="inlineStr" s="15">
         <is>
@@ -7096,7 +7096,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Current Balance = Principal (Deposits + Net Transactions) + Interest Earned. Interest is posted automatically on the Transactions tab and grows each day/month, so Current Balance rises on its own.</t>
+          <t xml:space="preserve">Current Balance = Principal (Deposits + Net Transactions) + Interest Earned. Interest accrues daily for every account and is posted automatically on the Transactions tab, so Current Balance rises a little every day.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -7264,11 +7264,11 @@
       </c>
       <c r="G7" s="23">
         <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>500.0</v>
+        <v>560.42</v>
       </c>
       <c r="H7" s="23">
         <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>100500.0</v>
+        <v>100560.42</v>
       </c>
       <c r="I7" s="8">
         <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7312,11 +7312,11 @@
       </c>
       <c r="G8" s="23">
         <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>500.0</v>
+        <v>560.42</v>
       </c>
       <c r="H8" s="23">
         <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>100500.0</v>
+        <v>100560.42</v>
       </c>
       <c r="I8" s="8">
         <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7360,11 +7360,11 @@
       </c>
       <c r="G9" s="23">
         <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>116.67</v>
+        <v>130.74</v>
       </c>
       <c r="H9" s="23">
         <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>25116.67</v>
+        <v>25130.74</v>
       </c>
       <c r="I9" s="8">
         <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7456,11 +7456,11 @@
       </c>
       <c r="G11" s="23">
         <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>250.0</v>
+        <v>280.21</v>
       </c>
       <c r="H11" s="23">
         <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>50250.0</v>
+        <v>50280.21</v>
       </c>
       <c r="I11" s="8">
         <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7504,11 +7504,11 @@
       </c>
       <c r="G12" s="23">
         <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>250.0</v>
+        <v>280.21</v>
       </c>
       <c r="H12" s="23">
         <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>50250.0</v>
+        <v>50280.21</v>
       </c>
       <c r="I12" s="8">
         <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7552,11 +7552,11 @@
       </c>
       <c r="G13" s="23">
         <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.33</v>
+        <v>37.33</v>
       </c>
       <c r="H13" s="23">
         <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>10033.33</v>
+        <v>10037.33</v>
       </c>
       <c r="I13" s="8">
         <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7600,11 +7600,11 @@
       </c>
       <c r="G14" s="23">
         <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.33</v>
+        <v>37.33</v>
       </c>
       <c r="H14" s="23">
         <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>10033.33</v>
+        <v>10037.33</v>
       </c>
       <c r="I14" s="8">
         <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7648,11 +7648,11 @@
       </c>
       <c r="G15" s="23">
         <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>200.0</v>
+        <v>224.37</v>
       </c>
       <c r="H15" s="23">
         <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>30200.0</v>
+        <v>30224.37</v>
       </c>
       <c r="I15" s="8">
         <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7792,11 +7792,11 @@
       </c>
       <c r="G18" s="23">
         <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>30.0</v>
+        <v>33.58</v>
       </c>
       <c r="H18" s="23">
         <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$Q$19,14,FALSE),0)</f>
-        <v>12030.0</v>
+        <v>12033.58</v>
       </c>
       <c r="I18" s="8">
         <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$L$19,9,FALSE),0)</f>
@@ -7880,11 +7880,11 @@
       </c>
       <c r="G20" s="16">
         <f>SUM(G6:G19)</f>
-        <v>2559.84</v>
+        <v>2791.13</v>
       </c>
       <c r="H20" s="16">
         <f>SUM(H6:H19)</f>
-        <v>495559.84</v>
+        <v>495791.13</v>
       </c>
       <c r="I20" s="16">
         <f>SUM(I6:I19)</f>
@@ -8010,7 +8010,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Interest auto-calculates and GROWS ON ITS OWN. 'Balance Today' accrues from the yellow 'Interest Start' date up to TODAY() every time you open the file - daily accounts step up each day, monthly accounts each month. Interest Start is pre-filled with your first deposit date; edit it if an account started elsewhere. Maya Savings = 10%.</t>
+          <t xml:space="preserve">Interest auto-calculates and GROWS ON ITS OWN. 'Balance Today' accrues DAILY for every account (annual rate / 365, compounded each day) from the yellow 'Interest Start' date up to TODAY(), so it grows a little every day you open the file. Interest Start is pre-filled with your first deposit date; edit it if an account started elsewhere. Maya Savings = 10%.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -8128,7 +8128,7 @@
       </c>
       <c r="O5" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Periods Elapsed</t>
+          <t xml:space="preserve">Days Elapsed</t>
         </is>
       </c>
       <c r="P5" t="inlineStr" s="6">
@@ -8208,11 +8208,11 @@
         <v>46174</v>
       </c>
       <c r="O6" s="10">
-        <f>IF(ISNUMBER(N6),IF(F6="Daily",MAX(0,TODAY()-N6),MAX(0,DATEDIF(N6,TODAY(),"m"))),0)</f>
+        <f>IF(ISNUMBER(N6),MAX(0,TODAY()-N6),0)</f>
         <v>34</v>
       </c>
       <c r="P6" s="8">
-        <f>G6*((1+H6)^O6-1)</f>
+        <f>G6*((1+E6/365)^O6-1)</f>
         <v>449.15</v>
       </c>
       <c r="Q6" s="8">
@@ -8285,16 +8285,16 @@
         <v>46174</v>
       </c>
       <c r="O7" s="10">
-        <f>IF(ISNUMBER(N7),IF(F7="Daily",MAX(0,TODAY()-N7),MAX(0,DATEDIF(N7,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N7),MAX(0,TODAY()-N7),0)</f>
+        <v>34</v>
       </c>
       <c r="P7" s="8">
-        <f>G7*((1+H7)^O7-1)</f>
-        <v>500.0</v>
+        <f>G7*((1+E7/365)^O7-1)</f>
+        <v>560.42</v>
       </c>
       <c r="Q7" s="8">
         <f>G7+P7</f>
-        <v>100500.0</v>
+        <v>100560.42</v>
       </c>
       <c r="R7" s="10">
         <f>IF(F7="Daily",365,12)</f>
@@ -8362,16 +8362,16 @@
         <v>46174</v>
       </c>
       <c r="O8" s="10">
-        <f>IF(ISNUMBER(N8),IF(F8="Daily",MAX(0,TODAY()-N8),MAX(0,DATEDIF(N8,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N8),MAX(0,TODAY()-N8),0)</f>
+        <v>34</v>
       </c>
       <c r="P8" s="8">
-        <f>G8*((1+H8)^O8-1)</f>
-        <v>500.0</v>
+        <f>G8*((1+E8/365)^O8-1)</f>
+        <v>560.42</v>
       </c>
       <c r="Q8" s="8">
         <f>G8+P8</f>
-        <v>100500.0</v>
+        <v>100560.42</v>
       </c>
       <c r="R8" s="10">
         <f>IF(F8="Daily",365,12)</f>
@@ -8439,16 +8439,16 @@
         <v>46174</v>
       </c>
       <c r="O9" s="10">
-        <f>IF(ISNUMBER(N9),IF(F9="Daily",MAX(0,TODAY()-N9),MAX(0,DATEDIF(N9,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N9),MAX(0,TODAY()-N9),0)</f>
+        <v>34</v>
       </c>
       <c r="P9" s="8">
-        <f>G9*((1+H9)^O9-1)</f>
-        <v>116.67</v>
+        <f>G9*((1+E9/365)^O9-1)</f>
+        <v>130.74</v>
       </c>
       <c r="Q9" s="8">
         <f>G9+P9</f>
-        <v>25116.67</v>
+        <v>25130.74</v>
       </c>
       <c r="R9" s="10">
         <f>IF(F9="Daily",365,12)</f>
@@ -8516,11 +8516,11 @@
         <v>46174</v>
       </c>
       <c r="O10" s="10">
-        <f>IF(ISNUMBER(N10),IF(F10="Daily",MAX(0,TODAY()-N10),MAX(0,DATEDIF(N10,TODAY(),"m"))),0)</f>
+        <f>IF(ISNUMBER(N10),MAX(0,TODAY()-N10),0)</f>
         <v>34</v>
       </c>
       <c r="P10" s="8">
-        <f>G10*((1+H10)^O10-1)</f>
+        <f>G10*((1+E10/365)^O10-1)</f>
         <v>81.64</v>
       </c>
       <c r="Q10" s="8">
@@ -8593,16 +8593,16 @@
         <v>46174</v>
       </c>
       <c r="O11" s="10">
-        <f>IF(ISNUMBER(N11),IF(F11="Daily",MAX(0,TODAY()-N11),MAX(0,DATEDIF(N11,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N11),MAX(0,TODAY()-N11),0)</f>
+        <v>34</v>
       </c>
       <c r="P11" s="8">
-        <f>G11*((1+H11)^O11-1)</f>
-        <v>250.0</v>
+        <f>G11*((1+E11/365)^O11-1)</f>
+        <v>280.21</v>
       </c>
       <c r="Q11" s="8">
         <f>G11+P11</f>
-        <v>50250.0</v>
+        <v>50280.21</v>
       </c>
       <c r="R11" s="10">
         <f>IF(F11="Daily",365,12)</f>
@@ -8670,16 +8670,16 @@
         <v>46174</v>
       </c>
       <c r="O12" s="10">
-        <f>IF(ISNUMBER(N12),IF(F12="Daily",MAX(0,TODAY()-N12),MAX(0,DATEDIF(N12,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N12),MAX(0,TODAY()-N12),0)</f>
+        <v>34</v>
       </c>
       <c r="P12" s="8">
-        <f>G12*((1+H12)^O12-1)</f>
-        <v>250.0</v>
+        <f>G12*((1+E12/365)^O12-1)</f>
+        <v>280.21</v>
       </c>
       <c r="Q12" s="8">
         <f>G12+P12</f>
-        <v>50250.0</v>
+        <v>50280.21</v>
       </c>
       <c r="R12" s="10">
         <f>IF(F12="Daily",365,12)</f>
@@ -8747,16 +8747,16 @@
         <v>46174</v>
       </c>
       <c r="O13" s="10">
-        <f>IF(ISNUMBER(N13),IF(F13="Daily",MAX(0,TODAY()-N13),MAX(0,DATEDIF(N13,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N13),MAX(0,TODAY()-N13),0)</f>
+        <v>34</v>
       </c>
       <c r="P13" s="8">
-        <f>G13*((1+H13)^O13-1)</f>
-        <v>33.33</v>
+        <f>G13*((1+E13/365)^O13-1)</f>
+        <v>37.33</v>
       </c>
       <c r="Q13" s="8">
         <f>G13+P13</f>
-        <v>10033.33</v>
+        <v>10037.33</v>
       </c>
       <c r="R13" s="10">
         <f>IF(F13="Daily",365,12)</f>
@@ -8824,16 +8824,16 @@
         <v>46174</v>
       </c>
       <c r="O14" s="10">
-        <f>IF(ISNUMBER(N14),IF(F14="Daily",MAX(0,TODAY()-N14),MAX(0,DATEDIF(N14,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N14),MAX(0,TODAY()-N14),0)</f>
+        <v>34</v>
       </c>
       <c r="P14" s="8">
-        <f>G14*((1+H14)^O14-1)</f>
-        <v>33.33</v>
+        <f>G14*((1+E14/365)^O14-1)</f>
+        <v>37.33</v>
       </c>
       <c r="Q14" s="8">
         <f>G14+P14</f>
-        <v>10033.33</v>
+        <v>10037.33</v>
       </c>
       <c r="R14" s="10">
         <f>IF(F14="Daily",365,12)</f>
@@ -8901,16 +8901,16 @@
         <v>46174</v>
       </c>
       <c r="O15" s="10">
-        <f>IF(ISNUMBER(N15),IF(F15="Daily",MAX(0,TODAY()-N15),MAX(0,DATEDIF(N15,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N15),MAX(0,TODAY()-N15),0)</f>
+        <v>34</v>
       </c>
       <c r="P15" s="8">
-        <f>G15*((1+H15)^O15-1)</f>
-        <v>200.0</v>
+        <f>G15*((1+E15/365)^O15-1)</f>
+        <v>224.37</v>
       </c>
       <c r="Q15" s="8">
         <f>G15+P15</f>
-        <v>30200.0</v>
+        <v>30224.37</v>
       </c>
       <c r="R15" s="10">
         <f>IF(F15="Daily",365,12)</f>
@@ -8978,11 +8978,11 @@
         <v>46174</v>
       </c>
       <c r="O16" s="10">
-        <f>IF(ISNUMBER(N16),IF(F16="Daily",MAX(0,TODAY()-N16),MAX(0,DATEDIF(N16,TODAY(),"m"))),0)</f>
+        <f>IF(ISNUMBER(N16),MAX(0,TODAY()-N16),0)</f>
         <v>34</v>
       </c>
       <c r="P16" s="8">
-        <f>G16*((1+H16)^O16-1)</f>
+        <f>G16*((1+E16/365)^O16-1)</f>
         <v>70.02</v>
       </c>
       <c r="Q16" s="8">
@@ -9055,11 +9055,11 @@
         <v>46174</v>
       </c>
       <c r="O17" s="10">
-        <f>IF(ISNUMBER(N17),IF(F17="Daily",MAX(0,TODAY()-N17),MAX(0,DATEDIF(N17,TODAY(),"m"))),0)</f>
+        <f>IF(ISNUMBER(N17),MAX(0,TODAY()-N17),0)</f>
         <v>34</v>
       </c>
       <c r="P17" s="8">
-        <f>G17*((1+H17)^O17-1)</f>
+        <f>G17*((1+E17/365)^O17-1)</f>
         <v>21.45</v>
       </c>
       <c r="Q17" s="8">
@@ -9132,16 +9132,16 @@
         <v>46174</v>
       </c>
       <c r="O18" s="10">
-        <f>IF(ISNUMBER(N18),IF(F18="Daily",MAX(0,TODAY()-N18),MAX(0,DATEDIF(N18,TODAY(),"m"))),0)</f>
-        <v>1</v>
+        <f>IF(ISNUMBER(N18),MAX(0,TODAY()-N18),0)</f>
+        <v>34</v>
       </c>
       <c r="P18" s="8">
-        <f>G18*((1+H18)^O18-1)</f>
-        <v>30.0</v>
+        <f>G18*((1+E18/365)^O18-1)</f>
+        <v>33.58</v>
       </c>
       <c r="Q18" s="8">
         <f>G18+P18</f>
-        <v>12030.0</v>
+        <v>12033.58</v>
       </c>
       <c r="R18" s="10">
         <f>IF(F18="Daily",365,12)</f>
@@ -9209,11 +9209,11 @@
         <v>46174</v>
       </c>
       <c r="O19" s="10">
-        <f>IF(ISNUMBER(N19),IF(F19="Daily",MAX(0,TODAY()-N19),MAX(0,DATEDIF(N19,TODAY(),"m"))),0)</f>
+        <f>IF(ISNUMBER(N19),MAX(0,TODAY()-N19),0)</f>
         <v>34</v>
       </c>
       <c r="P19" s="8">
-        <f>G19*((1+H19)^O19-1)</f>
+        <f>G19*((1+E19/365)^O19-1)</f>
         <v>24.25</v>
       </c>
       <c r="Q19" s="8">
@@ -9262,11 +9262,11 @@
       <c r="O20" s="15"/>
       <c r="P20" s="16">
         <f>SUM(P6:P19)</f>
-        <v>2559.84</v>
+        <v>2791.13</v>
       </c>
       <c r="Q20" s="16">
         <f>SUM(Q6:Q19)</f>
-        <v>495559.84</v>
+        <v>495791.13</v>
       </c>
       <c r="R20" s="15"/>
     </row>

</xml_diff>

<commit_message>
Transactions interest ledger now shows interest PER DAY (small daily amounts), not the running total
- Ledger Amount = each account's Interest / Day (Balance x rate/365), e.g. Maya Savings PHP 13.15/day
- Relabeled section 'Interest Earned per Day'; total row = total per day (PHP 81.87)
- Running cumulative total that feeds Current Balance stays on the Balance/Interest tabs
- Ledger is display-only (not summed into balances), so no double-count/loop; updated docx
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -6359,7 +6359,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Interest earned is shown at the TOP (auto-posted, read-only) and is already included in your Current Balance. Log the money you move (deposits/withdrawals/transfers) in the Transaction Log below - use negative amounts for money out and the filter arrows to search. The log can grow as long as you need (nothing sits beneath it).</t>
+          <t xml:space="preserve">Interest earned PER DAY is shown at the top (auto-posted, read-only) for each account. The running total of interest is added to your Current Balance automatically (see the Balance tab). Log the money you move (deposits/withdrawals/transfers) in the Transaction Log below - use negative amounts for money out and the filters to search; the log grows as you add rows.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -6378,7 +6378,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">🪙 Interest Earned  (auto-posted — do not edit)</t>
+          <t xml:space="preserve">🪙 Interest Earned per Day  (auto-posted — do not edit)</t>
         </is>
       </c>
       <c r="B4" s="4"/>
@@ -6447,12 +6447,12 @@
         </is>
       </c>
       <c r="E6" s="23">
-        <f>IFERROR(VLOOKUP(D6,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>449.15</v>
+        <f>IFERROR(VLOOKUP(D6,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>13.15</v>
       </c>
       <c r="F6" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6477,12 +6477,12 @@
         </is>
       </c>
       <c r="E7" s="23">
-        <f>IFERROR(VLOOKUP(D7,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>560.42</v>
+        <f>IFERROR(VLOOKUP(D7,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>16.44</v>
       </c>
       <c r="F7" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6507,12 +6507,12 @@
         </is>
       </c>
       <c r="E8" s="23">
-        <f>IFERROR(VLOOKUP(D8,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>560.42</v>
+        <f>IFERROR(VLOOKUP(D8,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>16.44</v>
       </c>
       <c r="F8" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6537,12 +6537,12 @@
         </is>
       </c>
       <c r="E9" s="23">
-        <f>IFERROR(VLOOKUP(D9,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>130.74</v>
+        <f>IFERROR(VLOOKUP(D9,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>3.84</v>
       </c>
       <c r="F9" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6567,12 +6567,12 @@
         </is>
       </c>
       <c r="E10" s="23">
-        <f>IFERROR(VLOOKUP(D10,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>81.64</v>
+        <f>IFERROR(VLOOKUP(D10,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>2.4</v>
       </c>
       <c r="F10" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6597,12 +6597,12 @@
         </is>
       </c>
       <c r="E11" s="23">
-        <f>IFERROR(VLOOKUP(D11,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>280.21</v>
+        <f>IFERROR(VLOOKUP(D11,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>8.22</v>
       </c>
       <c r="F11" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6627,12 +6627,12 @@
         </is>
       </c>
       <c r="E12" s="23">
-        <f>IFERROR(VLOOKUP(D12,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>280.21</v>
+        <f>IFERROR(VLOOKUP(D12,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>8.22</v>
       </c>
       <c r="F12" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6657,12 +6657,12 @@
         </is>
       </c>
       <c r="E13" s="23">
-        <f>IFERROR(VLOOKUP(D13,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>37.33</v>
+        <f>IFERROR(VLOOKUP(D13,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>1.1</v>
       </c>
       <c r="F13" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6687,12 +6687,12 @@
         </is>
       </c>
       <c r="E14" s="23">
-        <f>IFERROR(VLOOKUP(D14,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>37.33</v>
+        <f>IFERROR(VLOOKUP(D14,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>1.1</v>
       </c>
       <c r="F14" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6717,12 +6717,12 @@
         </is>
       </c>
       <c r="E15" s="23">
-        <f>IFERROR(VLOOKUP(D15,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>224.37</v>
+        <f>IFERROR(VLOOKUP(D15,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>6.58</v>
       </c>
       <c r="F15" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6747,12 +6747,12 @@
         </is>
       </c>
       <c r="E16" s="23">
-        <f>IFERROR(VLOOKUP(D16,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>70.02</v>
+        <f>IFERROR(VLOOKUP(D16,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>2.05</v>
       </c>
       <c r="F16" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6777,12 +6777,12 @@
         </is>
       </c>
       <c r="E17" s="23">
-        <f>IFERROR(VLOOKUP(D17,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>21.45</v>
+        <f>IFERROR(VLOOKUP(D17,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>0.63</v>
       </c>
       <c r="F17" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6807,12 +6807,12 @@
         </is>
       </c>
       <c r="E18" s="23">
-        <f>IFERROR(VLOOKUP(D18,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.58</v>
+        <f>IFERROR(VLOOKUP(D18,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>0.99</v>
       </c>
       <c r="F18" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6837,12 +6837,12 @@
         </is>
       </c>
       <c r="E19" s="23">
-        <f>IFERROR(VLOOKUP(D19,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>24.25</v>
+        <f>IFERROR(VLOOKUP(D19,Interest!$D$6:$R$19,6,FALSE),0)</f>
+        <v>0.71</v>
       </c>
       <c r="F19" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Interest earned to date</t>
+          <t xml:space="preserve">Interest earned per day</t>
         </is>
       </c>
     </row>
@@ -6864,12 +6864,12 @@
       </c>
       <c r="D20" t="inlineStr" s="15">
         <is>
-          <t xml:space="preserve">Total interest</t>
+          <t xml:space="preserve">Total per day</t>
         </is>
       </c>
       <c r="E20" s="16">
         <f>SUM(E6:E19)</f>
-        <v>2791.13</v>
+        <v>81.87</v>
       </c>
       <c r="F20" t="inlineStr" s="15">
         <is>

</xml_diff>

<commit_message>
Balance sheet: show Interest / Day (per-day) instead of the cumulative interest figure
- Balance 'Interest Earned' column -> 'Interest / Day' (Balance x rate/365), matching the Transactions ledger
- Current Balance (col H) unchanged: still Principal + interest accrued to date (daily)
- Dashboard 'Interest Earned to Date' KPI re-sourced to SUM(Interest!P) since Balance col is now per-day
- Updated formula .docx
</commit_message>
<xml_diff>
--- a/Digital-Bank-Savings-Tracker.xlsx
+++ b/Digital-Bank-Savings-Tracker.xlsx
@@ -3584,7 +3584,7 @@
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
       <c r="E7" s="27">
-        <f>SUM(Balance!$G$6:$G$19)</f>
+        <f>SUM(Interest!$P$6:$P$19)</f>
         <v>2791.13</v>
       </c>
       <c r="F7" s="27"/>
@@ -7096,7 +7096,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Current Balance = Principal (Deposits + Net Transactions) + Interest Earned. Interest accrues daily for every account and is posted automatically on the Transactions tab, so Current Balance rises a little every day.</t>
+          <t xml:space="preserve">Interest / Day shows each account's interest earned per day. Current Balance = Principal (Deposits + Net Transactions) + interest accrued to date; interest accrues daily for every account, so Current Balance rises a little every day.</t>
         </is>
       </c>
       <c r="B3" s="5"/>
@@ -7164,7 +7164,7 @@
       </c>
       <c r="G5" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Interest Earned</t>
+          <t xml:space="preserve">Interest / Day</t>
         </is>
       </c>
       <c r="H5" t="inlineStr" s="6">
@@ -7215,8 +7215,8 @@
         <v>48000.0</v>
       </c>
       <c r="G6" s="23">
-        <f>IFERROR(VLOOKUP(C6,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>449.15</v>
+        <f>IFERROR(VLOOKUP(C6,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>13.15</v>
       </c>
       <c r="H6" s="23">
         <f>IFERROR(VLOOKUP(C6,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7263,8 +7263,8 @@
         <v>100000.0</v>
       </c>
       <c r="G7" s="23">
-        <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>560.42</v>
+        <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>16.44</v>
       </c>
       <c r="H7" s="23">
         <f>IFERROR(VLOOKUP(C7,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7311,8 +7311,8 @@
         <v>100000.0</v>
       </c>
       <c r="G8" s="23">
-        <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>560.42</v>
+        <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>16.44</v>
       </c>
       <c r="H8" s="23">
         <f>IFERROR(VLOOKUP(C8,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7359,8 +7359,8 @@
         <v>25000.0</v>
       </c>
       <c r="G9" s="23">
-        <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>130.74</v>
+        <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>3.84</v>
       </c>
       <c r="H9" s="23">
         <f>IFERROR(VLOOKUP(C9,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7407,8 +7407,8 @@
         <v>25000.0</v>
       </c>
       <c r="G10" s="23">
-        <f>IFERROR(VLOOKUP(C10,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>81.64</v>
+        <f>IFERROR(VLOOKUP(C10,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>2.4</v>
       </c>
       <c r="H10" s="23">
         <f>IFERROR(VLOOKUP(C10,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7455,8 +7455,8 @@
         <v>50000.0</v>
       </c>
       <c r="G11" s="23">
-        <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>280.21</v>
+        <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>8.22</v>
       </c>
       <c r="H11" s="23">
         <f>IFERROR(VLOOKUP(C11,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7503,8 +7503,8 @@
         <v>50000.0</v>
       </c>
       <c r="G12" s="23">
-        <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>280.21</v>
+        <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>8.22</v>
       </c>
       <c r="H12" s="23">
         <f>IFERROR(VLOOKUP(C12,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7551,8 +7551,8 @@
         <v>10000.0</v>
       </c>
       <c r="G13" s="23">
-        <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>37.33</v>
+        <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>1.1</v>
       </c>
       <c r="H13" s="23">
         <f>IFERROR(VLOOKUP(C13,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7599,8 +7599,8 @@
         <v>10000.0</v>
       </c>
       <c r="G14" s="23">
-        <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>37.33</v>
+        <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>1.1</v>
       </c>
       <c r="H14" s="23">
         <f>IFERROR(VLOOKUP(C14,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7647,8 +7647,8 @@
         <v>30000.0</v>
       </c>
       <c r="G15" s="23">
-        <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>224.37</v>
+        <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>6.58</v>
       </c>
       <c r="H15" s="23">
         <f>IFERROR(VLOOKUP(C15,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7695,8 +7695,8 @@
         <v>15000.0</v>
       </c>
       <c r="G16" s="23">
-        <f>IFERROR(VLOOKUP(C16,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>70.02</v>
+        <f>IFERROR(VLOOKUP(C16,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>2.05</v>
       </c>
       <c r="H16" s="23">
         <f>IFERROR(VLOOKUP(C16,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7743,8 +7743,8 @@
         <v>10000.0</v>
       </c>
       <c r="G17" s="23">
-        <f>IFERROR(VLOOKUP(C17,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>21.45</v>
+        <f>IFERROR(VLOOKUP(C17,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>0.63</v>
       </c>
       <c r="H17" s="23">
         <f>IFERROR(VLOOKUP(C17,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7791,8 +7791,8 @@
         <v>12000.0</v>
       </c>
       <c r="G18" s="23">
-        <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>33.58</v>
+        <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>0.99</v>
       </c>
       <c r="H18" s="23">
         <f>IFERROR(VLOOKUP(C18,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7839,8 +7839,8 @@
         <v>8000.0</v>
       </c>
       <c r="G19" s="23">
-        <f>IFERROR(VLOOKUP(C19,Interest!$D$6:$Q$19,13,FALSE),0)</f>
-        <v>24.25</v>
+        <f>IFERROR(VLOOKUP(C19,Interest!$D$6:$Q$19,6,FALSE),0)</f>
+        <v>0.71</v>
       </c>
       <c r="H19" s="23">
         <f>IFERROR(VLOOKUP(C19,Interest!$D$6:$Q$19,14,FALSE),0)</f>
@@ -7880,7 +7880,7 @@
       </c>
       <c r="G20" s="16">
         <f>SUM(G6:G19)</f>
-        <v>2791.13</v>
+        <v>81.85</v>
       </c>
       <c r="H20" s="16">
         <f>SUM(H6:H19)</f>

</xml_diff>